<commit_message>
Improve contestant auto-assignment logic for groups and solos
Update auto-assignment logic to prevent self-matching, skip contestants with unavailable partners, and correctly identify true solo attendees.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: f123b9d7-6af8-472a-a75c-70d0b78d0583
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 24ee430e-127e-4e40-a07d-b725ede9ca0f
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/4ca2a1f8-42ce-4303-beff-eb92e3283d4c/f123b9d7-6af8-472a-a75c-70d0b78d0583/cLj8b3l
</commit_message>
<xml_diff>
--- a/storage/backups/automatic-backup.xlsx
+++ b/storage/backups/automatic-backup.xlsx
@@ -4,8 +4,9 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Record Days" sheetId="1" r:id="rId1"/>
-    <sheet name="Groups" sheetId="2" r:id="rId2"/>
-    <sheet name="Block Types" sheetId="3" r:id="rId3"/>
+    <sheet name="Contestants" sheetId="2" r:id="rId2"/>
+    <sheet name="Groups" sheetId="3" r:id="rId3"/>
+    <sheet name="Block Types" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -665,33 +666,1764 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:M51"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>ID</v>
       </c>
       <c r="B1" t="str">
-        <v>ReferenceNumber</v>
+        <v>Name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Age</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Gender</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Email</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Phone</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Location</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Rating</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="J1" t="str">
+        <v>AttendingWith</v>
+      </c>
+      <c r="K1" t="str">
+        <v>GroupID</v>
+      </c>
+      <c r="L1" t="str">
+        <v>MedicalInfo</v>
+      </c>
+      <c r="M1" t="str">
+        <v>MobilityNotes</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>f25a6094-c1a5-4eb4-a709-1cc3d9b3ab5e</v>
+        <v>efd8ab2e-988b-4afb-9374-3c3e3676f43a</v>
       </c>
       <c r="B2" t="str">
-        <v>GRP001</v>
+        <v>Matilda Sutherland</v>
+      </c>
+      <c r="C2">
+        <v>26</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E2" t="str">
+        <v>matilda.sutherland@hotmail.com</v>
+      </c>
+      <c r="F2" t="str">
+        <v>0467 165 012</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Bundoora</v>
+      </c>
+      <c r="H2" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I2" t="str">
+        <v>available</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Grace Mann</v>
+      </c>
+      <c r="M2" t="str">
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>f693566d-ea7c-40d1-89aa-158e842961d0</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Brent Barnett</v>
+      </c>
+      <c r="C3">
+        <v>37</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E3" t="str">
+        <v>brentbarnett88@gmail.com</v>
+      </c>
+      <c r="F3" t="str">
+        <v>423530043</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Preston</v>
+      </c>
+      <c r="H3" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I3" t="str">
+        <v>available</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Stephanie Squillacioti</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>82960b61-d36b-49e2-9ddf-a7b8e0b02a63</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Tara Saltzman</v>
+      </c>
+      <c r="C4">
+        <v>29</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E4" t="str">
+        <v>tarasaltzman@bigpond.com</v>
+      </c>
+      <c r="F4" t="str">
+        <v>448545599</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Melbourne</v>
+      </c>
+      <c r="H4" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I4" t="str">
+        <v>available</v>
+      </c>
+      <c r="J4" t="str">
+        <v xml:space="preserve">JACK AGIUS - NEEDS TO DO APPLICATION </v>
+      </c>
+      <c r="M4" t="str">
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>96d2c8ad-1e67-4659-b3d0-a3bbd4fe40cb</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Karina  Richmond</v>
+      </c>
+      <c r="C5">
+        <v>38</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E5" t="str">
+        <v>richmondkarina@yahoo.com</v>
+      </c>
+      <c r="F5" t="str">
+        <v>400554609</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Newcomb</v>
+      </c>
+      <c r="H5" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I5" t="str">
+        <v>available</v>
+      </c>
+      <c r="J5" t="str">
+        <v>AMY DILLON</v>
+      </c>
+      <c r="M5" t="str">
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>b1fc34e8-20cb-4607-9568-0761cf4520a6</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Troy Smith</v>
+      </c>
+      <c r="C6">
+        <v>31</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Troyssmith94@gmail.com</v>
+      </c>
+      <c r="F6" t="str">
+        <v>429354308</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Melbourne</v>
+      </c>
+      <c r="H6" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I6" t="str">
+        <v>available</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Tayla Huxtable</v>
+      </c>
+      <c r="K6" t="str">
+        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
+      </c>
+      <c r="L6" t="str">
+        <v xml:space="preserve">Peanut allergy </v>
+      </c>
+      <c r="M6" t="str">
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>6b9ae7f0-4a81-4dda-8e55-e49415d98ec6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Tayla Huxtable</v>
+      </c>
+      <c r="C7">
+        <v>28</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Taylahuxtable@gmail.com</v>
+      </c>
+      <c r="F7" t="str">
+        <v>435320280</v>
+      </c>
+      <c r="G7" t="str">
+        <v>FERNTREE GULLY</v>
+      </c>
+      <c r="I7" t="str">
+        <v>available</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Troy Smith</v>
+      </c>
+      <c r="K7" t="str">
+        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>7a05a613-1880-40c5-ab6a-cc078b418b6e</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Deb  Jones</v>
+      </c>
+      <c r="C8">
+        <v>66</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E8" t="str">
+        <v>fullhouse5@optusnet.com.au</v>
+      </c>
+      <c r="F8" t="str">
+        <v>438561474</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Bayswater North</v>
+      </c>
+      <c r="H8" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I8" t="str">
+        <v>available</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Daryl Jones</v>
+      </c>
+      <c r="M8" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>6cada433-8344-4d95-97dc-33c9c173ce7c</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Jeanette Quy</v>
+      </c>
+      <c r="C9">
+        <v>74</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E9" t="str">
+        <v>quyfamily@tpg.com.au</v>
+      </c>
+      <c r="F9" t="str">
+        <v>402902273</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Rowville</v>
+      </c>
+      <c r="H9" t="str">
+        <v>C</v>
+      </c>
+      <c r="I9" t="str">
+        <v>available</v>
+      </c>
+      <c r="M9" t="str">
+        <v xml:space="preserve">nothing of note </v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>6bbdadcb-23a8-41c9-964b-6152e234cb33</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Philip Natoli</v>
+      </c>
+      <c r="C10">
+        <v>29</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Philip.natoli@outlook.com</v>
+      </c>
+      <c r="F10" t="str">
+        <v>466021882</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Caulfield South</v>
+      </c>
+      <c r="H10" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I10" t="str">
+        <v>available</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Hayley Wright</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>34b3d848-f096-4bc9-bd55-dc4dd85ad1b3</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Donna Collins</v>
+      </c>
+      <c r="C11">
+        <v>65</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Donna0@hotmail.com</v>
+      </c>
+      <c r="F11" t="str">
+        <v>408122305</v>
+      </c>
+      <c r="G11" t="str">
+        <v xml:space="preserve">Coburg </v>
+      </c>
+      <c r="H11" t="str">
+        <v>B</v>
+      </c>
+      <c r="I11" t="str">
+        <v>available</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Donna Collins, Tom Collins</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>97e81b41-1b8d-4562-9e12-3747f87663a9</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Thomas Mckenna</v>
+      </c>
+      <c r="C12">
+        <v>36</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E12" t="str">
+        <v>mckenna.6@yahoo.com</v>
+      </c>
+      <c r="F12" t="str">
+        <v>421758700</v>
+      </c>
+      <c r="G12" t="str">
+        <v xml:space="preserve">Officer South </v>
+      </c>
+      <c r="H12" t="str">
+        <v>B</v>
+      </c>
+      <c r="I12" t="str">
+        <v>available</v>
+      </c>
+      <c r="J12" t="str">
+        <v>thomas mckenna, Carolyn (Caz) Wilby</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>607e3750-92e2-4480-b39d-1cb0e026cd4b</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Natasha Devers</v>
+      </c>
+      <c r="C13">
+        <v>22</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E13" t="str">
+        <v>natashadevers@gmail.com</v>
+      </c>
+      <c r="F13" t="str">
+        <v>484003770</v>
+      </c>
+      <c r="G13" t="str">
+        <v xml:space="preserve">Waterways </v>
+      </c>
+      <c r="H13" t="str">
+        <v>B</v>
+      </c>
+      <c r="I13" t="str">
+        <v>available</v>
+      </c>
+      <c r="J13" t="str">
+        <v>Oliver Moran</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>fb6dd634-cefe-4cce-a1cc-af5d1677fdcb</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Elizabeth Schembri</v>
+      </c>
+      <c r="C14">
+        <v>69</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E14" t="str">
+        <v>e-schembri@hotmail.com</v>
+      </c>
+      <c r="F14" t="str">
+        <v>452177157</v>
+      </c>
+      <c r="G14" t="str">
+        <v xml:space="preserve">Melbourne </v>
+      </c>
+      <c r="H14" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I14" t="str">
+        <v>available</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Elizabeth Schembri, Gerard Hayward</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15" t="str">
+        <v>dcd305dd-c710-4a1e-859c-835031154035</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Nicholas Boicos</v>
+      </c>
+      <c r="C15">
+        <v>22</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E15" t="str">
+        <v>nboicos@hotmail.com</v>
+      </c>
+      <c r="F15" t="str">
+        <v>429556400</v>
+      </c>
+      <c r="G15" t="str">
+        <v xml:space="preserve">Altona Meadows </v>
+      </c>
+      <c r="H15" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I15" t="str">
+        <v>available</v>
+      </c>
+      <c r="J15" t="str" xml:space="preserve">
+        <v xml:space="preserve">Nick Boicos 
+Matthew Boicos
+Brothers</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16" t="str">
+        <v>09dbfbb4-9f89-44a1-95f3-10cc82ec732a</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Gianni De Pasquale</v>
+      </c>
+      <c r="C16">
+        <v>20</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E16" t="str">
+        <v>gdp762.0@gmail.com</v>
+      </c>
+      <c r="F16" t="str">
+        <v>481978762</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Werribee</v>
+      </c>
+      <c r="H16" t="str">
+        <v>A</v>
+      </c>
+      <c r="I16" t="str">
+        <v>available</v>
+      </c>
+      <c r="J16" t="str" xml:space="preserve">
+        <v xml:space="preserve">Gianni De Pasquale
+Carmela De Pasquale
+Francesco De Pasquale</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>de606917-da6f-4fde-881b-7cbfd45cfe56</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Ricky Steve</v>
+      </c>
+      <c r="C17">
+        <v>31</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E17" t="str">
+        <v>tj-c-a@hotmail.com</v>
+      </c>
+      <c r="F17" t="str">
+        <v>411360449</v>
+      </c>
+      <c r="G17" t="str">
+        <v xml:space="preserve">Wangaratta </v>
+      </c>
+      <c r="H17" t="str">
+        <v>A</v>
+      </c>
+      <c r="I17" t="str">
+        <v>available</v>
+      </c>
+      <c r="J17" t="str">
+        <v>Taylah-Jayne Lockery</v>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
+        <v>1fe25fd6-dc69-4d29-b22f-9a15ad3d457f</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Sharon King</v>
+      </c>
+      <c r="C18">
+        <v>58</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E18" t="str">
+        <v>dreamweaversixtyseven@gmail.com</v>
+      </c>
+      <c r="F18" t="str">
+        <v>611488000000</v>
+      </c>
+      <c r="G18" t="str">
+        <v xml:space="preserve">Mooroopna </v>
+      </c>
+      <c r="H18" t="str">
+        <v>A</v>
+      </c>
+      <c r="I18" t="str">
+        <v>available</v>
+      </c>
+      <c r="J18" t="str" xml:space="preserve">
+        <v xml:space="preserve">
+Friend :Jacinda Austin
+ID:b6042a-1-1936475</v>
+      </c>
+      <c r="M18" t="str">
+        <v xml:space="preserve">No </v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>4f08069b-d828-429c-af5e-b1eee2c123df</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Sarah Desira</v>
+      </c>
+      <c r="C19">
+        <v>38</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E19" t="str">
+        <v>unicornwolf11@gmail.com</v>
+      </c>
+      <c r="F19" t="str">
+        <v>450765125</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Lara</v>
+      </c>
+      <c r="H19" t="str">
+        <v>B</v>
+      </c>
+      <c r="I19" t="str">
+        <v>available</v>
+      </c>
+      <c r="J19" t="str">
+        <v>Husband Daniel Desira b6042a-1-1936280</v>
+      </c>
+      <c r="M19" t="str">
+        <v xml:space="preserve">No </v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>e4a52d0d-9c54-4504-8a0f-85845cd88e27</v>
+      </c>
+      <c r="B20" t="str">
+        <v>David Fenwick</v>
+      </c>
+      <c r="C20">
+        <v>36</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E20" t="str">
+        <v>David.s.fenwick@gmail.com</v>
+      </c>
+      <c r="F20" t="str">
+        <v>429811171</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Teesdale</v>
+      </c>
+      <c r="H20" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I20" t="str">
+        <v>available</v>
+      </c>
+      <c r="J20" t="str">
+        <v>Solo</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>419afd3f-2406-423d-942f-2dfafe875f96</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Anna Fonua</v>
+      </c>
+      <c r="C21">
+        <v>36</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Annawallace89@hotmail.com</v>
+      </c>
+      <c r="F21" t="str">
+        <v>452452442</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Truganina</v>
+      </c>
+      <c r="H21" t="str">
+        <v>A</v>
+      </c>
+      <c r="I21" t="str">
+        <v>available</v>
+      </c>
+      <c r="J21" t="str">
+        <v>Dad Michael Wallace - b6042a-1-1936372</v>
+      </c>
+      <c r="M21" t="str">
+        <v xml:space="preserve">no </v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>1d96e742-18bb-4fc0-b741-154d1a4d9487</v>
+      </c>
+      <c r="B22" t="str">
+        <v>James Butler</v>
+      </c>
+      <c r="C22">
+        <v>42</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E22" t="str">
+        <v>butlerjg1509@gmail.com</v>
+      </c>
+      <c r="F22" t="str">
+        <v>428400584</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Mentone</v>
+      </c>
+      <c r="H22" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I22" t="str">
+        <v>available</v>
+      </c>
+      <c r="J22" t="str">
+        <v>Issy McReynolds</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>f7b766dc-a0d0-4a91-98ef-47472cdca803</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Mara Baumgardner</v>
+      </c>
+      <c r="C23">
+        <v>40</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Granic@hotmail.com</v>
+      </c>
+      <c r="F23" t="str">
+        <v>407364450</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Cockatoo</v>
+      </c>
+      <c r="H23" t="str">
+        <v>B</v>
+      </c>
+      <c r="I23" t="str">
+        <v>available</v>
+      </c>
+      <c r="J23" t="str">
+        <v xml:space="preserve">Mum - Mira Granic </v>
+      </c>
+      <c r="M23" t="str">
+        <v xml:space="preserve">No </v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>1bc7d8fc-def3-4f9f-8376-80b79696d1a5</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Eden Hayes</v>
+      </c>
+      <c r="C24">
+        <v>21</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E24" t="str">
+        <v>edenhayes19@gmail.com</v>
+      </c>
+      <c r="F24" t="str">
+        <v>448096139</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Elwood</v>
+      </c>
+      <c r="H24" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I24" t="str">
+        <v>available</v>
+      </c>
+      <c r="J24" t="str">
+        <v>Jackson Harris</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>614641dd-4e94-4c42-a1d9-db37c608dcbe</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Antonio Freno</v>
+      </c>
+      <c r="C25">
+        <v>39</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E25" t="str">
+        <v>frenoantonio@hotmail.it</v>
+      </c>
+      <c r="F25" t="str">
+        <v>422177371</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Glenroy</v>
+      </c>
+      <c r="H25" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I25" t="str">
+        <v>available</v>
+      </c>
+      <c r="J25" t="str">
+        <v>Solo</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>96c75db9-b001-4abe-8ddb-d5a73cb04529</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Kiran Rao</v>
+      </c>
+      <c r="C26">
+        <v>35</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E26" t="str">
+        <v>kiran.rao07@gmail.com</v>
+      </c>
+      <c r="F26" t="str">
+        <v>420486042</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Southbank</v>
+      </c>
+      <c r="H26" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I26" t="str">
+        <v>available</v>
+      </c>
+      <c r="J26" t="str">
+        <v>SOLO</v>
+      </c>
+      <c r="M26" t="str">
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>9f63aad3-aae1-4220-825c-8964694ec5d8</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Kerrie Donald</v>
+      </c>
+      <c r="C27">
+        <v>47</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E27" t="str">
+        <v>kerrieldonald@hotmail.com</v>
+      </c>
+      <c r="F27" t="str">
+        <v>61400826565</v>
+      </c>
+      <c r="G27" t="str">
+        <v>Mailor's Flat</v>
+      </c>
+      <c r="H27" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I27" t="str">
+        <v>available</v>
+      </c>
+      <c r="J27" t="str">
+        <v>kerrie donald, alistair donald</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>f048c8fe-e8c9-4357-8ec8-ef76793e5bc1</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Tamara Mifsud</v>
+      </c>
+      <c r="C28">
+        <v>32</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E28" t="str">
+        <v>tamara.mifsud@hotmail.com</v>
+      </c>
+      <c r="F28" t="str">
+        <v>416552122</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Aintree</v>
+      </c>
+      <c r="H28" t="str">
+        <v>B</v>
+      </c>
+      <c r="I28" t="str">
+        <v>available</v>
+      </c>
+      <c r="J28" t="str">
+        <v>Aliye Abcilar</v>
+      </c>
+    </row>
+    <row r="29" xml:space="preserve">
+      <c r="A29" t="str">
+        <v>ed91813b-2f74-4638-9d1a-ef8c54cff447</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Linda Browne</v>
+      </c>
+      <c r="C29">
+        <v>54</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Lindabrowne@iprimus.com.au</v>
+      </c>
+      <c r="F29" t="str">
+        <v>429570177</v>
+      </c>
+      <c r="G29" t="str">
+        <v>OFFICER</v>
+      </c>
+      <c r="H29" t="str">
+        <v>B</v>
+      </c>
+      <c r="I29" t="str">
+        <v>available</v>
+      </c>
+      <c r="J29" t="str" xml:space="preserve">
+        <v xml:space="preserve">Natalie Browne
+Linda Browne
+Aidan Miler</v>
+      </c>
+    </row>
+    <row r="30" xml:space="preserve">
+      <c r="A30" t="str">
+        <v>7fc083f6-6be3-42bf-b4e5-fc6412e1c559</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Meenakshi  Mehra</v>
+      </c>
+      <c r="C30">
+        <v>62</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E30" t="str">
+        <v>meenu.mehra@bigpond.com</v>
+      </c>
+      <c r="F30" t="str">
+        <v>420353322</v>
+      </c>
+      <c r="G30" t="str">
+        <v xml:space="preserve">Melbourne </v>
+      </c>
+      <c r="H30" t="str">
+        <v>B</v>
+      </c>
+      <c r="I30" t="str">
+        <v>available</v>
+      </c>
+      <c r="J30" t="str" xml:space="preserve">
+        <v xml:space="preserve">Meenakshi Mehra
+Dhananjay Mehra</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>8a905dfd-647c-4d96-a741-f7f1517a5136</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Deanna Hay</v>
+      </c>
+      <c r="C31">
+        <v>38</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E31" t="str">
+        <v>dee_hay24@hotmail.com</v>
+      </c>
+      <c r="F31" t="str">
+        <v>424504430</v>
+      </c>
+      <c r="G31" t="str">
+        <v xml:space="preserve">Melbourne </v>
+      </c>
+      <c r="H31" t="str">
+        <v>DNU</v>
+      </c>
+      <c r="I31" t="str">
+        <v>available</v>
+      </c>
+      <c r="J31" t="str">
+        <v>Lynetta Shan Faoa</v>
+      </c>
+      <c r="L31" t="str">
+        <v xml:space="preserve">Cerebral palsy in a wheelchair </v>
+      </c>
+    </row>
+    <row r="32" xml:space="preserve">
+      <c r="A32" t="str">
+        <v>d9b76f1c-0867-44fc-9215-6ef7b1184af6</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Kayla Lorenzini</v>
+      </c>
+      <c r="C32">
+        <v>29</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E32" t="str">
+        <v>kaylalorenzini_@hotmail.com</v>
+      </c>
+      <c r="F32" t="str">
+        <v>430517653</v>
+      </c>
+      <c r="G32" t="str">
+        <v>Melbourne</v>
+      </c>
+      <c r="H32" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I32" t="str">
+        <v>available</v>
+      </c>
+      <c r="J32" t="str" xml:space="preserve">
+        <v xml:space="preserve">Kayla Lorenzini
+James Lorenzini
+Deanna Gramola</v>
+      </c>
+    </row>
+    <row r="33" xml:space="preserve">
+      <c r="A33" t="str">
+        <v>15fb53d0-3916-4c9a-9f73-c28c879dec33</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Mozgda  Alime</v>
+      </c>
+      <c r="C33">
+        <v>39</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E33" t="str">
+        <v>smalimi@hotmail.com</v>
+      </c>
+      <c r="F33" t="str">
+        <v>402010235</v>
+      </c>
+      <c r="G33" t="str">
+        <v xml:space="preserve">Melbourne </v>
+      </c>
+      <c r="H33" t="str">
+        <v>C</v>
+      </c>
+      <c r="I33" t="str">
+        <v>available</v>
+      </c>
+      <c r="J33" t="str" xml:space="preserve">
+        <v xml:space="preserve">Sadaf Almini - I believe this is her cousin 
+Lida Alime - I believe this is her cousin or sister 
+Ahmad Alime - Ahmad is Lina's husband </v>
+      </c>
+      <c r="M33" t="str">
+        <v xml:space="preserve">No </v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>94b19240-6aee-4af6-ac66-0ebdb5e4403c</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Scott Clark</v>
+      </c>
+      <c r="C34">
+        <v>54</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E34" t="str">
+        <v>sclarkfitness@optusnet.com.au</v>
+      </c>
+      <c r="F34" t="str">
+        <v>448073035</v>
+      </c>
+      <c r="G34" t="str">
+        <v>Melbourne</v>
+      </c>
+      <c r="H34" t="str">
+        <v>A+</v>
+      </c>
+      <c r="I34" t="str">
+        <v>available</v>
+      </c>
+      <c r="J34" t="str">
+        <v xml:space="preserve">Would bring someone </v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>917bd31e-7781-44cc-936c-980cb1f844aa</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Angela Verspay</v>
+      </c>
+      <c r="C35">
+        <v>45</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E35" t="str">
+        <v>angelarileysmyth@hotmail.com</v>
+      </c>
+      <c r="F35" t="str">
+        <v>477660119</v>
+      </c>
+      <c r="G35" t="str">
+        <v>Warrnambool</v>
+      </c>
+      <c r="H35" t="str">
+        <v>B</v>
+      </c>
+      <c r="I35" t="str">
+        <v>available</v>
+      </c>
+      <c r="J35" t="str">
+        <v>SOLO</v>
+      </c>
+      <c r="M35" t="str">
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>eb3b2a7d-e6b0-421b-8987-00bfff95dda9</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Jasmine Miller</v>
+      </c>
+      <c r="C36">
+        <v>32</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E36" t="str">
+        <v>jasmine_courtney@hotmail.com</v>
+      </c>
+      <c r="F36" t="str">
+        <v>0432 387 712</v>
+      </c>
+      <c r="G36" t="str">
+        <v>Hughesdale</v>
+      </c>
+      <c r="H36" t="str">
+        <v>C</v>
+      </c>
+      <c r="I36" t="str">
+        <v>available</v>
+      </c>
+      <c r="J36" t="str">
+        <v>ablo - partner</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>45c7f69f-dd89-41d8-b7f0-a83f77fa9d12</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Sherif Haggag</v>
+      </c>
+      <c r="C37">
+        <v>38</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Shaggag87@gmail.com</v>
+      </c>
+      <c r="F37" t="str">
+        <v>426233449</v>
+      </c>
+      <c r="G37" t="str">
+        <v>Belmont</v>
+      </c>
+      <c r="H37" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I37" t="str">
+        <v>available</v>
+      </c>
+      <c r="J37" t="str">
+        <v>Solo</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>300ac025-db3a-42ba-a9dd-777f02fb3454</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Jeanette Quy</v>
+      </c>
+      <c r="C38">
+        <v>74</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E38" t="str">
+        <v>koalaleaf@hotmail.com</v>
+      </c>
+      <c r="F38" t="str">
+        <v>402902273</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Rowville</v>
+      </c>
+      <c r="H38" t="str">
+        <v>C</v>
+      </c>
+      <c r="I38" t="str">
+        <v>available</v>
+      </c>
+      <c r="J38" t="str">
+        <v>Husband Ted Quy b6042a-1-1872960</v>
+      </c>
+      <c r="M38" t="str">
+        <v xml:space="preserve">Nothing of note </v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>0ea22efb-f85f-400a-b28d-d1312568ba67</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Jess Cossari</v>
+      </c>
+      <c r="C39">
+        <v>35</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Jcossari@hotmail.com</v>
+      </c>
+      <c r="F39" t="str">
+        <v xml:space="preserve">0458 746 551 </v>
+      </c>
+      <c r="G39" t="str">
+        <v xml:space="preserve">Melbourne </v>
+      </c>
+      <c r="H39" t="str">
+        <v>C</v>
+      </c>
+      <c r="I39" t="str">
+        <v>available</v>
+      </c>
+      <c r="J39" t="str">
+        <v>Andrea Cocco</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>646d2ff7-803b-4c80-bdd6-09d44eec6929</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Leanne Bryant</v>
+      </c>
+      <c r="C40">
+        <v>63</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E40" t="str">
+        <v>blazeandcougar@gmail.com</v>
+      </c>
+      <c r="F40" t="str">
+        <v>61415438228</v>
+      </c>
+      <c r="G40" t="str">
+        <v xml:space="preserve">Hampton Park </v>
+      </c>
+      <c r="H40" t="str">
+        <v>B</v>
+      </c>
+      <c r="I40" t="str">
+        <v>available</v>
+      </c>
+      <c r="J40" t="str">
+        <v>Solo</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>c60666dd-e08c-4aa0-8582-4e7a3ad280f8</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Bashar Mona</v>
+      </c>
+      <c r="C41">
+        <v>33</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E41" t="str">
+        <v>bashar.mona92@gmail.com</v>
+      </c>
+      <c r="F41" t="str">
+        <v>490871416</v>
+      </c>
+      <c r="G41" t="str">
+        <v>Roxburgh park</v>
+      </c>
+      <c r="H41" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I41" t="str">
+        <v>available</v>
+      </c>
+      <c r="J41" t="str">
+        <v>Solo</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>2aadb3db-ad8e-4edd-a81d-f045a926ceb9</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Alexander Leonard</v>
+      </c>
+      <c r="C42">
+        <v>38</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E42" t="str">
+        <v>alexleonardedit@gmail.com</v>
+      </c>
+      <c r="F42" t="str">
+        <v>421834476</v>
+      </c>
+      <c r="G42" t="str">
+        <v>Croydon</v>
+      </c>
+      <c r="H42" t="str">
+        <v>A+</v>
+      </c>
+      <c r="I42" t="str">
+        <v>available</v>
+      </c>
+      <c r="J42" t="str">
+        <v>melissa francis, Alexander Leonard</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>441f345e-57a2-403b-a9a9-8284261eba7b</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Kadisha  Bruton</v>
+      </c>
+      <c r="C43">
+        <v>23</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E43" t="str">
+        <v>kadishaann@icloud.com</v>
+      </c>
+      <c r="F43" t="str">
+        <v>434829249</v>
+      </c>
+      <c r="G43" t="str">
+        <v xml:space="preserve">Kurunjang </v>
+      </c>
+      <c r="H43" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I43" t="str">
+        <v>available</v>
+      </c>
+      <c r="J43" t="str">
+        <v>Jacob Steele</v>
+      </c>
+    </row>
+    <row r="44" xml:space="preserve">
+      <c r="A44" t="str">
+        <v>37fadce4-5d89-4542-a6e1-5e3e50620b85</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Sharyn  McKinnis</v>
+      </c>
+      <c r="C44">
+        <v>50</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E44" t="str">
+        <v>s.lmckinnis@bigpond.com</v>
+      </c>
+      <c r="F44" t="str">
+        <v>419880873</v>
+      </c>
+      <c r="G44" t="str">
+        <v>Newtown</v>
+      </c>
+      <c r="H44" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I44" t="str">
+        <v>available</v>
+      </c>
+      <c r="J44" t="str" xml:space="preserve">
+        <v xml:space="preserve">Isabelle McKinnis, Sharyn McKinnis
+</v>
+      </c>
+    </row>
+    <row r="45" xml:space="preserve">
+      <c r="A45" t="str">
+        <v>23f118f9-20db-422c-8cef-939dc73dd803</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Paige Greig</v>
+      </c>
+      <c r="C45">
+        <v>31</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E45" t="str">
+        <v>paigegreig@hotmail.com</v>
+      </c>
+      <c r="F45" t="str">
+        <v>406598552</v>
+      </c>
+      <c r="G45" t="str">
+        <v>Mooroolbark</v>
+      </c>
+      <c r="H45" t="str">
+        <v>C</v>
+      </c>
+      <c r="I45" t="str">
+        <v>available</v>
+      </c>
+      <c r="J45" t="str" xml:space="preserve">
+        <v xml:space="preserve">Erin
+Morgan (sister) - need to do application</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>cfd3f567-ab69-4fa9-8a35-ca9c949fba91</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Michael Stevens</v>
+      </c>
+      <c r="C46">
+        <v>32</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E46" t="str">
+        <v>mjstevens1306@gmail.com</v>
+      </c>
+      <c r="F46" t="str">
+        <v>424659733</v>
+      </c>
+      <c r="G46" t="str">
+        <v xml:space="preserve">Heathcote Junction </v>
+      </c>
+      <c r="H46" t="str">
+        <v>A</v>
+      </c>
+      <c r="I46" t="str">
+        <v>available</v>
+      </c>
+      <c r="J46" t="str">
+        <v>Libby Dunbar</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>f50d5074-9b3e-4386-9039-5e4cbd121267</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Keera Bell</v>
+      </c>
+      <c r="C47">
+        <v>44</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E47" t="str">
+        <v>Keera_b@hotmail.com</v>
+      </c>
+      <c r="F47" t="str">
+        <v>404754383</v>
+      </c>
+      <c r="G47" t="str">
+        <v xml:space="preserve">Melbourne </v>
+      </c>
+      <c r="H47" t="str">
+        <v>B</v>
+      </c>
+      <c r="I47" t="str">
+        <v>available</v>
+      </c>
+      <c r="J47" t="str">
+        <v>Dek Bell</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>cbfeb8b0-bd5d-4614-a055-cbac047cf152</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Tamika Colville</v>
+      </c>
+      <c r="C48">
+        <v>31</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E48" t="str">
+        <v>tamika.colville@gmail.com</v>
+      </c>
+      <c r="F48" t="str">
+        <v>409132141</v>
+      </c>
+      <c r="G48" t="str">
+        <v>Golden square</v>
+      </c>
+      <c r="H48" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I48" t="str">
+        <v>available</v>
+      </c>
+      <c r="J48" t="str">
+        <v>Shinae Colville</v>
+      </c>
+      <c r="L48" t="str">
+        <v>Diagnosed with MS in 2018</v>
+      </c>
+      <c r="M48" t="str">
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>0b96f877-e1c4-4c17-aa89-21b4a5f7f002</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Stephen Deacon</v>
+      </c>
+      <c r="C49">
+        <v>67</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E49" t="str">
+        <v>StephenDeacon@duck.com</v>
+      </c>
+      <c r="F49" t="str">
+        <v>435353108</v>
+      </c>
+      <c r="G49" t="str">
+        <v>St Kilda</v>
+      </c>
+      <c r="H49" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I49" t="str">
+        <v>available</v>
+      </c>
+      <c r="J49" t="str">
+        <v>Chanyapach Deacon</v>
+      </c>
+    </row>
+    <row r="50" xml:space="preserve">
+      <c r="A50" t="str">
+        <v>54de1dd9-b7eb-489d-b4a1-8b3744a385c4</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Dhananjay  Mehra</v>
+      </c>
+      <c r="C50">
+        <v>68</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Dmehra@bigpond.net.au</v>
+      </c>
+      <c r="F50" t="str">
+        <v>419353328</v>
+      </c>
+      <c r="G50" t="str">
+        <v xml:space="preserve">Point Cook </v>
+      </c>
+      <c r="H50" t="str">
+        <v>B</v>
+      </c>
+      <c r="I50" t="str">
+        <v>available</v>
+      </c>
+      <c r="J50" t="str" xml:space="preserve">
+        <v xml:space="preserve">Meenakshi Mehra
+Dhananjay Mehra</v>
+      </c>
+    </row>
+    <row r="51" xml:space="preserve">
+      <c r="A51" t="str">
+        <v>1211456d-ea92-4a7b-9d94-885982cf345c</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Bronwyn Parsons</v>
+      </c>
+      <c r="C51">
+        <v>72</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E51" t="str">
+        <v>Babybear61153@gmail.com</v>
+      </c>
+      <c r="F51" t="str">
+        <v>432543647</v>
+      </c>
+      <c r="G51" t="str">
+        <v>Rosebud</v>
+      </c>
+      <c r="H51" t="str">
+        <v>A+</v>
+      </c>
+      <c r="I51" t="str">
+        <v>available</v>
+      </c>
+      <c r="J51" t="str" xml:space="preserve">
+        <v xml:space="preserve">Yolette Huon - yol-et Hue on
+Bronwyn Parsons - Would like to be called Bron Emmerson - maiden name</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M51"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>ReferenceNumber</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>f25a6094-c1a5-4eb4-a709-1cc3d9b3ab5e</v>
+      </c>
+      <c r="B2" t="str">
+        <v>GRP001</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
+      </c>
+      <c r="B3" t="str">
+        <v>GRP002</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D27"/>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Enlarge contestant photo view and update contestant data
Increase the maximum width of the photo lightbox dialog in the contestant table component and update contestant data, including swapping contestant records and modifying seat assignments in the automatic backup files.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: f123b9d7-6af8-472a-a75c-70d0b78d0583
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 567b9ccf-b0e0-490c-893d-c27dd95e93f9
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/4ca2a1f8-42ce-4303-beff-eb92e3283d4c/f123b9d7-6af8-472a-a75c-70d0b78d0583/cLj8b3l
</commit_message>
<xml_diff>
--- a/storage/backups/automatic-backup.xlsx
+++ b/storage/backups/automatic-backup.xlsx
@@ -5,8 +5,9 @@
   <sheets>
     <sheet name="Record Days" sheetId="1" r:id="rId1"/>
     <sheet name="Contestants" sheetId="2" r:id="rId2"/>
-    <sheet name="Groups" sheetId="3" r:id="rId3"/>
-    <sheet name="Block Types" sheetId="4" r:id="rId4"/>
+    <sheet name="Seat Assignments" sheetId="3" r:id="rId3"/>
+    <sheet name="Groups" sheetId="4" r:id="rId4"/>
+    <sheet name="Block Types" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -709,27 +710,27 @@
         <v>MobilityNotes</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>34b3d848-f096-4bc9-bd55-dc4dd85ad1b3</v>
+        <v>7fc083f6-6be3-42bf-b4e5-fc6412e1c559</v>
       </c>
       <c r="B2" t="str">
-        <v>Donna Collins</v>
+        <v>Meenakshi  Mehra</v>
       </c>
       <c r="C2">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D2" t="str">
         <v>Female</v>
       </c>
       <c r="E2" t="str">
-        <v>Donna0@hotmail.com</v>
+        <v>meenu.mehra@bigpond.com</v>
       </c>
       <c r="F2" t="str">
-        <v>408122305</v>
+        <v>420353322</v>
       </c>
       <c r="G2" t="str">
-        <v xml:space="preserve">Coburg </v>
+        <v xml:space="preserve">Melbourne </v>
       </c>
       <c r="H2" t="str">
         <v>B</v>
@@ -737,41 +738,41 @@
       <c r="I2" t="str">
         <v>available</v>
       </c>
-      <c r="J2" t="str">
-        <v>Donna Collins, Tom Collins</v>
-      </c>
-    </row>
-    <row r="3" xml:space="preserve">
+      <c r="J2" t="str" xml:space="preserve">
+        <v xml:space="preserve">Meenakshi Mehra
+Dhananjay Mehra</v>
+      </c>
+    </row>
+    <row r="3">
       <c r="A3" t="str">
-        <v>7fc083f6-6be3-42bf-b4e5-fc6412e1c559</v>
+        <v>34b3d848-f096-4bc9-bd55-dc4dd85ad1b3</v>
       </c>
       <c r="B3" t="str">
-        <v>Meenakshi  Mehra</v>
+        <v>Donna Collins</v>
       </c>
       <c r="C3">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D3" t="str">
         <v>Female</v>
       </c>
       <c r="E3" t="str">
-        <v>meenu.mehra@bigpond.com</v>
+        <v>Donna0@hotmail.com</v>
       </c>
       <c r="F3" t="str">
-        <v>420353322</v>
+        <v>408122305</v>
       </c>
       <c r="G3" t="str">
-        <v xml:space="preserve">Melbourne </v>
+        <v xml:space="preserve">Coburg </v>
       </c>
       <c r="H3" t="str">
         <v>B</v>
       </c>
       <c r="I3" t="str">
-        <v>available</v>
-      </c>
-      <c r="J3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Meenakshi Mehra
-Dhananjay Mehra</v>
+        <v>assigned</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Donna Collins, Tom Collins</v>
       </c>
     </row>
     <row r="4">
@@ -2389,6 +2390,60 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>RecordDayID</v>
+      </c>
+      <c r="C1" t="str">
+        <v>ContestantID</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Block</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Seat</v>
+      </c>
+      <c r="F1" t="str">
+        <v>BookingEmailSent</v>
+      </c>
+      <c r="G1" t="str">
+        <v>ConfirmedRSVP</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>1208c385-b9b8-47af-b3d2-f30717990aef</v>
+      </c>
+      <c r="B2" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C2" t="str">
+        <v>34b3d848-f096-4bc9-bd55-dc4dd85ad1b3</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="str">
+        <v>E1</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B3"/>
   <sheetData>
     <row r="1">
@@ -2422,7 +2477,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D27"/>
   <sheetData>

</xml_diff>

<commit_message>
Improve contestant seat assignment dialog for better user experience
Redesign the contestant assignment dialog with enhanced UI/UX, including a clearer header, visual rating indicators, group booking previews, and improved filtering options.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: f123b9d7-6af8-472a-a75c-70d0b78d0583
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 95120401-317f-436b-9e23-9f12856dc0d5
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/4ca2a1f8-42ce-4303-beff-eb92e3283d4c/f123b9d7-6af8-472a-a75c-70d0b78d0583/SA70FQN
</commit_message>
<xml_diff>
--- a/storage/backups/automatic-backup.xlsx
+++ b/storage/backups/automatic-backup.xlsx
@@ -5,9 +5,8 @@
   <sheets>
     <sheet name="Record Days" sheetId="1" r:id="rId1"/>
     <sheet name="Contestants" sheetId="2" r:id="rId2"/>
-    <sheet name="Seat Assignments" sheetId="3" r:id="rId3"/>
-    <sheet name="Groups" sheetId="4" r:id="rId4"/>
-    <sheet name="Block Types" sheetId="5" r:id="rId5"/>
+    <sheet name="Groups" sheetId="3" r:id="rId3"/>
+    <sheet name="Block Types" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -769,7 +768,7 @@
         <v>B</v>
       </c>
       <c r="I3" t="str">
-        <v>assigned</v>
+        <v>available</v>
       </c>
       <c r="J3" t="str">
         <v>Donna Collins, Tom Collins</v>
@@ -2390,60 +2389,6 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>ID</v>
-      </c>
-      <c r="B1" t="str">
-        <v>RecordDayID</v>
-      </c>
-      <c r="C1" t="str">
-        <v>ContestantID</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Block</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Seat</v>
-      </c>
-      <c r="F1" t="str">
-        <v>BookingEmailSent</v>
-      </c>
-      <c r="G1" t="str">
-        <v>ConfirmedRSVP</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Notes</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>1208c385-b9b8-47af-b3d2-f30717990aef</v>
-      </c>
-      <c r="B2" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C2" t="str">
-        <v>34b3d848-f096-4bc9-bd55-dc4dd85ad1b3</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2" t="str">
-        <v>E1</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B3"/>
   <sheetData>
     <row r="1">
@@ -2477,7 +2422,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D27"/>
   <sheetData>

</xml_diff>

<commit_message>
Improve scrolling and sizing of the contestant list dialog
Fixes the contestant list dialog's scroll area by setting a fixed height, resolving previous overflow and visibility issues.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: f123b9d7-6af8-472a-a75c-70d0b78d0583
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 35334692-0383-475b-939e-88104803698a
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/4ca2a1f8-42ce-4303-beff-eb92e3283d4c/f123b9d7-6af8-472a-a75c-70d0b78d0583/SA70FQN
</commit_message>
<xml_diff>
--- a/storage/backups/automatic-backup.xlsx
+++ b/storage/backups/automatic-backup.xlsx
@@ -774,131 +774,134 @@
         <v>Donna Collins, Tom Collins</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" xml:space="preserve">
       <c r="A4" t="str">
-        <v>6b9ae7f0-4a81-4dda-8e55-e49415d98ec6</v>
+        <v>1fe25fd6-dc69-4d29-b22f-9a15ad3d457f</v>
       </c>
       <c r="B4" t="str">
-        <v>Tayla Huxtable</v>
+        <v>Sharon King</v>
       </c>
       <c r="C4">
-        <v>28</v>
+        <v>58</v>
       </c>
       <c r="D4" t="str">
         <v>Female</v>
       </c>
       <c r="E4" t="str">
-        <v>Taylahuxtable@gmail.com</v>
+        <v>dreamweaversixtyseven@gmail.com</v>
       </c>
       <c r="F4" t="str">
-        <v>435320280</v>
+        <v>611488000000</v>
       </c>
       <c r="G4" t="str">
-        <v>FERNTREE GULLY</v>
+        <v xml:space="preserve">Mooroopna </v>
+      </c>
+      <c r="H4" t="str">
+        <v>A</v>
       </c>
       <c r="I4" t="str">
         <v>available</v>
       </c>
-      <c r="J4" t="str">
-        <v>Troy Smith</v>
-      </c>
-      <c r="K4" t="str">
-        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
-      </c>
-    </row>
-    <row r="5" xml:space="preserve">
-      <c r="A5" t="str">
-        <v>1fe25fd6-dc69-4d29-b22f-9a15ad3d457f</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Sharon King</v>
-      </c>
-      <c r="C5">
-        <v>58</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E5" t="str">
-        <v>dreamweaversixtyseven@gmail.com</v>
-      </c>
-      <c r="F5" t="str">
-        <v>611488000000</v>
-      </c>
-      <c r="G5" t="str">
-        <v xml:space="preserve">Mooroopna </v>
-      </c>
-      <c r="H5" t="str">
-        <v>A</v>
-      </c>
-      <c r="I5" t="str">
-        <v>available</v>
-      </c>
-      <c r="J5" t="str" xml:space="preserve">
+      <c r="J4" t="str" xml:space="preserve">
         <v xml:space="preserve">
 Friend :Jacinda Austin
 ID:b6042a-1-1936475</v>
       </c>
-      <c r="M5" t="str">
+      <c r="M4" t="str">
         <v xml:space="preserve">No </v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>8a905dfd-647c-4d96-a741-f7f1517a5136</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Deanna Hay</v>
+      </c>
+      <c r="C5">
+        <v>38</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E5" t="str">
+        <v>dee_hay24@hotmail.com</v>
+      </c>
+      <c r="F5" t="str">
+        <v>424504430</v>
+      </c>
+      <c r="G5" t="str">
+        <v xml:space="preserve">Melbourne </v>
+      </c>
+      <c r="H5" t="str">
+        <v>DNU</v>
+      </c>
+      <c r="I5" t="str">
+        <v>available</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Lynetta Shan Faoa</v>
+      </c>
+      <c r="L5" t="str">
+        <v xml:space="preserve">Cerebral palsy in a wheelchair </v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>8a905dfd-647c-4d96-a741-f7f1517a5136</v>
+        <v>efd8ab2e-988b-4afb-9374-3c3e3676f43a</v>
       </c>
       <c r="B6" t="str">
-        <v>Deanna Hay</v>
+        <v>Matilda Sutherland</v>
       </c>
       <c r="C6">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="D6" t="str">
         <v>Female</v>
       </c>
       <c r="E6" t="str">
-        <v>dee_hay24@hotmail.com</v>
+        <v>matilda.sutherland@hotmail.com</v>
       </c>
       <c r="F6" t="str">
-        <v>424504430</v>
+        <v>0467 165 012</v>
       </c>
       <c r="G6" t="str">
-        <v xml:space="preserve">Melbourne </v>
+        <v>Bundoora</v>
       </c>
       <c r="H6" t="str">
-        <v>DNU</v>
+        <v>B+</v>
       </c>
       <c r="I6" t="str">
         <v>available</v>
       </c>
       <c r="J6" t="str">
-        <v>Lynetta Shan Faoa</v>
-      </c>
-      <c r="L6" t="str">
-        <v xml:space="preserve">Cerebral palsy in a wheelchair </v>
+        <v>Grace Mann</v>
+      </c>
+      <c r="M6" t="str">
+        <v>NA</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>efd8ab2e-988b-4afb-9374-3c3e3676f43a</v>
+        <v>96d2c8ad-1e67-4659-b3d0-a3bbd4fe40cb</v>
       </c>
       <c r="B7" t="str">
-        <v>Matilda Sutherland</v>
+        <v>Karina  Richmond</v>
       </c>
       <c r="C7">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="D7" t="str">
         <v>Female</v>
       </c>
       <c r="E7" t="str">
-        <v>matilda.sutherland@hotmail.com</v>
+        <v>richmondkarina@yahoo.com</v>
       </c>
       <c r="F7" t="str">
-        <v>0467 165 012</v>
+        <v>400554609</v>
       </c>
       <c r="G7" t="str">
-        <v>Bundoora</v>
+        <v>Newcomb</v>
       </c>
       <c r="H7" t="str">
         <v>B+</v>
@@ -907,7 +910,7 @@
         <v>available</v>
       </c>
       <c r="J7" t="str">
-        <v>Grace Mann</v>
+        <v>AMY DILLON</v>
       </c>
       <c r="M7" t="str">
         <v>NA</v>
@@ -915,25 +918,25 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>96d2c8ad-1e67-4659-b3d0-a3bbd4fe40cb</v>
+        <v>7a05a613-1880-40c5-ab6a-cc078b418b6e</v>
       </c>
       <c r="B8" t="str">
-        <v>Karina  Richmond</v>
+        <v>Deb  Jones</v>
       </c>
       <c r="C8">
-        <v>38</v>
+        <v>66</v>
       </c>
       <c r="D8" t="str">
         <v>Female</v>
       </c>
       <c r="E8" t="str">
-        <v>richmondkarina@yahoo.com</v>
+        <v>fullhouse5@optusnet.com.au</v>
       </c>
       <c r="F8" t="str">
-        <v>400554609</v>
+        <v>438561474</v>
       </c>
       <c r="G8" t="str">
-        <v>Newcomb</v>
+        <v>Bayswater North</v>
       </c>
       <c r="H8" t="str">
         <v>B+</v>
@@ -942,33 +945,33 @@
         <v>available</v>
       </c>
       <c r="J8" t="str">
-        <v>AMY DILLON</v>
+        <v>Daryl Jones</v>
       </c>
       <c r="M8" t="str">
-        <v>NA</v>
+        <v>No</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>7a05a613-1880-40c5-ab6a-cc078b418b6e</v>
+        <v>f693566d-ea7c-40d1-89aa-158e842961d0</v>
       </c>
       <c r="B9" t="str">
-        <v>Deb  Jones</v>
+        <v>Brent Barnett</v>
       </c>
       <c r="C9">
-        <v>66</v>
+        <v>37</v>
       </c>
       <c r="D9" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E9" t="str">
-        <v>fullhouse5@optusnet.com.au</v>
+        <v>brentbarnett88@gmail.com</v>
       </c>
       <c r="F9" t="str">
-        <v>438561474</v>
+        <v>423530043</v>
       </c>
       <c r="G9" t="str">
-        <v>Bayswater North</v>
+        <v>Preston</v>
       </c>
       <c r="H9" t="str">
         <v>B+</v>
@@ -977,33 +980,30 @@
         <v>available</v>
       </c>
       <c r="J9" t="str">
-        <v>Daryl Jones</v>
-      </c>
-      <c r="M9" t="str">
-        <v>No</v>
+        <v>Stephanie Squillacioti</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>f693566d-ea7c-40d1-89aa-158e842961d0</v>
+        <v>82960b61-d36b-49e2-9ddf-a7b8e0b02a63</v>
       </c>
       <c r="B10" t="str">
-        <v>Brent Barnett</v>
+        <v>Tara Saltzman</v>
       </c>
       <c r="C10">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="D10" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E10" t="str">
-        <v>brentbarnett88@gmail.com</v>
+        <v>tarasaltzman@bigpond.com</v>
       </c>
       <c r="F10" t="str">
-        <v>423530043</v>
+        <v>448545599</v>
       </c>
       <c r="G10" t="str">
-        <v>Preston</v>
+        <v>Melbourne</v>
       </c>
       <c r="H10" t="str">
         <v>B+</v>
@@ -1012,27 +1012,30 @@
         <v>available</v>
       </c>
       <c r="J10" t="str">
-        <v>Stephanie Squillacioti</v>
+        <v xml:space="preserve">JACK AGIUS - NEEDS TO DO APPLICATION </v>
+      </c>
+      <c r="M10" t="str">
+        <v>NA</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>82960b61-d36b-49e2-9ddf-a7b8e0b02a63</v>
+        <v>b1fc34e8-20cb-4607-9568-0761cf4520a6</v>
       </c>
       <c r="B11" t="str">
-        <v>Tara Saltzman</v>
+        <v>Troy Smith</v>
       </c>
       <c r="C11">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D11" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E11" t="str">
-        <v>tarasaltzman@bigpond.com</v>
+        <v>Troyssmith94@gmail.com</v>
       </c>
       <c r="F11" t="str">
-        <v>448545599</v>
+        <v>429354308</v>
       </c>
       <c r="G11" t="str">
         <v>Melbourne</v>
@@ -1044,7 +1047,13 @@
         <v>available</v>
       </c>
       <c r="J11" t="str">
-        <v xml:space="preserve">JACK AGIUS - NEEDS TO DO APPLICATION </v>
+        <v>Tayla Huxtable</v>
+      </c>
+      <c r="K11" t="str">
+        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
+      </c>
+      <c r="L11" t="str">
+        <v xml:space="preserve">Peanut allergy </v>
       </c>
       <c r="M11" t="str">
         <v>NA</v>
@@ -1052,43 +1061,34 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>b1fc34e8-20cb-4607-9568-0761cf4520a6</v>
+        <v>6b9ae7f0-4a81-4dda-8e55-e49415d98ec6</v>
       </c>
       <c r="B12" t="str">
+        <v>Tayla Huxtable</v>
+      </c>
+      <c r="C12">
+        <v>28</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Taylahuxtable@gmail.com</v>
+      </c>
+      <c r="F12" t="str">
+        <v>435320280</v>
+      </c>
+      <c r="G12" t="str">
+        <v>FERNTREE GULLY</v>
+      </c>
+      <c r="I12" t="str">
+        <v>available</v>
+      </c>
+      <c r="J12" t="str">
         <v>Troy Smith</v>
-      </c>
-      <c r="C12">
-        <v>31</v>
-      </c>
-      <c r="D12" t="str">
-        <v>Male</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Troyssmith94@gmail.com</v>
-      </c>
-      <c r="F12" t="str">
-        <v>429354308</v>
-      </c>
-      <c r="G12" t="str">
-        <v>Melbourne</v>
-      </c>
-      <c r="H12" t="str">
-        <v>B+</v>
-      </c>
-      <c r="I12" t="str">
-        <v>available</v>
-      </c>
-      <c r="J12" t="str">
-        <v>Tayla Huxtable</v>
       </c>
       <c r="K12" t="str">
         <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
-      </c>
-      <c r="L12" t="str">
-        <v xml:space="preserve">Peanut allergy </v>
-      </c>
-      <c r="M12" t="str">
-        <v>NA</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Update contestant data and seat assignments in backup file
Modify `exportedAt` timestamp, update contestant availability status, add a new contestant record, and include seat assignment data in the automatic backup file.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: f123b9d7-6af8-472a-a75c-70d0b78d0583
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 036d7a0f-179f-459e-b315-8c231ad4bd31
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/4ca2a1f8-42ce-4303-beff-eb92e3283d4c/f123b9d7-6af8-472a-a75c-70d0b78d0583/SA70FQN
</commit_message>
<xml_diff>
--- a/storage/backups/automatic-backup.xlsx
+++ b/storage/backups/automatic-backup.xlsx
@@ -5,8 +5,9 @@
   <sheets>
     <sheet name="Record Days" sheetId="1" r:id="rId1"/>
     <sheet name="Contestants" sheetId="2" r:id="rId2"/>
-    <sheet name="Groups" sheetId="3" r:id="rId3"/>
-    <sheet name="Block Types" sheetId="4" r:id="rId4"/>
+    <sheet name="Seat Assignments" sheetId="3" r:id="rId3"/>
+    <sheet name="Groups" sheetId="4" r:id="rId4"/>
+    <sheet name="Block Types" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -953,57 +954,57 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>f693566d-ea7c-40d1-89aa-158e842961d0</v>
+        <v>6b9ae7f0-4a81-4dda-8e55-e49415d98ec6</v>
       </c>
       <c r="B9" t="str">
-        <v>Brent Barnett</v>
+        <v>Tayla Huxtable</v>
       </c>
       <c r="C9">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="D9" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E9" t="str">
-        <v>brentbarnett88@gmail.com</v>
+        <v>Taylahuxtable@gmail.com</v>
       </c>
       <c r="F9" t="str">
-        <v>423530043</v>
+        <v>435320280</v>
       </c>
       <c r="G9" t="str">
-        <v>Preston</v>
-      </c>
-      <c r="H9" t="str">
-        <v>B+</v>
+        <v>FERNTREE GULLY</v>
       </c>
       <c r="I9" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J9" t="str">
-        <v>Stephanie Squillacioti</v>
+        <v>Troy Smith</v>
+      </c>
+      <c r="K9" t="str">
+        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>82960b61-d36b-49e2-9ddf-a7b8e0b02a63</v>
+        <v>f693566d-ea7c-40d1-89aa-158e842961d0</v>
       </c>
       <c r="B10" t="str">
-        <v>Tara Saltzman</v>
+        <v>Brent Barnett</v>
       </c>
       <c r="C10">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="D10" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E10" t="str">
-        <v>tarasaltzman@bigpond.com</v>
+        <v>brentbarnett88@gmail.com</v>
       </c>
       <c r="F10" t="str">
-        <v>448545599</v>
+        <v>423530043</v>
       </c>
       <c r="G10" t="str">
-        <v>Melbourne</v>
+        <v>Preston</v>
       </c>
       <c r="H10" t="str">
         <v>B+</v>
@@ -1012,30 +1013,27 @@
         <v>available</v>
       </c>
       <c r="J10" t="str">
-        <v xml:space="preserve">JACK AGIUS - NEEDS TO DO APPLICATION </v>
-      </c>
-      <c r="M10" t="str">
-        <v>NA</v>
+        <v>Stephanie Squillacioti</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>b1fc34e8-20cb-4607-9568-0761cf4520a6</v>
+        <v>82960b61-d36b-49e2-9ddf-a7b8e0b02a63</v>
       </c>
       <c r="B11" t="str">
-        <v>Troy Smith</v>
+        <v>Tara Saltzman</v>
       </c>
       <c r="C11">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D11" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E11" t="str">
-        <v>Troyssmith94@gmail.com</v>
+        <v>tarasaltzman@bigpond.com</v>
       </c>
       <c r="F11" t="str">
-        <v>429354308</v>
+        <v>448545599</v>
       </c>
       <c r="G11" t="str">
         <v>Melbourne</v>
@@ -1047,13 +1045,7 @@
         <v>available</v>
       </c>
       <c r="J11" t="str">
-        <v>Tayla Huxtable</v>
-      </c>
-      <c r="K11" t="str">
-        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
-      </c>
-      <c r="L11" t="str">
-        <v xml:space="preserve">Peanut allergy </v>
+        <v xml:space="preserve">JACK AGIUS - NEEDS TO DO APPLICATION </v>
       </c>
       <c r="M11" t="str">
         <v>NA</v>
@@ -1061,34 +1053,43 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>6b9ae7f0-4a81-4dda-8e55-e49415d98ec6</v>
+        <v>b1fc34e8-20cb-4607-9568-0761cf4520a6</v>
       </c>
       <c r="B12" t="str">
+        <v>Troy Smith</v>
+      </c>
+      <c r="C12">
+        <v>31</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Troyssmith94@gmail.com</v>
+      </c>
+      <c r="F12" t="str">
+        <v>429354308</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Melbourne</v>
+      </c>
+      <c r="H12" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I12" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="J12" t="str">
         <v>Tayla Huxtable</v>
-      </c>
-      <c r="C12">
-        <v>28</v>
-      </c>
-      <c r="D12" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Taylahuxtable@gmail.com</v>
-      </c>
-      <c r="F12" t="str">
-        <v>435320280</v>
-      </c>
-      <c r="G12" t="str">
-        <v>FERNTREE GULLY</v>
-      </c>
-      <c r="I12" t="str">
-        <v>available</v>
-      </c>
-      <c r="J12" t="str">
-        <v>Troy Smith</v>
       </c>
       <c r="K12" t="str">
         <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
+      </c>
+      <c r="L12" t="str">
+        <v xml:space="preserve">Peanut allergy </v>
+      </c>
+      <c r="M12" t="str">
+        <v>NA</v>
       </c>
     </row>
     <row r="13">
@@ -2389,6 +2390,77 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>RecordDayID</v>
+      </c>
+      <c r="C1" t="str">
+        <v>ContestantID</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Block</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Seat</v>
+      </c>
+      <c r="F1" t="str">
+        <v>BookingEmailSent</v>
+      </c>
+      <c r="G1" t="str">
+        <v>ConfirmedRSVP</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>73d6afb0-cfb6-4853-ba4e-78207c8c06d5</v>
+      </c>
+      <c r="B2" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C2" t="str">
+        <v>b1fc34e8-20cb-4607-9568-0761cf4520a6</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="str">
+        <v>E2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>cd112197-9251-4276-b185-2ade91c758f2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C3" t="str">
+        <v>6b9ae7f0-4a81-4dda-8e55-e49415d98ec6</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3" t="str">
+        <v>E3</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B3"/>
   <sheetData>
     <row r="1">
@@ -2422,7 +2494,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D27"/>
   <sheetData>

</xml_diff>

<commit_message>
Improve contestant auto-assignment by correctly identifying solo attendees
Adjust auto-assignment logic to treat contestants with 'Solo' or similar indicators in attendingWith as solo participants, preventing them from being skipped due to missing partners.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: f123b9d7-6af8-472a-a75c-70d0b78d0583
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 28a7e076-93b9-43cb-8bee-5acfb1fb4298
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/4ca2a1f8-42ce-4303-beff-eb92e3283d4c/f123b9d7-6af8-472a-a75c-70d0b78d0583/SA70FQN
</commit_message>
<xml_diff>
--- a/storage/backups/automatic-backup.xlsx
+++ b/storage/backups/automatic-backup.xlsx
@@ -5,9 +5,8 @@
   <sheets>
     <sheet name="Record Days" sheetId="1" r:id="rId1"/>
     <sheet name="Contestants" sheetId="2" r:id="rId2"/>
-    <sheet name="Seat Assignments" sheetId="3" r:id="rId3"/>
-    <sheet name="Groups" sheetId="4" r:id="rId4"/>
-    <sheet name="Block Types" sheetId="5" r:id="rId5"/>
+    <sheet name="Groups" sheetId="3" r:id="rId3"/>
+    <sheet name="Block Types" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -954,89 +953,98 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>6b9ae7f0-4a81-4dda-8e55-e49415d98ec6</v>
+        <v>b1fc34e8-20cb-4607-9568-0761cf4520a6</v>
       </c>
       <c r="B9" t="str">
+        <v>Troy Smith</v>
+      </c>
+      <c r="C9">
+        <v>31</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Troyssmith94@gmail.com</v>
+      </c>
+      <c r="F9" t="str">
+        <v>429354308</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Melbourne</v>
+      </c>
+      <c r="H9" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I9" t="str">
+        <v>available</v>
+      </c>
+      <c r="J9" t="str">
         <v>Tayla Huxtable</v>
-      </c>
-      <c r="C9">
-        <v>28</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Taylahuxtable@gmail.com</v>
-      </c>
-      <c r="F9" t="str">
-        <v>435320280</v>
-      </c>
-      <c r="G9" t="str">
-        <v>FERNTREE GULLY</v>
-      </c>
-      <c r="I9" t="str">
-        <v>assigned</v>
-      </c>
-      <c r="J9" t="str">
-        <v>Troy Smith</v>
       </c>
       <c r="K9" t="str">
         <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
       </c>
+      <c r="L9" t="str">
+        <v xml:space="preserve">Peanut allergy </v>
+      </c>
+      <c r="M9" t="str">
+        <v>NA</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>f693566d-ea7c-40d1-89aa-158e842961d0</v>
+        <v>6b9ae7f0-4a81-4dda-8e55-e49415d98ec6</v>
       </c>
       <c r="B10" t="str">
-        <v>Brent Barnett</v>
+        <v>Tayla Huxtable</v>
       </c>
       <c r="C10">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="D10" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E10" t="str">
-        <v>brentbarnett88@gmail.com</v>
+        <v>Taylahuxtable@gmail.com</v>
       </c>
       <c r="F10" t="str">
-        <v>423530043</v>
+        <v>435320280</v>
       </c>
       <c r="G10" t="str">
-        <v>Preston</v>
-      </c>
-      <c r="H10" t="str">
-        <v>B+</v>
+        <v>FERNTREE GULLY</v>
       </c>
       <c r="I10" t="str">
         <v>available</v>
       </c>
       <c r="J10" t="str">
-        <v>Stephanie Squillacioti</v>
+        <v>Troy Smith</v>
+      </c>
+      <c r="K10" t="str">
+        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>82960b61-d36b-49e2-9ddf-a7b8e0b02a63</v>
+        <v>f693566d-ea7c-40d1-89aa-158e842961d0</v>
       </c>
       <c r="B11" t="str">
-        <v>Tara Saltzman</v>
+        <v>Brent Barnett</v>
       </c>
       <c r="C11">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="D11" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E11" t="str">
-        <v>tarasaltzman@bigpond.com</v>
+        <v>brentbarnett88@gmail.com</v>
       </c>
       <c r="F11" t="str">
-        <v>448545599</v>
+        <v>423530043</v>
       </c>
       <c r="G11" t="str">
-        <v>Melbourne</v>
+        <v>Preston</v>
       </c>
       <c r="H11" t="str">
         <v>B+</v>
@@ -1045,30 +1053,27 @@
         <v>available</v>
       </c>
       <c r="J11" t="str">
-        <v xml:space="preserve">JACK AGIUS - NEEDS TO DO APPLICATION </v>
-      </c>
-      <c r="M11" t="str">
-        <v>NA</v>
+        <v>Stephanie Squillacioti</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>b1fc34e8-20cb-4607-9568-0761cf4520a6</v>
+        <v>82960b61-d36b-49e2-9ddf-a7b8e0b02a63</v>
       </c>
       <c r="B12" t="str">
-        <v>Troy Smith</v>
+        <v>Tara Saltzman</v>
       </c>
       <c r="C12">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D12" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E12" t="str">
-        <v>Troyssmith94@gmail.com</v>
+        <v>tarasaltzman@bigpond.com</v>
       </c>
       <c r="F12" t="str">
-        <v>429354308</v>
+        <v>448545599</v>
       </c>
       <c r="G12" t="str">
         <v>Melbourne</v>
@@ -1077,16 +1082,10 @@
         <v>B+</v>
       </c>
       <c r="I12" t="str">
-        <v>assigned</v>
+        <v>available</v>
       </c>
       <c r="J12" t="str">
-        <v>Tayla Huxtable</v>
-      </c>
-      <c r="K12" t="str">
-        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
-      </c>
-      <c r="L12" t="str">
-        <v xml:space="preserve">Peanut allergy </v>
+        <v xml:space="preserve">JACK AGIUS - NEEDS TO DO APPLICATION </v>
       </c>
       <c r="M12" t="str">
         <v>NA</v>
@@ -2390,77 +2389,6 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H3"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>ID</v>
-      </c>
-      <c r="B1" t="str">
-        <v>RecordDayID</v>
-      </c>
-      <c r="C1" t="str">
-        <v>ContestantID</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Block</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Seat</v>
-      </c>
-      <c r="F1" t="str">
-        <v>BookingEmailSent</v>
-      </c>
-      <c r="G1" t="str">
-        <v>ConfirmedRSVP</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Notes</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>73d6afb0-cfb6-4853-ba4e-78207c8c06d5</v>
-      </c>
-      <c r="B2" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C2" t="str">
-        <v>b1fc34e8-20cb-4607-9568-0761cf4520a6</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2" t="str">
-        <v>E2</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>cd112197-9251-4276-b185-2ade91c758f2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C3" t="str">
-        <v>6b9ae7f0-4a81-4dda-8e55-e49415d98ec6</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3" t="str">
-        <v>E3</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B3"/>
   <sheetData>
     <row r="1">
@@ -2494,7 +2422,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D27"/>
   <sheetData>

</xml_diff>

<commit_message>
Make the contestant assignment dialog larger for easier use
Update the seating chart page to increase the size of the contestant assignment dialog from max-w-2xl to max-w-4xl and max-h-85vh to max-h-90vh. Also, update the automatic backup file with new exportedAt timestamp and modified contestant availability statuses.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: f123b9d7-6af8-472a-a75c-70d0b78d0583
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: b0c911aa-cf73-4e43-905c-4f76bb81a0db
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/4ca2a1f8-42ce-4303-beff-eb92e3283d4c/f123b9d7-6af8-472a-a75c-70d0b78d0583/SA70FQN
</commit_message>
<xml_diff>
--- a/storage/backups/automatic-backup.xlsx
+++ b/storage/backups/automatic-backup.xlsx
@@ -5,8 +5,9 @@
   <sheets>
     <sheet name="Record Days" sheetId="1" r:id="rId1"/>
     <sheet name="Contestants" sheetId="2" r:id="rId2"/>
-    <sheet name="Groups" sheetId="3" r:id="rId3"/>
-    <sheet name="Block Types" sheetId="4" r:id="rId4"/>
+    <sheet name="Seat Assignments" sheetId="3" r:id="rId3"/>
+    <sheet name="Groups" sheetId="4" r:id="rId4"/>
+    <sheet name="Block Types" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -953,25 +954,25 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>b1fc34e8-20cb-4607-9568-0761cf4520a6</v>
+        <v>f693566d-ea7c-40d1-89aa-158e842961d0</v>
       </c>
       <c r="B9" t="str">
-        <v>Troy Smith</v>
+        <v>Brent Barnett</v>
       </c>
       <c r="C9">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D9" t="str">
         <v>Male</v>
       </c>
       <c r="E9" t="str">
-        <v>Troyssmith94@gmail.com</v>
+        <v>brentbarnett88@gmail.com</v>
       </c>
       <c r="F9" t="str">
-        <v>429354308</v>
+        <v>423530043</v>
       </c>
       <c r="G9" t="str">
-        <v>Melbourne</v>
+        <v>Preston</v>
       </c>
       <c r="H9" t="str">
         <v>B+</v>
@@ -980,115 +981,115 @@
         <v>available</v>
       </c>
       <c r="J9" t="str">
-        <v>Tayla Huxtable</v>
-      </c>
-      <c r="K9" t="str">
-        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
-      </c>
-      <c r="L9" t="str">
-        <v xml:space="preserve">Peanut allergy </v>
-      </c>
-      <c r="M9" t="str">
-        <v>NA</v>
+        <v>Stephanie Squillacioti</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>6b9ae7f0-4a81-4dda-8e55-e49415d98ec6</v>
+        <v>82960b61-d36b-49e2-9ddf-a7b8e0b02a63</v>
       </c>
       <c r="B10" t="str">
-        <v>Tayla Huxtable</v>
+        <v>Tara Saltzman</v>
       </c>
       <c r="C10">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D10" t="str">
         <v>Female</v>
       </c>
       <c r="E10" t="str">
-        <v>Taylahuxtable@gmail.com</v>
+        <v>tarasaltzman@bigpond.com</v>
       </c>
       <c r="F10" t="str">
-        <v>435320280</v>
+        <v>448545599</v>
       </c>
       <c r="G10" t="str">
-        <v>FERNTREE GULLY</v>
+        <v>Melbourne</v>
+      </c>
+      <c r="H10" t="str">
+        <v>B+</v>
       </c>
       <c r="I10" t="str">
         <v>available</v>
       </c>
       <c r="J10" t="str">
-        <v>Troy Smith</v>
-      </c>
-      <c r="K10" t="str">
-        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
+        <v xml:space="preserve">JACK AGIUS - NEEDS TO DO APPLICATION </v>
+      </c>
+      <c r="M10" t="str">
+        <v>NA</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>f693566d-ea7c-40d1-89aa-158e842961d0</v>
+        <v>b1fc34e8-20cb-4607-9568-0761cf4520a6</v>
       </c>
       <c r="B11" t="str">
-        <v>Brent Barnett</v>
+        <v>Troy Smith</v>
       </c>
       <c r="C11">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="D11" t="str">
         <v>Male</v>
       </c>
       <c r="E11" t="str">
-        <v>brentbarnett88@gmail.com</v>
+        <v>Troyssmith94@gmail.com</v>
       </c>
       <c r="F11" t="str">
-        <v>423530043</v>
+        <v>429354308</v>
       </c>
       <c r="G11" t="str">
-        <v>Preston</v>
+        <v>Melbourne</v>
       </c>
       <c r="H11" t="str">
         <v>B+</v>
       </c>
       <c r="I11" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J11" t="str">
-        <v>Stephanie Squillacioti</v>
+        <v>Tayla Huxtable</v>
+      </c>
+      <c r="K11" t="str">
+        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
+      </c>
+      <c r="L11" t="str">
+        <v xml:space="preserve">Peanut allergy </v>
+      </c>
+      <c r="M11" t="str">
+        <v>NA</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>82960b61-d36b-49e2-9ddf-a7b8e0b02a63</v>
+        <v>6b9ae7f0-4a81-4dda-8e55-e49415d98ec6</v>
       </c>
       <c r="B12" t="str">
-        <v>Tara Saltzman</v>
+        <v>Tayla Huxtable</v>
       </c>
       <c r="C12">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D12" t="str">
         <v>Female</v>
       </c>
       <c r="E12" t="str">
-        <v>tarasaltzman@bigpond.com</v>
+        <v>Taylahuxtable@gmail.com</v>
       </c>
       <c r="F12" t="str">
-        <v>448545599</v>
+        <v>435320280</v>
       </c>
       <c r="G12" t="str">
-        <v>Melbourne</v>
-      </c>
-      <c r="H12" t="str">
-        <v>B+</v>
+        <v>FERNTREE GULLY</v>
       </c>
       <c r="I12" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J12" t="str">
-        <v xml:space="preserve">JACK AGIUS - NEEDS TO DO APPLICATION </v>
-      </c>
-      <c r="M12" t="str">
-        <v>NA</v>
+        <v>Troy Smith</v>
+      </c>
+      <c r="K12" t="str">
+        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
       </c>
     </row>
     <row r="13">
@@ -2389,6 +2390,77 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>RecordDayID</v>
+      </c>
+      <c r="C1" t="str">
+        <v>ContestantID</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Block</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Seat</v>
+      </c>
+      <c r="F1" t="str">
+        <v>BookingEmailSent</v>
+      </c>
+      <c r="G1" t="str">
+        <v>ConfirmedRSVP</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ad340cba-9702-4a35-9a1f-7098bb2792d2</v>
+      </c>
+      <c r="B2" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C2" t="str">
+        <v>b1fc34e8-20cb-4607-9568-0761cf4520a6</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="str">
+        <v>A1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>055b0eeb-95e3-48d2-bab8-608bbe0173ce</v>
+      </c>
+      <c r="B3" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C3" t="str">
+        <v>6b9ae7f0-4a81-4dda-8e55-e49415d98ec6</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3" t="str">
+        <v>A2</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B3"/>
   <sheetData>
     <row r="1">
@@ -2422,7 +2494,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D27"/>
   <sheetData>

</xml_diff>

<commit_message>
Refine solo partner detection logic to improve contestant assignment
Update the `isSoloIndicator` function to differentiate between exact solo matches and contained phrases, preventing misclassification of contestants with dashes in their `attendingWith` field.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: f123b9d7-6af8-472a-a75c-70d0b78d0583
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 763731b5-3c84-4c7a-bbb8-e6b2ffa8d996
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/4ca2a1f8-42ce-4303-beff-eb92e3283d4c/f123b9d7-6af8-472a-a75c-70d0b78d0583/SA70FQN
</commit_message>
<xml_diff>
--- a/storage/backups/automatic-backup.xlsx
+++ b/storage/backups/automatic-backup.xlsx
@@ -736,7 +736,7 @@
         <v>B</v>
       </c>
       <c r="I2" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J2" t="str" xml:space="preserve">
         <v xml:space="preserve">Meenakshi Mehra
@@ -769,242 +769,245 @@
         <v>B</v>
       </c>
       <c r="I3" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J3" t="str">
         <v>Donna Collins, Tom Collins</v>
       </c>
     </row>
-    <row r="4" xml:space="preserve">
+    <row r="4">
       <c r="A4" t="str">
-        <v>1fe25fd6-dc69-4d29-b22f-9a15ad3d457f</v>
+        <v>8a905dfd-647c-4d96-a741-f7f1517a5136</v>
       </c>
       <c r="B4" t="str">
-        <v>Sharon King</v>
+        <v>Deanna Hay</v>
       </c>
       <c r="C4">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="D4" t="str">
         <v>Female</v>
       </c>
       <c r="E4" t="str">
-        <v>dreamweaversixtyseven@gmail.com</v>
+        <v>dee_hay24@hotmail.com</v>
       </c>
       <c r="F4" t="str">
-        <v>611488000000</v>
+        <v>424504430</v>
       </c>
       <c r="G4" t="str">
-        <v xml:space="preserve">Mooroopna </v>
+        <v xml:space="preserve">Melbourne </v>
       </c>
       <c r="H4" t="str">
-        <v>A</v>
+        <v>DNU</v>
       </c>
       <c r="I4" t="str">
         <v>available</v>
       </c>
-      <c r="J4" t="str" xml:space="preserve">
+      <c r="J4" t="str">
+        <v>Lynetta Shan Faoa</v>
+      </c>
+      <c r="L4" t="str">
+        <v xml:space="preserve">Cerebral palsy in a wheelchair </v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>efd8ab2e-988b-4afb-9374-3c3e3676f43a</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Matilda Sutherland</v>
+      </c>
+      <c r="C5">
+        <v>26</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E5" t="str">
+        <v>matilda.sutherland@hotmail.com</v>
+      </c>
+      <c r="F5" t="str">
+        <v>0467 165 012</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Bundoora</v>
+      </c>
+      <c r="H5" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I5" t="str">
+        <v>available</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Grace Mann</v>
+      </c>
+      <c r="M5" t="str">
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>96d2c8ad-1e67-4659-b3d0-a3bbd4fe40cb</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Karina  Richmond</v>
+      </c>
+      <c r="C6">
+        <v>38</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E6" t="str">
+        <v>richmondkarina@yahoo.com</v>
+      </c>
+      <c r="F6" t="str">
+        <v>400554609</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Newcomb</v>
+      </c>
+      <c r="H6" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I6" t="str">
+        <v>available</v>
+      </c>
+      <c r="J6" t="str">
+        <v>AMY DILLON</v>
+      </c>
+      <c r="M6" t="str">
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>7a05a613-1880-40c5-ab6a-cc078b418b6e</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Deb  Jones</v>
+      </c>
+      <c r="C7">
+        <v>66</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E7" t="str">
+        <v>fullhouse5@optusnet.com.au</v>
+      </c>
+      <c r="F7" t="str">
+        <v>438561474</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Bayswater North</v>
+      </c>
+      <c r="H7" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I7" t="str">
+        <v>available</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Daryl Jones</v>
+      </c>
+      <c r="M7" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>1fe25fd6-dc69-4d29-b22f-9a15ad3d457f</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Sharon King</v>
+      </c>
+      <c r="C8">
+        <v>58</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E8" t="str">
+        <v>dreamweaversixtyseven@gmail.com</v>
+      </c>
+      <c r="F8" t="str">
+        <v>611488000000</v>
+      </c>
+      <c r="G8" t="str">
+        <v xml:space="preserve">Mooroopna </v>
+      </c>
+      <c r="H8" t="str">
+        <v>A</v>
+      </c>
+      <c r="I8" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="J8" t="str" xml:space="preserve">
         <v xml:space="preserve">
 Friend :Jacinda Austin
 ID:b6042a-1-1936475</v>
       </c>
-      <c r="M4" t="str">
+      <c r="M8" t="str">
         <v xml:space="preserve">No </v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>8a905dfd-647c-4d96-a741-f7f1517a5136</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Deanna Hay</v>
-      </c>
-      <c r="C5">
-        <v>38</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E5" t="str">
-        <v>dee_hay24@hotmail.com</v>
-      </c>
-      <c r="F5" t="str">
-        <v>424504430</v>
-      </c>
-      <c r="G5" t="str">
-        <v xml:space="preserve">Melbourne </v>
-      </c>
-      <c r="H5" t="str">
-        <v>DNU</v>
-      </c>
-      <c r="I5" t="str">
-        <v>available</v>
-      </c>
-      <c r="J5" t="str">
-        <v>Lynetta Shan Faoa</v>
-      </c>
-      <c r="L5" t="str">
-        <v xml:space="preserve">Cerebral palsy in a wheelchair </v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>efd8ab2e-988b-4afb-9374-3c3e3676f43a</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Matilda Sutherland</v>
-      </c>
-      <c r="C6">
-        <v>26</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E6" t="str">
-        <v>matilda.sutherland@hotmail.com</v>
-      </c>
-      <c r="F6" t="str">
-        <v>0467 165 012</v>
-      </c>
-      <c r="G6" t="str">
-        <v>Bundoora</v>
-      </c>
-      <c r="H6" t="str">
-        <v>B+</v>
-      </c>
-      <c r="I6" t="str">
-        <v>available</v>
-      </c>
-      <c r="J6" t="str">
-        <v>Grace Mann</v>
-      </c>
-      <c r="M6" t="str">
-        <v>NA</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>96d2c8ad-1e67-4659-b3d0-a3bbd4fe40cb</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Karina  Richmond</v>
-      </c>
-      <c r="C7">
-        <v>38</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E7" t="str">
-        <v>richmondkarina@yahoo.com</v>
-      </c>
-      <c r="F7" t="str">
-        <v>400554609</v>
-      </c>
-      <c r="G7" t="str">
-        <v>Newcomb</v>
-      </c>
-      <c r="H7" t="str">
-        <v>B+</v>
-      </c>
-      <c r="I7" t="str">
-        <v>available</v>
-      </c>
-      <c r="J7" t="str">
-        <v>AMY DILLON</v>
-      </c>
-      <c r="M7" t="str">
-        <v>NA</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>7a05a613-1880-40c5-ab6a-cc078b418b6e</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Deb  Jones</v>
-      </c>
-      <c r="C8">
-        <v>66</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E8" t="str">
-        <v>fullhouse5@optusnet.com.au</v>
-      </c>
-      <c r="F8" t="str">
-        <v>438561474</v>
-      </c>
-      <c r="G8" t="str">
-        <v>Bayswater North</v>
-      </c>
-      <c r="H8" t="str">
-        <v>B+</v>
-      </c>
-      <c r="I8" t="str">
-        <v>available</v>
-      </c>
-      <c r="J8" t="str">
-        <v>Daryl Jones</v>
-      </c>
-      <c r="M8" t="str">
-        <v>No</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>f693566d-ea7c-40d1-89aa-158e842961d0</v>
+        <v>82960b61-d36b-49e2-9ddf-a7b8e0b02a63</v>
       </c>
       <c r="B9" t="str">
-        <v>Brent Barnett</v>
+        <v>Tara Saltzman</v>
       </c>
       <c r="C9">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="D9" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E9" t="str">
-        <v>brentbarnett88@gmail.com</v>
+        <v>tarasaltzman@bigpond.com</v>
       </c>
       <c r="F9" t="str">
-        <v>423530043</v>
+        <v>448545599</v>
       </c>
       <c r="G9" t="str">
-        <v>Preston</v>
+        <v>Melbourne</v>
       </c>
       <c r="H9" t="str">
         <v>B+</v>
       </c>
       <c r="I9" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J9" t="str">
-        <v>Stephanie Squillacioti</v>
+        <v xml:space="preserve">JACK AGIUS - NEEDS TO DO APPLICATION </v>
+      </c>
+      <c r="M9" t="str">
+        <v>NA</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>82960b61-d36b-49e2-9ddf-a7b8e0b02a63</v>
+        <v>f693566d-ea7c-40d1-89aa-158e842961d0</v>
       </c>
       <c r="B10" t="str">
-        <v>Tara Saltzman</v>
+        <v>Brent Barnett</v>
       </c>
       <c r="C10">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="D10" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E10" t="str">
-        <v>tarasaltzman@bigpond.com</v>
+        <v>brentbarnett88@gmail.com</v>
       </c>
       <c r="F10" t="str">
-        <v>448545599</v>
+        <v>423530043</v>
       </c>
       <c r="G10" t="str">
-        <v>Melbourne</v>
+        <v>Preston</v>
       </c>
       <c r="H10" t="str">
         <v>B+</v>
@@ -1013,10 +1016,7 @@
         <v>available</v>
       </c>
       <c r="J10" t="str">
-        <v xml:space="preserve">JACK AGIUS - NEEDS TO DO APPLICATION </v>
-      </c>
-      <c r="M10" t="str">
-        <v>NA</v>
+        <v>Stephanie Squillacioti</v>
       </c>
     </row>
     <row r="11">
@@ -1160,127 +1160,124 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>4f08069b-d828-429c-af5e-b1eee2c123df</v>
+        <v>97e81b41-1b8d-4562-9e12-3747f87663a9</v>
       </c>
       <c r="B15" t="str">
-        <v>Sarah Desira</v>
+        <v>Thomas Mckenna</v>
       </c>
       <c r="C15">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D15" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E15" t="str">
-        <v>unicornwolf11@gmail.com</v>
+        <v>mckenna.6@yahoo.com</v>
       </c>
       <c r="F15" t="str">
-        <v>450765125</v>
+        <v>421758700</v>
       </c>
       <c r="G15" t="str">
-        <v>Lara</v>
+        <v xml:space="preserve">Officer South </v>
       </c>
       <c r="H15" t="str">
         <v>B</v>
       </c>
       <c r="I15" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J15" t="str">
-        <v>Husband Daniel Desira b6042a-1-1936280</v>
-      </c>
-      <c r="M15" t="str">
-        <v xml:space="preserve">No </v>
+        <v>thomas mckenna, Carolyn (Caz) Wilby</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>419afd3f-2406-423d-942f-2dfafe875f96</v>
+        <v>1d96e742-18bb-4fc0-b741-154d1a4d9487</v>
       </c>
       <c r="B16" t="str">
-        <v>Anna Fonua</v>
+        <v>James Butler</v>
       </c>
       <c r="C16">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="D16" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E16" t="str">
-        <v>Annawallace89@hotmail.com</v>
+        <v>butlerjg1509@gmail.com</v>
       </c>
       <c r="F16" t="str">
-        <v>452452442</v>
+        <v>428400584</v>
       </c>
       <c r="G16" t="str">
-        <v>Truganina</v>
+        <v>Mentone</v>
       </c>
       <c r="H16" t="str">
-        <v>A</v>
+        <v>B+</v>
       </c>
       <c r="I16" t="str">
         <v>available</v>
       </c>
       <c r="J16" t="str">
-        <v>Dad Michael Wallace - b6042a-1-1936372</v>
-      </c>
-      <c r="M16" t="str">
-        <v xml:space="preserve">no </v>
+        <v>Issy McReynolds</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>e4a52d0d-9c54-4504-8a0f-85845cd88e27</v>
+        <v>f7b766dc-a0d0-4a91-98ef-47472cdca803</v>
       </c>
       <c r="B17" t="str">
-        <v>David Fenwick</v>
+        <v>Mara Baumgardner</v>
       </c>
       <c r="C17">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D17" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E17" t="str">
-        <v>David.s.fenwick@gmail.com</v>
+        <v>Granic@hotmail.com</v>
       </c>
       <c r="F17" t="str">
-        <v>429811171</v>
+        <v>407364450</v>
       </c>
       <c r="G17" t="str">
-        <v>Teesdale</v>
+        <v>Cockatoo</v>
       </c>
       <c r="H17" t="str">
-        <v>B+</v>
+        <v>B</v>
       </c>
       <c r="I17" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J17" t="str">
-        <v>Solo</v>
+        <v xml:space="preserve">Mum - Mira Granic </v>
+      </c>
+      <c r="M17" t="str">
+        <v xml:space="preserve">No </v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>1d96e742-18bb-4fc0-b741-154d1a4d9487</v>
+        <v>1bc7d8fc-def3-4f9f-8376-80b79696d1a5</v>
       </c>
       <c r="B18" t="str">
-        <v>James Butler</v>
+        <v>Eden Hayes</v>
       </c>
       <c r="C18">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="D18" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E18" t="str">
-        <v>butlerjg1509@gmail.com</v>
+        <v>edenhayes19@gmail.com</v>
       </c>
       <c r="F18" t="str">
-        <v>428400584</v>
+        <v>448096139</v>
       </c>
       <c r="G18" t="str">
-        <v>Mentone</v>
+        <v>Elwood</v>
       </c>
       <c r="H18" t="str">
         <v>B+</v>
@@ -1289,74 +1286,71 @@
         <v>available</v>
       </c>
       <c r="J18" t="str">
-        <v>Issy McReynolds</v>
+        <v>Jackson Harris</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>f7b766dc-a0d0-4a91-98ef-47472cdca803</v>
+        <v>614641dd-4e94-4c42-a1d9-db37c608dcbe</v>
       </c>
       <c r="B19" t="str">
-        <v>Mara Baumgardner</v>
+        <v>Antonio Freno</v>
       </c>
       <c r="C19">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D19" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E19" t="str">
-        <v>Granic@hotmail.com</v>
+        <v>frenoantonio@hotmail.it</v>
       </c>
       <c r="F19" t="str">
-        <v>407364450</v>
+        <v>422177371</v>
       </c>
       <c r="G19" t="str">
-        <v>Cockatoo</v>
+        <v>Glenroy</v>
       </c>
       <c r="H19" t="str">
-        <v>B</v>
+        <v>B+</v>
       </c>
       <c r="I19" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J19" t="str">
-        <v xml:space="preserve">Mum - Mira Granic </v>
-      </c>
-      <c r="M19" t="str">
-        <v xml:space="preserve">No </v>
+        <v>Solo</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>1bc7d8fc-def3-4f9f-8376-80b79696d1a5</v>
+        <v>e4a52d0d-9c54-4504-8a0f-85845cd88e27</v>
       </c>
       <c r="B20" t="str">
-        <v>Eden Hayes</v>
+        <v>David Fenwick</v>
       </c>
       <c r="C20">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="D20" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E20" t="str">
-        <v>edenhayes19@gmail.com</v>
+        <v>David.s.fenwick@gmail.com</v>
       </c>
       <c r="F20" t="str">
-        <v>448096139</v>
+        <v>429811171</v>
       </c>
       <c r="G20" t="str">
-        <v>Elwood</v>
+        <v>Teesdale</v>
       </c>
       <c r="H20" t="str">
         <v>B+</v>
       </c>
       <c r="I20" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J20" t="str">
-        <v>Jackson Harris</v>
+        <v>Solo</v>
       </c>
     </row>
     <row r="21">
@@ -1385,7 +1379,7 @@
         <v>B+</v>
       </c>
       <c r="I21" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J21" t="str">
         <v>SOLO</v>
@@ -1394,365 +1388,371 @@
         <v>NA</v>
       </c>
     </row>
-    <row r="22" xml:space="preserve">
+    <row r="22">
       <c r="A22" t="str">
-        <v>d9b76f1c-0867-44fc-9215-6ef7b1184af6</v>
+        <v>f048c8fe-e8c9-4357-8ec8-ef76793e5bc1</v>
       </c>
       <c r="B22" t="str">
-        <v>Kayla Lorenzini</v>
+        <v>Tamara Mifsud</v>
       </c>
       <c r="C22">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D22" t="str">
         <v>Female</v>
       </c>
       <c r="E22" t="str">
-        <v>kaylalorenzini_@hotmail.com</v>
+        <v>tamara.mifsud@hotmail.com</v>
       </c>
       <c r="F22" t="str">
-        <v>430517653</v>
+        <v>416552122</v>
       </c>
       <c r="G22" t="str">
-        <v>Melbourne</v>
+        <v>Aintree</v>
       </c>
       <c r="H22" t="str">
-        <v>B+</v>
+        <v>B</v>
       </c>
       <c r="I22" t="str">
         <v>available</v>
       </c>
-      <c r="J22" t="str" xml:space="preserve">
+      <c r="J22" t="str">
+        <v>Aliye Abcilar</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>6bbdadcb-23a8-41c9-964b-6152e234cb33</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Philip Natoli</v>
+      </c>
+      <c r="C23">
+        <v>29</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Philip.natoli@outlook.com</v>
+      </c>
+      <c r="F23" t="str">
+        <v>466021882</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Caulfield South</v>
+      </c>
+      <c r="H23" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I23" t="str">
+        <v>available</v>
+      </c>
+      <c r="J23" t="str">
+        <v>Hayley Wright</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>de606917-da6f-4fde-881b-7cbfd45cfe56</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Ricky Steve</v>
+      </c>
+      <c r="C24">
+        <v>31</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E24" t="str">
+        <v>tj-c-a@hotmail.com</v>
+      </c>
+      <c r="F24" t="str">
+        <v>411360449</v>
+      </c>
+      <c r="G24" t="str">
+        <v xml:space="preserve">Wangaratta </v>
+      </c>
+      <c r="H24" t="str">
+        <v>A</v>
+      </c>
+      <c r="I24" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="J24" t="str">
+        <v>Taylah-Jayne Lockery</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>6cada433-8344-4d95-97dc-33c9c173ce7c</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Jeanette Quy</v>
+      </c>
+      <c r="C25">
+        <v>74</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E25" t="str">
+        <v>quyfamily@tpg.com.au</v>
+      </c>
+      <c r="F25" t="str">
+        <v>402902273</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Rowville</v>
+      </c>
+      <c r="H25" t="str">
+        <v>C</v>
+      </c>
+      <c r="I25" t="str">
+        <v>available</v>
+      </c>
+      <c r="M25" t="str">
+        <v xml:space="preserve">nothing of note </v>
+      </c>
+    </row>
+    <row r="26" xml:space="preserve">
+      <c r="A26" t="str">
+        <v>dcd305dd-c710-4a1e-859c-835031154035</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Nicholas Boicos</v>
+      </c>
+      <c r="C26">
+        <v>22</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E26" t="str">
+        <v>nboicos@hotmail.com</v>
+      </c>
+      <c r="F26" t="str">
+        <v>429556400</v>
+      </c>
+      <c r="G26" t="str">
+        <v xml:space="preserve">Altona Meadows </v>
+      </c>
+      <c r="H26" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I26" t="str">
+        <v>available</v>
+      </c>
+      <c r="J26" t="str" xml:space="preserve">
+        <v xml:space="preserve">Nick Boicos 
+Matthew Boicos
+Brothers</v>
+      </c>
+    </row>
+    <row r="27" xml:space="preserve">
+      <c r="A27" t="str">
+        <v>15fb53d0-3916-4c9a-9f73-c28c879dec33</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Mozgda  Alime</v>
+      </c>
+      <c r="C27">
+        <v>39</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E27" t="str">
+        <v>smalimi@hotmail.com</v>
+      </c>
+      <c r="F27" t="str">
+        <v>402010235</v>
+      </c>
+      <c r="G27" t="str">
+        <v xml:space="preserve">Melbourne </v>
+      </c>
+      <c r="H27" t="str">
+        <v>C</v>
+      </c>
+      <c r="I27" t="str">
+        <v>available</v>
+      </c>
+      <c r="J27" t="str" xml:space="preserve">
+        <v xml:space="preserve">Sadaf Almini - I believe this is her cousin 
+Lida Alime - I believe this is her cousin or sister 
+Ahmad Alime - Ahmad is Lina's husband </v>
+      </c>
+      <c r="M27" t="str">
+        <v xml:space="preserve">No </v>
+      </c>
+    </row>
+    <row r="28" xml:space="preserve">
+      <c r="A28" t="str">
+        <v>d9b76f1c-0867-44fc-9215-6ef7b1184af6</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Kayla Lorenzini</v>
+      </c>
+      <c r="C28">
+        <v>29</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E28" t="str">
+        <v>kaylalorenzini_@hotmail.com</v>
+      </c>
+      <c r="F28" t="str">
+        <v>430517653</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Melbourne</v>
+      </c>
+      <c r="H28" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I28" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="J28" t="str" xml:space="preserve">
         <v xml:space="preserve">Kayla Lorenzini
 James Lorenzini
 Deanna Gramola</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>9f63aad3-aae1-4220-825c-8964694ec5d8</v>
-      </c>
-      <c r="B23" t="str">
-        <v>Kerrie Donald</v>
-      </c>
-      <c r="C23">
-        <v>47</v>
-      </c>
-      <c r="D23" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E23" t="str">
-        <v>kerrieldonald@hotmail.com</v>
-      </c>
-      <c r="F23" t="str">
-        <v>61400826565</v>
-      </c>
-      <c r="G23" t="str">
-        <v>Mailor's Flat</v>
-      </c>
-      <c r="H23" t="str">
-        <v>B+</v>
-      </c>
-      <c r="I23" t="str">
-        <v>available</v>
-      </c>
-      <c r="J23" t="str">
-        <v>kerrie donald, alistair donald</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>f048c8fe-e8c9-4357-8ec8-ef76793e5bc1</v>
-      </c>
-      <c r="B24" t="str">
-        <v>Tamara Mifsud</v>
-      </c>
-      <c r="C24">
-        <v>32</v>
-      </c>
-      <c r="D24" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E24" t="str">
-        <v>tamara.mifsud@hotmail.com</v>
-      </c>
-      <c r="F24" t="str">
-        <v>416552122</v>
-      </c>
-      <c r="G24" t="str">
-        <v>Aintree</v>
-      </c>
-      <c r="H24" t="str">
-        <v>B</v>
-      </c>
-      <c r="I24" t="str">
-        <v>available</v>
-      </c>
-      <c r="J24" t="str">
-        <v>Aliye Abcilar</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>6bbdadcb-23a8-41c9-964b-6152e234cb33</v>
-      </c>
-      <c r="B25" t="str">
-        <v>Philip Natoli</v>
-      </c>
-      <c r="C25">
-        <v>29</v>
-      </c>
-      <c r="D25" t="str">
-        <v>Male</v>
-      </c>
-      <c r="E25" t="str">
-        <v>Philip.natoli@outlook.com</v>
-      </c>
-      <c r="F25" t="str">
-        <v>466021882</v>
-      </c>
-      <c r="G25" t="str">
-        <v>Caulfield South</v>
-      </c>
-      <c r="H25" t="str">
-        <v>B+</v>
-      </c>
-      <c r="I25" t="str">
-        <v>available</v>
-      </c>
-      <c r="J25" t="str">
-        <v>Hayley Wright</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>6cada433-8344-4d95-97dc-33c9c173ce7c</v>
-      </c>
-      <c r="B26" t="str">
-        <v>Jeanette Quy</v>
-      </c>
-      <c r="C26">
-        <v>74</v>
-      </c>
-      <c r="D26" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E26" t="str">
-        <v>quyfamily@tpg.com.au</v>
-      </c>
-      <c r="F26" t="str">
-        <v>402902273</v>
-      </c>
-      <c r="G26" t="str">
-        <v>Rowville</v>
-      </c>
-      <c r="H26" t="str">
-        <v>C</v>
-      </c>
-      <c r="I26" t="str">
-        <v>available</v>
-      </c>
-      <c r="M26" t="str">
-        <v xml:space="preserve">nothing of note </v>
-      </c>
-    </row>
-    <row r="27" xml:space="preserve">
-      <c r="A27" t="str">
-        <v>dcd305dd-c710-4a1e-859c-835031154035</v>
-      </c>
-      <c r="B27" t="str">
-        <v>Nicholas Boicos</v>
-      </c>
-      <c r="C27">
+    <row r="29">
+      <c r="A29" t="str">
+        <v>607e3750-92e2-4480-b39d-1cb0e026cd4b</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Natasha Devers</v>
+      </c>
+      <c r="C29">
         <v>22</v>
-      </c>
-      <c r="D27" t="str">
-        <v>Male</v>
-      </c>
-      <c r="E27" t="str">
-        <v>nboicos@hotmail.com</v>
-      </c>
-      <c r="F27" t="str">
-        <v>429556400</v>
-      </c>
-      <c r="G27" t="str">
-        <v xml:space="preserve">Altona Meadows </v>
-      </c>
-      <c r="H27" t="str">
-        <v>B+</v>
-      </c>
-      <c r="I27" t="str">
-        <v>available</v>
-      </c>
-      <c r="J27" t="str" xml:space="preserve">
-        <v xml:space="preserve">Nick Boicos 
-Matthew Boicos
-Brothers</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>de606917-da6f-4fde-881b-7cbfd45cfe56</v>
-      </c>
-      <c r="B28" t="str">
-        <v>Ricky Steve</v>
-      </c>
-      <c r="C28">
-        <v>31</v>
-      </c>
-      <c r="D28" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E28" t="str">
-        <v>tj-c-a@hotmail.com</v>
-      </c>
-      <c r="F28" t="str">
-        <v>411360449</v>
-      </c>
-      <c r="G28" t="str">
-        <v xml:space="preserve">Wangaratta </v>
-      </c>
-      <c r="H28" t="str">
-        <v>A</v>
-      </c>
-      <c r="I28" t="str">
-        <v>available</v>
-      </c>
-      <c r="J28" t="str">
-        <v>Taylah-Jayne Lockery</v>
-      </c>
-    </row>
-    <row r="29" xml:space="preserve">
-      <c r="A29" t="str">
-        <v>15fb53d0-3916-4c9a-9f73-c28c879dec33</v>
-      </c>
-      <c r="B29" t="str">
-        <v>Mozgda  Alime</v>
-      </c>
-      <c r="C29">
-        <v>39</v>
       </c>
       <c r="D29" t="str">
         <v>Female</v>
       </c>
       <c r="E29" t="str">
-        <v>smalimi@hotmail.com</v>
+        <v>natashadevers@gmail.com</v>
       </c>
       <c r="F29" t="str">
-        <v>402010235</v>
+        <v>484003770</v>
       </c>
       <c r="G29" t="str">
-        <v xml:space="preserve">Melbourne </v>
+        <v xml:space="preserve">Waterways </v>
       </c>
       <c r="H29" t="str">
-        <v>C</v>
+        <v>B</v>
       </c>
       <c r="I29" t="str">
         <v>available</v>
       </c>
-      <c r="J29" t="str" xml:space="preserve">
-        <v xml:space="preserve">Sadaf Almini - I believe this is her cousin 
-Lida Alime - I believe this is her cousin or sister 
-Ahmad Alime - Ahmad is Lina's husband </v>
-      </c>
-      <c r="M29" t="str">
-        <v xml:space="preserve">No </v>
+      <c r="J29" t="str">
+        <v>Oliver Moran</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>97e81b41-1b8d-4562-9e12-3747f87663a9</v>
+        <v>4f08069b-d828-429c-af5e-b1eee2c123df</v>
       </c>
       <c r="B30" t="str">
-        <v>Thomas Mckenna</v>
+        <v>Sarah Desira</v>
       </c>
       <c r="C30">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D30" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E30" t="str">
-        <v>mckenna.6@yahoo.com</v>
+        <v>unicornwolf11@gmail.com</v>
       </c>
       <c r="F30" t="str">
-        <v>421758700</v>
+        <v>450765125</v>
       </c>
       <c r="G30" t="str">
-        <v xml:space="preserve">Officer South </v>
+        <v>Lara</v>
       </c>
       <c r="H30" t="str">
         <v>B</v>
       </c>
       <c r="I30" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J30" t="str">
-        <v>thomas mckenna, Carolyn (Caz) Wilby</v>
+        <v>Husband Daniel Desira b6042a-1-1936280</v>
+      </c>
+      <c r="M30" t="str">
+        <v xml:space="preserve">No </v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>607e3750-92e2-4480-b39d-1cb0e026cd4b</v>
+        <v>419afd3f-2406-423d-942f-2dfafe875f96</v>
       </c>
       <c r="B31" t="str">
-        <v>Natasha Devers</v>
+        <v>Anna Fonua</v>
       </c>
       <c r="C31">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="D31" t="str">
         <v>Female</v>
       </c>
       <c r="E31" t="str">
-        <v>natashadevers@gmail.com</v>
+        <v>Annawallace89@hotmail.com</v>
       </c>
       <c r="F31" t="str">
-        <v>484003770</v>
+        <v>452452442</v>
       </c>
       <c r="G31" t="str">
-        <v xml:space="preserve">Waterways </v>
+        <v>Truganina</v>
       </c>
       <c r="H31" t="str">
-        <v>B</v>
+        <v>A</v>
       </c>
       <c r="I31" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J31" t="str">
-        <v>Oliver Moran</v>
+        <v>Dad Michael Wallace - b6042a-1-1936372</v>
+      </c>
+      <c r="M31" t="str">
+        <v xml:space="preserve">no </v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>614641dd-4e94-4c42-a1d9-db37c608dcbe</v>
+        <v>9f63aad3-aae1-4220-825c-8964694ec5d8</v>
       </c>
       <c r="B32" t="str">
-        <v>Antonio Freno</v>
+        <v>Kerrie Donald</v>
       </c>
       <c r="C32">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="D32" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E32" t="str">
-        <v>frenoantonio@hotmail.it</v>
+        <v>kerrieldonald@hotmail.com</v>
       </c>
       <c r="F32" t="str">
-        <v>422177371</v>
+        <v>61400826565</v>
       </c>
       <c r="G32" t="str">
-        <v>Glenroy</v>
+        <v>Mailor's Flat</v>
       </c>
       <c r="H32" t="str">
         <v>B+</v>
       </c>
       <c r="I32" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J32" t="str">
-        <v>Solo</v>
+        <v>kerrie donald, alistair donald</v>
       </c>
     </row>
     <row r="33">
@@ -1789,10 +1789,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>45c7f69f-dd89-41d8-b7f0-a83f77fa9d12</v>
+        <v>2aadb3db-ad8e-4edd-a81d-f045a926ceb9</v>
       </c>
       <c r="B34" t="str">
-        <v>Sherif Haggag</v>
+        <v>Alexander Leonard</v>
       </c>
       <c r="C34">
         <v>38</v>
@@ -1801,45 +1801,45 @@
         <v>Male</v>
       </c>
       <c r="E34" t="str">
-        <v>Shaggag87@gmail.com</v>
+        <v>alexleonardedit@gmail.com</v>
       </c>
       <c r="F34" t="str">
-        <v>426233449</v>
+        <v>421834476</v>
       </c>
       <c r="G34" t="str">
-        <v>Belmont</v>
+        <v>Croydon</v>
       </c>
       <c r="H34" t="str">
-        <v>B+</v>
+        <v>A+</v>
       </c>
       <c r="I34" t="str">
         <v>available</v>
       </c>
       <c r="J34" t="str">
-        <v>Solo</v>
-      </c>
-    </row>
-    <row r="35">
+        <v>melissa francis, Alexander Leonard</v>
+      </c>
+    </row>
+    <row r="35" xml:space="preserve">
       <c r="A35" t="str">
-        <v>2aadb3db-ad8e-4edd-a81d-f045a926ceb9</v>
+        <v>1211456d-ea92-4a7b-9d94-885982cf345c</v>
       </c>
       <c r="B35" t="str">
-        <v>Alexander Leonard</v>
+        <v>Bronwyn Parsons</v>
       </c>
       <c r="C35">
-        <v>38</v>
+        <v>72</v>
       </c>
       <c r="D35" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E35" t="str">
-        <v>alexleonardedit@gmail.com</v>
+        <v>Babybear61153@gmail.com</v>
       </c>
       <c r="F35" t="str">
-        <v>421834476</v>
+        <v>432543647</v>
       </c>
       <c r="G35" t="str">
-        <v>Croydon</v>
+        <v>Rosebud</v>
       </c>
       <c r="H35" t="str">
         <v>A+</v>
@@ -1847,180 +1847,180 @@
       <c r="I35" t="str">
         <v>available</v>
       </c>
-      <c r="J35" t="str">
-        <v>melissa francis, Alexander Leonard</v>
-      </c>
-    </row>
-    <row r="36">
+      <c r="J35" t="str" xml:space="preserve">
+        <v xml:space="preserve">Yolette Huon - yol-et Hue on
+Bronwyn Parsons - Would like to be called Bron Emmerson - maiden name</v>
+      </c>
+    </row>
+    <row r="36" xml:space="preserve">
       <c r="A36" t="str">
-        <v>646d2ff7-803b-4c80-bdd6-09d44eec6929</v>
+        <v>23f118f9-20db-422c-8cef-939dc73dd803</v>
       </c>
       <c r="B36" t="str">
-        <v>Leanne Bryant</v>
+        <v>Paige Greig</v>
       </c>
       <c r="C36">
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="D36" t="str">
         <v>Female</v>
       </c>
       <c r="E36" t="str">
-        <v>blazeandcougar@gmail.com</v>
+        <v>paigegreig@hotmail.com</v>
       </c>
       <c r="F36" t="str">
-        <v>61415438228</v>
+        <v>406598552</v>
       </c>
       <c r="G36" t="str">
-        <v xml:space="preserve">Hampton Park </v>
+        <v>Mooroolbark</v>
       </c>
       <c r="H36" t="str">
-        <v>B</v>
+        <v>C</v>
       </c>
       <c r="I36" t="str">
         <v>available</v>
       </c>
-      <c r="J36" t="str">
-        <v>Solo</v>
-      </c>
-    </row>
-    <row r="37" xml:space="preserve">
+      <c r="J36" t="str" xml:space="preserve">
+        <v xml:space="preserve">Erin
+Morgan (sister) - need to do application</v>
+      </c>
+    </row>
+    <row r="37">
       <c r="A37" t="str">
-        <v>1211456d-ea92-4a7b-9d94-885982cf345c</v>
+        <v>cbfeb8b0-bd5d-4614-a055-cbac047cf152</v>
       </c>
       <c r="B37" t="str">
-        <v>Bronwyn Parsons</v>
+        <v>Tamika Colville</v>
       </c>
       <c r="C37">
-        <v>72</v>
+        <v>31</v>
       </c>
       <c r="D37" t="str">
         <v>Female</v>
       </c>
       <c r="E37" t="str">
-        <v>Babybear61153@gmail.com</v>
+        <v>tamika.colville@gmail.com</v>
       </c>
       <c r="F37" t="str">
-        <v>432543647</v>
+        <v>409132141</v>
       </c>
       <c r="G37" t="str">
-        <v>Rosebud</v>
+        <v>Golden square</v>
       </c>
       <c r="H37" t="str">
-        <v>A+</v>
+        <v>B+</v>
       </c>
       <c r="I37" t="str">
-        <v>available</v>
-      </c>
-      <c r="J37" t="str" xml:space="preserve">
-        <v xml:space="preserve">Yolette Huon - yol-et Hue on
-Bronwyn Parsons - Would like to be called Bron Emmerson - maiden name</v>
-      </c>
-    </row>
-    <row r="38">
+        <v>assigned</v>
+      </c>
+      <c r="J37" t="str">
+        <v>Shinae Colville</v>
+      </c>
+      <c r="L37" t="str">
+        <v>Diagnosed with MS in 2018</v>
+      </c>
+      <c r="M37" t="str">
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="38" xml:space="preserve">
       <c r="A38" t="str">
-        <v>cbfeb8b0-bd5d-4614-a055-cbac047cf152</v>
+        <v>ed91813b-2f74-4638-9d1a-ef8c54cff447</v>
       </c>
       <c r="B38" t="str">
-        <v>Tamika Colville</v>
+        <v>Linda Browne</v>
       </c>
       <c r="C38">
-        <v>31</v>
+        <v>54</v>
       </c>
       <c r="D38" t="str">
         <v>Female</v>
       </c>
       <c r="E38" t="str">
-        <v>tamika.colville@gmail.com</v>
+        <v>Lindabrowne@iprimus.com.au</v>
       </c>
       <c r="F38" t="str">
-        <v>409132141</v>
+        <v>429570177</v>
       </c>
       <c r="G38" t="str">
-        <v>Golden square</v>
+        <v>OFFICER</v>
       </c>
       <c r="H38" t="str">
-        <v>B+</v>
+        <v>B</v>
       </c>
       <c r="I38" t="str">
-        <v>available</v>
-      </c>
-      <c r="J38" t="str">
-        <v>Shinae Colville</v>
-      </c>
-      <c r="L38" t="str">
-        <v>Diagnosed with MS in 2018</v>
-      </c>
-      <c r="M38" t="str">
-        <v>NA</v>
-      </c>
-    </row>
-    <row r="39" xml:space="preserve">
-      <c r="A39" t="str">
-        <v>23f118f9-20db-422c-8cef-939dc73dd803</v>
-      </c>
-      <c r="B39" t="str">
-        <v>Paige Greig</v>
-      </c>
-      <c r="C39">
-        <v>31</v>
-      </c>
-      <c r="D39" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E39" t="str">
-        <v>paigegreig@hotmail.com</v>
-      </c>
-      <c r="F39" t="str">
-        <v>406598552</v>
-      </c>
-      <c r="G39" t="str">
-        <v>Mooroolbark</v>
-      </c>
-      <c r="H39" t="str">
-        <v>C</v>
-      </c>
-      <c r="I39" t="str">
-        <v>available</v>
-      </c>
-      <c r="J39" t="str" xml:space="preserve">
-        <v xml:space="preserve">Erin
-Morgan (sister) - need to do application</v>
-      </c>
-    </row>
-    <row r="40" xml:space="preserve">
-      <c r="A40" t="str">
-        <v>ed91813b-2f74-4638-9d1a-ef8c54cff447</v>
-      </c>
-      <c r="B40" t="str">
-        <v>Linda Browne</v>
-      </c>
-      <c r="C40">
-        <v>54</v>
-      </c>
-      <c r="D40" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E40" t="str">
-        <v>Lindabrowne@iprimus.com.au</v>
-      </c>
-      <c r="F40" t="str">
-        <v>429570177</v>
-      </c>
-      <c r="G40" t="str">
-        <v>OFFICER</v>
-      </c>
-      <c r="H40" t="str">
-        <v>B</v>
-      </c>
-      <c r="I40" t="str">
-        <v>available</v>
-      </c>
-      <c r="J40" t="str" xml:space="preserve">
+        <v>assigned</v>
+      </c>
+      <c r="J38" t="str" xml:space="preserve">
         <v xml:space="preserve">Natalie Browne
 Linda Browne
 Aidan Miler</v>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>45c7f69f-dd89-41d8-b7f0-a83f77fa9d12</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Sherif Haggag</v>
+      </c>
+      <c r="C39">
+        <v>38</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Shaggag87@gmail.com</v>
+      </c>
+      <c r="F39" t="str">
+        <v>426233449</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Belmont</v>
+      </c>
+      <c r="H39" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I39" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="J39" t="str">
+        <v>Solo</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>646d2ff7-803b-4c80-bdd6-09d44eec6929</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Leanne Bryant</v>
+      </c>
+      <c r="C40">
+        <v>63</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E40" t="str">
+        <v>blazeandcougar@gmail.com</v>
+      </c>
+      <c r="F40" t="str">
+        <v>61415438228</v>
+      </c>
+      <c r="G40" t="str">
+        <v xml:space="preserve">Hampton Park </v>
+      </c>
+      <c r="H40" t="str">
+        <v>B</v>
+      </c>
+      <c r="I40" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="J40" t="str">
+        <v>Solo</v>
+      </c>
+    </row>
     <row r="41">
       <c r="A41" t="str">
         <v>441f345e-57a2-403b-a9a9-8284261eba7b</v>
@@ -2079,7 +2079,7 @@
         <v>B+</v>
       </c>
       <c r="I42" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J42" t="str">
         <v>Solo</v>
@@ -2144,7 +2144,7 @@
         <v>B</v>
       </c>
       <c r="I44" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J44" t="str">
         <v>SOLO</v>
@@ -2179,7 +2179,7 @@
         <v>B</v>
       </c>
       <c r="I45" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J45" t="str" xml:space="preserve">
         <v xml:space="preserve">Meenakshi Mehra
@@ -2390,7 +2390,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H24"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2452,9 +2452,366 @@
         <v>A2</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>69e786fd-e21d-4e14-88da-7125c5f4a1d2</v>
+      </c>
+      <c r="B4" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C4" t="str">
+        <v>7fc083f6-6be3-42bf-b4e5-fc6412e1c559</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" t="str">
+        <v>A3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>eb8bfbdd-63a6-4079-aba9-5800fb7a540b</v>
+      </c>
+      <c r="B5" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C5" t="str">
+        <v>34b3d848-f096-4bc9-bd55-dc4dd85ad1b3</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" t="str">
+        <v>B1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>a3858d3d-55d1-4fdb-97d8-320bba44e137</v>
+      </c>
+      <c r="B6" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C6" t="str">
+        <v>e4a52d0d-9c54-4504-8a0f-85845cd88e27</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" t="str">
+        <v>B2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>b52bba5a-5df3-4857-bd40-94b252176098</v>
+      </c>
+      <c r="B7" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C7" t="str">
+        <v>96c75db9-b001-4abe-8ddb-d5a73cb04529</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7" t="str">
+        <v>B3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>4f0e1cd0-0b97-41cf-8546-066d8aacaa18</v>
+      </c>
+      <c r="B8" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C8" t="str">
+        <v>d9b76f1c-0867-44fc-9215-6ef7b1184af6</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8" t="str">
+        <v>B4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>e1a80551-d2da-4874-91db-588715a4fac4</v>
+      </c>
+      <c r="B9" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C9" t="str">
+        <v>9f63aad3-aae1-4220-825c-8964694ec5d8</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9" t="str">
+        <v>B5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>abc48d6d-e2be-45f3-b39d-aab68fd3a887</v>
+      </c>
+      <c r="B10" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C10" t="str">
+        <v>97e81b41-1b8d-4562-9e12-3747f87663a9</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10" t="str">
+        <v>C1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>1996d94e-e4b6-41eb-9c86-6f2ce57c0d3e</v>
+      </c>
+      <c r="B11" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C11" t="str">
+        <v>614641dd-4e94-4c42-a1d9-db37c608dcbe</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11" t="str">
+        <v>C2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>15371ee3-0b7e-4086-84f6-3720ca1ff543</v>
+      </c>
+      <c r="B12" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C12" t="str">
+        <v>45c7f69f-dd89-41d8-b7f0-a83f77fa9d12</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12" t="str">
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>9c31ffbb-2789-43bb-a60e-90c4b8100cef</v>
+      </c>
+      <c r="B13" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C13" t="str">
+        <v>646d2ff7-803b-4c80-bdd6-09d44eec6929</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13" t="str">
+        <v>C4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>bc578b4a-ddea-41c3-9540-e88f6659f18c</v>
+      </c>
+      <c r="B14" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C14" t="str">
+        <v>cbfeb8b0-bd5d-4614-a055-cbac047cf152</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14" t="str">
+        <v>D1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>72473e20-842c-4521-a6c8-ba7c2d625b26</v>
+      </c>
+      <c r="B15" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C15" t="str">
+        <v>ed91813b-2f74-4638-9d1a-ef8c54cff447</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15" t="str">
+        <v>D2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>cdfce1b8-2ada-4f40-a965-ec4421f32195</v>
+      </c>
+      <c r="B16" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C16" t="str">
+        <v>c60666dd-e08c-4aa0-8582-4e7a3ad280f8</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16" t="str">
+        <v>D3</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>0bafba7c-79a0-4bae-b175-028f5c764b20</v>
+      </c>
+      <c r="B17" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C17" t="str">
+        <v>917bd31e-7781-44cc-936c-980cb1f844aa</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17" t="str">
+        <v>D4</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>94521f77-45d2-4af9-952a-a692cd7c7aa8</v>
+      </c>
+      <c r="B18" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C18" t="str">
+        <v>54de1dd9-b7eb-489d-b4a1-8b3744a385c4</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18" t="str">
+        <v>E1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>38e2c0fc-5873-43aa-9394-f7c2709f8a83</v>
+      </c>
+      <c r="B19" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C19" t="str">
+        <v>1fe25fd6-dc69-4d29-b22f-9a15ad3d457f</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19" t="str">
+        <v>E2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>c21a4154-3157-46c8-a878-b599e0689d93</v>
+      </c>
+      <c r="B20" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C20" t="str">
+        <v>82960b61-d36b-49e2-9ddf-a7b8e0b02a63</v>
+      </c>
+      <c r="D20">
+        <v>2</v>
+      </c>
+      <c r="E20" t="str">
+        <v>A1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>ffc84c94-f1d0-4b10-aa29-30dc6ffbda57</v>
+      </c>
+      <c r="B21" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C21" t="str">
+        <v>4f08069b-d828-429c-af5e-b1eee2c123df</v>
+      </c>
+      <c r="D21">
+        <v>2</v>
+      </c>
+      <c r="E21" t="str">
+        <v>A2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>b27d2d06-2e2c-4115-9995-db7dd2a60c77</v>
+      </c>
+      <c r="B22" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C22" t="str">
+        <v>419afd3f-2406-423d-942f-2dfafe875f96</v>
+      </c>
+      <c r="D22">
+        <v>2</v>
+      </c>
+      <c r="E22" t="str">
+        <v>A3</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>7a2cb7e6-2374-470d-916d-9e0890d7fde8</v>
+      </c>
+      <c r="B23" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C23" t="str">
+        <v>f7b766dc-a0d0-4a91-98ef-47472cdca803</v>
+      </c>
+      <c r="D23">
+        <v>2</v>
+      </c>
+      <c r="E23" t="str">
+        <v>A4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>36893ad6-bfef-4de4-b6f2-a5c5f1b825b0</v>
+      </c>
+      <c r="B24" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C24" t="str">
+        <v>de606917-da6f-4fde-881b-7cbfd45cfe56</v>
+      </c>
+      <c r="D24">
+        <v>2</v>
+      </c>
+      <c r="E24" t="str">
+        <v>A5</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H24"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Make the contestant assignment dialog significantly larger
Increase the dialog width for contestant assignment to max-w-6xl and update backup data including exported timestamp and availability status for several contestants.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: f123b9d7-6af8-472a-a75c-70d0b78d0583
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 0ba77241-0784-41a1-895c-564f07c26d2f
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/4ca2a1f8-42ce-4303-beff-eb92e3283d4c/f123b9d7-6af8-472a-a75c-70d0b78d0583/SA70FQN
</commit_message>
<xml_diff>
--- a/storage/backups/automatic-backup.xlsx
+++ b/storage/backups/automatic-backup.xlsx
@@ -736,7 +736,7 @@
         <v>B</v>
       </c>
       <c r="I2" t="str">
-        <v>assigned</v>
+        <v>available</v>
       </c>
       <c r="J2" t="str" xml:space="preserve">
         <v xml:space="preserve">Meenakshi Mehra
@@ -769,7 +769,7 @@
         <v>B</v>
       </c>
       <c r="I3" t="str">
-        <v>assigned</v>
+        <v>available</v>
       </c>
       <c r="J3" t="str">
         <v>Donna Collins, Tom Collins</v>
@@ -941,7 +941,7 @@
         <v>A</v>
       </c>
       <c r="I8" t="str">
-        <v>assigned</v>
+        <v>available</v>
       </c>
       <c r="J8" t="str" xml:space="preserve">
         <v xml:space="preserve">
@@ -978,7 +978,7 @@
         <v>B+</v>
       </c>
       <c r="I9" t="str">
-        <v>assigned</v>
+        <v>available</v>
       </c>
       <c r="J9" t="str">
         <v xml:space="preserve">JACK AGIUS - NEEDS TO DO APPLICATION </v>
@@ -1021,75 +1021,75 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>b1fc34e8-20cb-4607-9568-0761cf4520a6</v>
+        <v>6b9ae7f0-4a81-4dda-8e55-e49415d98ec6</v>
       </c>
       <c r="B11" t="str">
-        <v>Troy Smith</v>
+        <v>Tayla Huxtable</v>
       </c>
       <c r="C11">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D11" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E11" t="str">
-        <v>Troyssmith94@gmail.com</v>
+        <v>Taylahuxtable@gmail.com</v>
       </c>
       <c r="F11" t="str">
-        <v>429354308</v>
+        <v>435320280</v>
       </c>
       <c r="G11" t="str">
-        <v>Melbourne</v>
-      </c>
-      <c r="H11" t="str">
-        <v>B+</v>
+        <v>FERNTREE GULLY</v>
       </c>
       <c r="I11" t="str">
         <v>assigned</v>
       </c>
       <c r="J11" t="str">
-        <v>Tayla Huxtable</v>
+        <v>Troy Smith</v>
       </c>
       <c r="K11" t="str">
         <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
       </c>
-      <c r="L11" t="str">
-        <v xml:space="preserve">Peanut allergy </v>
-      </c>
-      <c r="M11" t="str">
-        <v>NA</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>6b9ae7f0-4a81-4dda-8e55-e49415d98ec6</v>
+        <v>b1fc34e8-20cb-4607-9568-0761cf4520a6</v>
       </c>
       <c r="B12" t="str">
-        <v>Tayla Huxtable</v>
+        <v>Troy Smith</v>
       </c>
       <c r="C12">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D12" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E12" t="str">
-        <v>Taylahuxtable@gmail.com</v>
+        <v>Troyssmith94@gmail.com</v>
       </c>
       <c r="F12" t="str">
-        <v>435320280</v>
+        <v>429354308</v>
       </c>
       <c r="G12" t="str">
-        <v>FERNTREE GULLY</v>
+        <v>Melbourne</v>
+      </c>
+      <c r="H12" t="str">
+        <v>B+</v>
       </c>
       <c r="I12" t="str">
         <v>assigned</v>
       </c>
       <c r="J12" t="str">
-        <v>Troy Smith</v>
+        <v>Tayla Huxtable</v>
       </c>
       <c r="K12" t="str">
         <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
+      </c>
+      <c r="L12" t="str">
+        <v xml:space="preserve">Peanut allergy </v>
+      </c>
+      <c r="M12" t="str">
+        <v>NA</v>
       </c>
     </row>
     <row r="13">
@@ -1160,98 +1160,98 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>97e81b41-1b8d-4562-9e12-3747f87663a9</v>
+        <v>9f63aad3-aae1-4220-825c-8964694ec5d8</v>
       </c>
       <c r="B15" t="str">
-        <v>Thomas Mckenna</v>
+        <v>Kerrie Donald</v>
       </c>
       <c r="C15">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="D15" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E15" t="str">
-        <v>mckenna.6@yahoo.com</v>
+        <v>kerrieldonald@hotmail.com</v>
       </c>
       <c r="F15" t="str">
-        <v>421758700</v>
+        <v>61400826565</v>
       </c>
       <c r="G15" t="str">
-        <v xml:space="preserve">Officer South </v>
+        <v>Mailor's Flat</v>
       </c>
       <c r="H15" t="str">
-        <v>B</v>
+        <v>B+</v>
       </c>
       <c r="I15" t="str">
-        <v>assigned</v>
+        <v>available</v>
       </c>
       <c r="J15" t="str">
-        <v>thomas mckenna, Carolyn (Caz) Wilby</v>
+        <v>kerrie donald, alistair donald</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>1d96e742-18bb-4fc0-b741-154d1a4d9487</v>
+        <v>97e81b41-1b8d-4562-9e12-3747f87663a9</v>
       </c>
       <c r="B16" t="str">
-        <v>James Butler</v>
+        <v>Thomas Mckenna</v>
       </c>
       <c r="C16">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="D16" t="str">
         <v>Male</v>
       </c>
       <c r="E16" t="str">
-        <v>butlerjg1509@gmail.com</v>
+        <v>mckenna.6@yahoo.com</v>
       </c>
       <c r="F16" t="str">
-        <v>428400584</v>
+        <v>421758700</v>
       </c>
       <c r="G16" t="str">
-        <v>Mentone</v>
+        <v xml:space="preserve">Officer South </v>
       </c>
       <c r="H16" t="str">
-        <v>B+</v>
+        <v>B</v>
       </c>
       <c r="I16" t="str">
         <v>available</v>
       </c>
       <c r="J16" t="str">
-        <v>Issy McReynolds</v>
+        <v>thomas mckenna, Carolyn (Caz) Wilby</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>f7b766dc-a0d0-4a91-98ef-47472cdca803</v>
+        <v>4f08069b-d828-429c-af5e-b1eee2c123df</v>
       </c>
       <c r="B17" t="str">
-        <v>Mara Baumgardner</v>
+        <v>Sarah Desira</v>
       </c>
       <c r="C17">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D17" t="str">
         <v>Female</v>
       </c>
       <c r="E17" t="str">
-        <v>Granic@hotmail.com</v>
+        <v>unicornwolf11@gmail.com</v>
       </c>
       <c r="F17" t="str">
-        <v>407364450</v>
+        <v>450765125</v>
       </c>
       <c r="G17" t="str">
-        <v>Cockatoo</v>
+        <v>Lara</v>
       </c>
       <c r="H17" t="str">
         <v>B</v>
       </c>
       <c r="I17" t="str">
-        <v>assigned</v>
+        <v>available</v>
       </c>
       <c r="J17" t="str">
-        <v xml:space="preserve">Mum - Mira Granic </v>
+        <v>Husband Daniel Desira b6042a-1-1936280</v>
       </c>
       <c r="M17" t="str">
         <v xml:space="preserve">No </v>
@@ -1259,25 +1259,25 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>1bc7d8fc-def3-4f9f-8376-80b79696d1a5</v>
+        <v>1d96e742-18bb-4fc0-b741-154d1a4d9487</v>
       </c>
       <c r="B18" t="str">
-        <v>Eden Hayes</v>
+        <v>James Butler</v>
       </c>
       <c r="C18">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="D18" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E18" t="str">
-        <v>edenhayes19@gmail.com</v>
+        <v>butlerjg1509@gmail.com</v>
       </c>
       <c r="F18" t="str">
-        <v>448096139</v>
+        <v>428400584</v>
       </c>
       <c r="G18" t="str">
-        <v>Elwood</v>
+        <v>Mentone</v>
       </c>
       <c r="H18" t="str">
         <v>B+</v>
@@ -1286,30 +1286,30 @@
         <v>available</v>
       </c>
       <c r="J18" t="str">
-        <v>Jackson Harris</v>
+        <v>Issy McReynolds</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>614641dd-4e94-4c42-a1d9-db37c608dcbe</v>
+        <v>e4a52d0d-9c54-4504-8a0f-85845cd88e27</v>
       </c>
       <c r="B19" t="str">
-        <v>Antonio Freno</v>
+        <v>David Fenwick</v>
       </c>
       <c r="C19">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D19" t="str">
         <v>Male</v>
       </c>
       <c r="E19" t="str">
-        <v>frenoantonio@hotmail.it</v>
+        <v>David.s.fenwick@gmail.com</v>
       </c>
       <c r="F19" t="str">
-        <v>422177371</v>
+        <v>429811171</v>
       </c>
       <c r="G19" t="str">
-        <v>Glenroy</v>
+        <v>Teesdale</v>
       </c>
       <c r="H19" t="str">
         <v>B+</v>
@@ -1323,325 +1323,328 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>e4a52d0d-9c54-4504-8a0f-85845cd88e27</v>
+        <v>1bc7d8fc-def3-4f9f-8376-80b79696d1a5</v>
       </c>
       <c r="B20" t="str">
-        <v>David Fenwick</v>
+        <v>Eden Hayes</v>
       </c>
       <c r="C20">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="D20" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E20" t="str">
-        <v>David.s.fenwick@gmail.com</v>
+        <v>edenhayes19@gmail.com</v>
       </c>
       <c r="F20" t="str">
-        <v>429811171</v>
+        <v>448096139</v>
       </c>
       <c r="G20" t="str">
-        <v>Teesdale</v>
+        <v>Elwood</v>
       </c>
       <c r="H20" t="str">
         <v>B+</v>
       </c>
       <c r="I20" t="str">
-        <v>assigned</v>
+        <v>available</v>
       </c>
       <c r="J20" t="str">
-        <v>Solo</v>
+        <v>Jackson Harris</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>96c75db9-b001-4abe-8ddb-d5a73cb04529</v>
+        <v>419afd3f-2406-423d-942f-2dfafe875f96</v>
       </c>
       <c r="B21" t="str">
-        <v>Kiran Rao</v>
+        <v>Anna Fonua</v>
       </c>
       <c r="C21">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D21" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E21" t="str">
-        <v>kiran.rao07@gmail.com</v>
+        <v>Annawallace89@hotmail.com</v>
       </c>
       <c r="F21" t="str">
-        <v>420486042</v>
+        <v>452452442</v>
       </c>
       <c r="G21" t="str">
-        <v>Southbank</v>
+        <v>Truganina</v>
       </c>
       <c r="H21" t="str">
+        <v>A</v>
+      </c>
+      <c r="I21" t="str">
+        <v>available</v>
+      </c>
+      <c r="J21" t="str">
+        <v>Dad Michael Wallace - b6042a-1-1936372</v>
+      </c>
+      <c r="M21" t="str">
+        <v xml:space="preserve">no </v>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
+      <c r="A22" t="str">
+        <v>d9b76f1c-0867-44fc-9215-6ef7b1184af6</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Kayla Lorenzini</v>
+      </c>
+      <c r="C22">
+        <v>29</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E22" t="str">
+        <v>kaylalorenzini_@hotmail.com</v>
+      </c>
+      <c r="F22" t="str">
+        <v>430517653</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Melbourne</v>
+      </c>
+      <c r="H22" t="str">
         <v>B+</v>
       </c>
-      <c r="I21" t="str">
-        <v>assigned</v>
-      </c>
-      <c r="J21" t="str">
-        <v>SOLO</v>
-      </c>
-      <c r="M21" t="str">
-        <v>NA</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>f048c8fe-e8c9-4357-8ec8-ef76793e5bc1</v>
-      </c>
-      <c r="B22" t="str">
-        <v>Tamara Mifsud</v>
-      </c>
-      <c r="C22">
-        <v>32</v>
-      </c>
-      <c r="D22" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E22" t="str">
-        <v>tamara.mifsud@hotmail.com</v>
-      </c>
-      <c r="F22" t="str">
-        <v>416552122</v>
-      </c>
-      <c r="G22" t="str">
-        <v>Aintree</v>
-      </c>
-      <c r="H22" t="str">
-        <v>B</v>
-      </c>
       <c r="I22" t="str">
         <v>available</v>
       </c>
-      <c r="J22" t="str">
-        <v>Aliye Abcilar</v>
+      <c r="J22" t="str" xml:space="preserve">
+        <v xml:space="preserve">Kayla Lorenzini
+James Lorenzini
+Deanna Gramola</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>6bbdadcb-23a8-41c9-964b-6152e234cb33</v>
+        <v>96c75db9-b001-4abe-8ddb-d5a73cb04529</v>
       </c>
       <c r="B23" t="str">
-        <v>Philip Natoli</v>
+        <v>Kiran Rao</v>
       </c>
       <c r="C23">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="D23" t="str">
         <v>Male</v>
       </c>
       <c r="E23" t="str">
-        <v>Philip.natoli@outlook.com</v>
+        <v>kiran.rao07@gmail.com</v>
       </c>
       <c r="F23" t="str">
-        <v>466021882</v>
+        <v>420486042</v>
       </c>
       <c r="G23" t="str">
-        <v>Caulfield South</v>
+        <v>Southbank</v>
       </c>
       <c r="H23" t="str">
         <v>B+</v>
       </c>
       <c r="I23" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J23" t="str">
-        <v>Hayley Wright</v>
+        <v>SOLO</v>
+      </c>
+      <c r="M23" t="str">
+        <v>NA</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>de606917-da6f-4fde-881b-7cbfd45cfe56</v>
+        <v>f048c8fe-e8c9-4357-8ec8-ef76793e5bc1</v>
       </c>
       <c r="B24" t="str">
-        <v>Ricky Steve</v>
+        <v>Tamara Mifsud</v>
       </c>
       <c r="C24">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D24" t="str">
         <v>Female</v>
       </c>
       <c r="E24" t="str">
-        <v>tj-c-a@hotmail.com</v>
+        <v>tamara.mifsud@hotmail.com</v>
       </c>
       <c r="F24" t="str">
-        <v>411360449</v>
+        <v>416552122</v>
       </c>
       <c r="G24" t="str">
-        <v xml:space="preserve">Wangaratta </v>
+        <v>Aintree</v>
       </c>
       <c r="H24" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="I24" t="str">
-        <v>assigned</v>
+        <v>available</v>
       </c>
       <c r="J24" t="str">
-        <v>Taylah-Jayne Lockery</v>
+        <v>Aliye Abcilar</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
+        <v>6bbdadcb-23a8-41c9-964b-6152e234cb33</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Philip Natoli</v>
+      </c>
+      <c r="C25">
+        <v>29</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Philip.natoli@outlook.com</v>
+      </c>
+      <c r="F25" t="str">
+        <v>466021882</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Caulfield South</v>
+      </c>
+      <c r="H25" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I25" t="str">
+        <v>available</v>
+      </c>
+      <c r="J25" t="str">
+        <v>Hayley Wright</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
         <v>6cada433-8344-4d95-97dc-33c9c173ce7c</v>
       </c>
-      <c r="B25" t="str">
+      <c r="B26" t="str">
         <v>Jeanette Quy</v>
       </c>
-      <c r="C25">
+      <c r="C26">
         <v>74</v>
       </c>
-      <c r="D25" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E25" t="str">
+      <c r="D26" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E26" t="str">
         <v>quyfamily@tpg.com.au</v>
       </c>
-      <c r="F25" t="str">
+      <c r="F26" t="str">
         <v>402902273</v>
       </c>
-      <c r="G25" t="str">
+      <c r="G26" t="str">
         <v>Rowville</v>
       </c>
-      <c r="H25" t="str">
+      <c r="H26" t="str">
         <v>C</v>
       </c>
-      <c r="I25" t="str">
-        <v>available</v>
-      </c>
-      <c r="M25" t="str">
+      <c r="I26" t="str">
+        <v>available</v>
+      </c>
+      <c r="M26" t="str">
         <v xml:space="preserve">nothing of note </v>
       </c>
     </row>
-    <row r="26" xml:space="preserve">
-      <c r="A26" t="str">
+    <row r="27" xml:space="preserve">
+      <c r="A27" t="str">
         <v>dcd305dd-c710-4a1e-859c-835031154035</v>
       </c>
-      <c r="B26" t="str">
+      <c r="B27" t="str">
         <v>Nicholas Boicos</v>
       </c>
-      <c r="C26">
+      <c r="C27">
         <v>22</v>
       </c>
-      <c r="D26" t="str">
+      <c r="D27" t="str">
         <v>Male</v>
       </c>
-      <c r="E26" t="str">
+      <c r="E27" t="str">
         <v>nboicos@hotmail.com</v>
       </c>
-      <c r="F26" t="str">
+      <c r="F27" t="str">
         <v>429556400</v>
       </c>
-      <c r="G26" t="str">
+      <c r="G27" t="str">
         <v xml:space="preserve">Altona Meadows </v>
       </c>
-      <c r="H26" t="str">
+      <c r="H27" t="str">
         <v>B+</v>
       </c>
-      <c r="I26" t="str">
-        <v>available</v>
-      </c>
-      <c r="J26" t="str" xml:space="preserve">
+      <c r="I27" t="str">
+        <v>available</v>
+      </c>
+      <c r="J27" t="str" xml:space="preserve">
         <v xml:space="preserve">Nick Boicos 
 Matthew Boicos
 Brothers</v>
       </c>
     </row>
-    <row r="27" xml:space="preserve">
-      <c r="A27" t="str">
+    <row r="28" xml:space="preserve">
+      <c r="A28" t="str">
         <v>15fb53d0-3916-4c9a-9f73-c28c879dec33</v>
       </c>
-      <c r="B27" t="str">
+      <c r="B28" t="str">
         <v>Mozgda  Alime</v>
       </c>
-      <c r="C27">
+      <c r="C28">
         <v>39</v>
       </c>
-      <c r="D27" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E27" t="str">
+      <c r="D28" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E28" t="str">
         <v>smalimi@hotmail.com</v>
       </c>
-      <c r="F27" t="str">
+      <c r="F28" t="str">
         <v>402010235</v>
       </c>
-      <c r="G27" t="str">
+      <c r="G28" t="str">
         <v xml:space="preserve">Melbourne </v>
       </c>
-      <c r="H27" t="str">
+      <c r="H28" t="str">
         <v>C</v>
       </c>
-      <c r="I27" t="str">
-        <v>available</v>
-      </c>
-      <c r="J27" t="str" xml:space="preserve">
+      <c r="I28" t="str">
+        <v>available</v>
+      </c>
+      <c r="J28" t="str" xml:space="preserve">
         <v xml:space="preserve">Sadaf Almini - I believe this is her cousin 
 Lida Alime - I believe this is her cousin or sister 
 Ahmad Alime - Ahmad is Lina's husband </v>
       </c>
-      <c r="M27" t="str">
+      <c r="M28" t="str">
         <v xml:space="preserve">No </v>
-      </c>
-    </row>
-    <row r="28" xml:space="preserve">
-      <c r="A28" t="str">
-        <v>d9b76f1c-0867-44fc-9215-6ef7b1184af6</v>
-      </c>
-      <c r="B28" t="str">
-        <v>Kayla Lorenzini</v>
-      </c>
-      <c r="C28">
-        <v>29</v>
-      </c>
-      <c r="D28" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E28" t="str">
-        <v>kaylalorenzini_@hotmail.com</v>
-      </c>
-      <c r="F28" t="str">
-        <v>430517653</v>
-      </c>
-      <c r="G28" t="str">
-        <v>Melbourne</v>
-      </c>
-      <c r="H28" t="str">
-        <v>B+</v>
-      </c>
-      <c r="I28" t="str">
-        <v>assigned</v>
-      </c>
-      <c r="J28" t="str" xml:space="preserve">
-        <v xml:space="preserve">Kayla Lorenzini
-James Lorenzini
-Deanna Gramola</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>607e3750-92e2-4480-b39d-1cb0e026cd4b</v>
+        <v>f7b766dc-a0d0-4a91-98ef-47472cdca803</v>
       </c>
       <c r="B29" t="str">
-        <v>Natasha Devers</v>
+        <v>Mara Baumgardner</v>
       </c>
       <c r="C29">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="D29" t="str">
         <v>Female</v>
       </c>
       <c r="E29" t="str">
-        <v>natashadevers@gmail.com</v>
+        <v>Granic@hotmail.com</v>
       </c>
       <c r="F29" t="str">
-        <v>484003770</v>
+        <v>407364450</v>
       </c>
       <c r="G29" t="str">
-        <v xml:space="preserve">Waterways </v>
+        <v>Cockatoo</v>
       </c>
       <c r="H29" t="str">
         <v>B</v>
@@ -1650,109 +1653,106 @@
         <v>available</v>
       </c>
       <c r="J29" t="str">
-        <v>Oliver Moran</v>
+        <v xml:space="preserve">Mum - Mira Granic </v>
+      </c>
+      <c r="M29" t="str">
+        <v xml:space="preserve">No </v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>4f08069b-d828-429c-af5e-b1eee2c123df</v>
+        <v>607e3750-92e2-4480-b39d-1cb0e026cd4b</v>
       </c>
       <c r="B30" t="str">
-        <v>Sarah Desira</v>
+        <v>Natasha Devers</v>
       </c>
       <c r="C30">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="D30" t="str">
         <v>Female</v>
       </c>
       <c r="E30" t="str">
-        <v>unicornwolf11@gmail.com</v>
+        <v>natashadevers@gmail.com</v>
       </c>
       <c r="F30" t="str">
-        <v>450765125</v>
+        <v>484003770</v>
       </c>
       <c r="G30" t="str">
-        <v>Lara</v>
+        <v xml:space="preserve">Waterways </v>
       </c>
       <c r="H30" t="str">
         <v>B</v>
       </c>
       <c r="I30" t="str">
-        <v>assigned</v>
+        <v>available</v>
       </c>
       <c r="J30" t="str">
-        <v>Husband Daniel Desira b6042a-1-1936280</v>
-      </c>
-      <c r="M30" t="str">
-        <v xml:space="preserve">No </v>
+        <v>Oliver Moran</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>419afd3f-2406-423d-942f-2dfafe875f96</v>
+        <v>614641dd-4e94-4c42-a1d9-db37c608dcbe</v>
       </c>
       <c r="B31" t="str">
-        <v>Anna Fonua</v>
+        <v>Antonio Freno</v>
       </c>
       <c r="C31">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D31" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E31" t="str">
-        <v>Annawallace89@hotmail.com</v>
+        <v>frenoantonio@hotmail.it</v>
       </c>
       <c r="F31" t="str">
-        <v>452452442</v>
+        <v>422177371</v>
       </c>
       <c r="G31" t="str">
-        <v>Truganina</v>
+        <v>Glenroy</v>
       </c>
       <c r="H31" t="str">
-        <v>A</v>
+        <v>B+</v>
       </c>
       <c r="I31" t="str">
         <v>assigned</v>
       </c>
       <c r="J31" t="str">
-        <v>Dad Michael Wallace - b6042a-1-1936372</v>
-      </c>
-      <c r="M31" t="str">
-        <v xml:space="preserve">no </v>
+        <v>Solo</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>9f63aad3-aae1-4220-825c-8964694ec5d8</v>
+        <v>de606917-da6f-4fde-881b-7cbfd45cfe56</v>
       </c>
       <c r="B32" t="str">
-        <v>Kerrie Donald</v>
+        <v>Ricky Steve</v>
       </c>
       <c r="C32">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="D32" t="str">
         <v>Female</v>
       </c>
       <c r="E32" t="str">
-        <v>kerrieldonald@hotmail.com</v>
+        <v>tj-c-a@hotmail.com</v>
       </c>
       <c r="F32" t="str">
-        <v>61400826565</v>
+        <v>411360449</v>
       </c>
       <c r="G32" t="str">
-        <v>Mailor's Flat</v>
+        <v xml:space="preserve">Wangaratta </v>
       </c>
       <c r="H32" t="str">
-        <v>B+</v>
+        <v>A</v>
       </c>
       <c r="I32" t="str">
-        <v>assigned</v>
+        <v>available</v>
       </c>
       <c r="J32" t="str">
-        <v>kerrie donald, alistair donald</v>
+        <v>Taylah-Jayne Lockery</v>
       </c>
     </row>
     <row r="33">
@@ -1789,10 +1789,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2aadb3db-ad8e-4edd-a81d-f045a926ceb9</v>
+        <v>45c7f69f-dd89-41d8-b7f0-a83f77fa9d12</v>
       </c>
       <c r="B34" t="str">
-        <v>Alexander Leonard</v>
+        <v>Sherif Haggag</v>
       </c>
       <c r="C34">
         <v>38</v>
@@ -1801,45 +1801,45 @@
         <v>Male</v>
       </c>
       <c r="E34" t="str">
+        <v>Shaggag87@gmail.com</v>
+      </c>
+      <c r="F34" t="str">
+        <v>426233449</v>
+      </c>
+      <c r="G34" t="str">
+        <v>Belmont</v>
+      </c>
+      <c r="H34" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I34" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="J34" t="str">
+        <v>Solo</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>2aadb3db-ad8e-4edd-a81d-f045a926ceb9</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Alexander Leonard</v>
+      </c>
+      <c r="C35">
+        <v>38</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E35" t="str">
         <v>alexleonardedit@gmail.com</v>
       </c>
-      <c r="F34" t="str">
+      <c r="F35" t="str">
         <v>421834476</v>
       </c>
-      <c r="G34" t="str">
+      <c r="G35" t="str">
         <v>Croydon</v>
-      </c>
-      <c r="H34" t="str">
-        <v>A+</v>
-      </c>
-      <c r="I34" t="str">
-        <v>available</v>
-      </c>
-      <c r="J34" t="str">
-        <v>melissa francis, Alexander Leonard</v>
-      </c>
-    </row>
-    <row r="35" xml:space="preserve">
-      <c r="A35" t="str">
-        <v>1211456d-ea92-4a7b-9d94-885982cf345c</v>
-      </c>
-      <c r="B35" t="str">
-        <v>Bronwyn Parsons</v>
-      </c>
-      <c r="C35">
-        <v>72</v>
-      </c>
-      <c r="D35" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E35" t="str">
-        <v>Babybear61153@gmail.com</v>
-      </c>
-      <c r="F35" t="str">
-        <v>432543647</v>
-      </c>
-      <c r="G35" t="str">
-        <v>Rosebud</v>
       </c>
       <c r="H35" t="str">
         <v>A+</v>
@@ -1847,178 +1847,179 @@
       <c r="I35" t="str">
         <v>available</v>
       </c>
-      <c r="J35" t="str" xml:space="preserve">
-        <v xml:space="preserve">Yolette Huon - yol-et Hue on
-Bronwyn Parsons - Would like to be called Bron Emmerson - maiden name</v>
+      <c r="J35" t="str">
+        <v>melissa francis, Alexander Leonard</v>
       </c>
     </row>
     <row r="36" xml:space="preserve">
       <c r="A36" t="str">
-        <v>23f118f9-20db-422c-8cef-939dc73dd803</v>
+        <v>ed91813b-2f74-4638-9d1a-ef8c54cff447</v>
       </c>
       <c r="B36" t="str">
-        <v>Paige Greig</v>
+        <v>Linda Browne</v>
       </c>
       <c r="C36">
-        <v>31</v>
+        <v>54</v>
       </c>
       <c r="D36" t="str">
         <v>Female</v>
       </c>
       <c r="E36" t="str">
-        <v>paigegreig@hotmail.com</v>
+        <v>Lindabrowne@iprimus.com.au</v>
       </c>
       <c r="F36" t="str">
-        <v>406598552</v>
+        <v>429570177</v>
       </c>
       <c r="G36" t="str">
-        <v>Mooroolbark</v>
+        <v>OFFICER</v>
       </c>
       <c r="H36" t="str">
-        <v>C</v>
+        <v>B</v>
       </c>
       <c r="I36" t="str">
         <v>available</v>
       </c>
       <c r="J36" t="str" xml:space="preserve">
-        <v xml:space="preserve">Erin
-Morgan (sister) - need to do application</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <v>cbfeb8b0-bd5d-4614-a055-cbac047cf152</v>
-      </c>
-      <c r="B37" t="str">
-        <v>Tamika Colville</v>
-      </c>
-      <c r="C37">
-        <v>31</v>
-      </c>
-      <c r="D37" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E37" t="str">
-        <v>tamika.colville@gmail.com</v>
-      </c>
-      <c r="F37" t="str">
-        <v>409132141</v>
-      </c>
-      <c r="G37" t="str">
-        <v>Golden square</v>
-      </c>
-      <c r="H37" t="str">
-        <v>B+</v>
-      </c>
-      <c r="I37" t="str">
-        <v>assigned</v>
-      </c>
-      <c r="J37" t="str">
-        <v>Shinae Colville</v>
-      </c>
-      <c r="L37" t="str">
-        <v>Diagnosed with MS in 2018</v>
-      </c>
-      <c r="M37" t="str">
-        <v>NA</v>
-      </c>
-    </row>
-    <row r="38" xml:space="preserve">
-      <c r="A38" t="str">
-        <v>ed91813b-2f74-4638-9d1a-ef8c54cff447</v>
-      </c>
-      <c r="B38" t="str">
-        <v>Linda Browne</v>
-      </c>
-      <c r="C38">
-        <v>54</v>
-      </c>
-      <c r="D38" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E38" t="str">
-        <v>Lindabrowne@iprimus.com.au</v>
-      </c>
-      <c r="F38" t="str">
-        <v>429570177</v>
-      </c>
-      <c r="G38" t="str">
-        <v>OFFICER</v>
-      </c>
-      <c r="H38" t="str">
-        <v>B</v>
-      </c>
-      <c r="I38" t="str">
-        <v>assigned</v>
-      </c>
-      <c r="J38" t="str" xml:space="preserve">
         <v xml:space="preserve">Natalie Browne
 Linda Browne
 Aidan Miler</v>
       </c>
     </row>
-    <row r="39">
+    <row r="37" xml:space="preserve">
+      <c r="A37" t="str">
+        <v>54de1dd9-b7eb-489d-b4a1-8b3744a385c4</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Dhananjay  Mehra</v>
+      </c>
+      <c r="C37">
+        <v>68</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Dmehra@bigpond.net.au</v>
+      </c>
+      <c r="F37" t="str">
+        <v>419353328</v>
+      </c>
+      <c r="G37" t="str">
+        <v xml:space="preserve">Point Cook </v>
+      </c>
+      <c r="H37" t="str">
+        <v>B</v>
+      </c>
+      <c r="I37" t="str">
+        <v>available</v>
+      </c>
+      <c r="J37" t="str" xml:space="preserve">
+        <v xml:space="preserve">Meenakshi Mehra
+Dhananjay Mehra</v>
+      </c>
+    </row>
+    <row r="38" xml:space="preserve">
+      <c r="A38" t="str">
+        <v>1211456d-ea92-4a7b-9d94-885982cf345c</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Bronwyn Parsons</v>
+      </c>
+      <c r="C38">
+        <v>72</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Babybear61153@gmail.com</v>
+      </c>
+      <c r="F38" t="str">
+        <v>432543647</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Rosebud</v>
+      </c>
+      <c r="H38" t="str">
+        <v>A+</v>
+      </c>
+      <c r="I38" t="str">
+        <v>available</v>
+      </c>
+      <c r="J38" t="str" xml:space="preserve">
+        <v xml:space="preserve">Yolette Huon - yol-et Hue on
+Bronwyn Parsons - Would like to be called Bron Emmerson - maiden name</v>
+      </c>
+    </row>
+    <row r="39" xml:space="preserve">
       <c r="A39" t="str">
-        <v>45c7f69f-dd89-41d8-b7f0-a83f77fa9d12</v>
+        <v>23f118f9-20db-422c-8cef-939dc73dd803</v>
       </c>
       <c r="B39" t="str">
-        <v>Sherif Haggag</v>
+        <v>Paige Greig</v>
       </c>
       <c r="C39">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="D39" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E39" t="str">
-        <v>Shaggag87@gmail.com</v>
+        <v>paigegreig@hotmail.com</v>
       </c>
       <c r="F39" t="str">
-        <v>426233449</v>
+        <v>406598552</v>
       </c>
       <c r="G39" t="str">
-        <v>Belmont</v>
+        <v>Mooroolbark</v>
       </c>
       <c r="H39" t="str">
-        <v>B+</v>
+        <v>C</v>
       </c>
       <c r="I39" t="str">
-        <v>assigned</v>
-      </c>
-      <c r="J39" t="str">
-        <v>Solo</v>
+        <v>available</v>
+      </c>
+      <c r="J39" t="str" xml:space="preserve">
+        <v xml:space="preserve">Erin
+Morgan (sister) - need to do application</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>646d2ff7-803b-4c80-bdd6-09d44eec6929</v>
+        <v>cbfeb8b0-bd5d-4614-a055-cbac047cf152</v>
       </c>
       <c r="B40" t="str">
-        <v>Leanne Bryant</v>
+        <v>Tamika Colville</v>
       </c>
       <c r="C40">
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="D40" t="str">
         <v>Female</v>
       </c>
       <c r="E40" t="str">
-        <v>blazeandcougar@gmail.com</v>
+        <v>tamika.colville@gmail.com</v>
       </c>
       <c r="F40" t="str">
-        <v>61415438228</v>
+        <v>409132141</v>
       </c>
       <c r="G40" t="str">
-        <v xml:space="preserve">Hampton Park </v>
+        <v>Golden square</v>
       </c>
       <c r="H40" t="str">
-        <v>B</v>
+        <v>B+</v>
       </c>
       <c r="I40" t="str">
-        <v>assigned</v>
+        <v>available</v>
       </c>
       <c r="J40" t="str">
-        <v>Solo</v>
+        <v>Shinae Colville</v>
+      </c>
+      <c r="L40" t="str">
+        <v>Diagnosed with MS in 2018</v>
+      </c>
+      <c r="M40" t="str">
+        <v>NA</v>
       </c>
     </row>
     <row r="41">
@@ -2055,28 +2056,28 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>c60666dd-e08c-4aa0-8582-4e7a3ad280f8</v>
+        <v>646d2ff7-803b-4c80-bdd6-09d44eec6929</v>
       </c>
       <c r="B42" t="str">
-        <v>Bashar Mona</v>
+        <v>Leanne Bryant</v>
       </c>
       <c r="C42">
-        <v>33</v>
+        <v>63</v>
       </c>
       <c r="D42" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E42" t="str">
-        <v>bashar.mona92@gmail.com</v>
+        <v>blazeandcougar@gmail.com</v>
       </c>
       <c r="F42" t="str">
-        <v>490871416</v>
+        <v>61415438228</v>
       </c>
       <c r="G42" t="str">
-        <v>Roxburgh park</v>
+        <v xml:space="preserve">Hampton Park </v>
       </c>
       <c r="H42" t="str">
-        <v>B+</v>
+        <v>B</v>
       </c>
       <c r="I42" t="str">
         <v>assigned</v>
@@ -2153,37 +2154,36 @@
         <v>NA</v>
       </c>
     </row>
-    <row r="45" xml:space="preserve">
+    <row r="45">
       <c r="A45" t="str">
-        <v>54de1dd9-b7eb-489d-b4a1-8b3744a385c4</v>
+        <v>c60666dd-e08c-4aa0-8582-4e7a3ad280f8</v>
       </c>
       <c r="B45" t="str">
-        <v>Dhananjay  Mehra</v>
+        <v>Bashar Mona</v>
       </c>
       <c r="C45">
-        <v>68</v>
+        <v>33</v>
       </c>
       <c r="D45" t="str">
         <v>Male</v>
       </c>
       <c r="E45" t="str">
-        <v>Dmehra@bigpond.net.au</v>
+        <v>bashar.mona92@gmail.com</v>
       </c>
       <c r="F45" t="str">
-        <v>419353328</v>
+        <v>490871416</v>
       </c>
       <c r="G45" t="str">
-        <v xml:space="preserve">Point Cook </v>
+        <v>Roxburgh park</v>
       </c>
       <c r="H45" t="str">
-        <v>B</v>
+        <v>B+</v>
       </c>
       <c r="I45" t="str">
         <v>assigned</v>
       </c>
-      <c r="J45" t="str" xml:space="preserve">
-        <v xml:space="preserve">Meenakshi Mehra
-Dhananjay Mehra</v>
+      <c r="J45" t="str">
+        <v>Solo</v>
       </c>
     </row>
     <row r="46">
@@ -2390,7 +2390,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2420,64 +2420,64 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ad340cba-9702-4a35-9a1f-7098bb2792d2</v>
+        <v>57d358cb-d720-4484-8903-846208a88129</v>
       </c>
       <c r="B2" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C2" t="str">
-        <v>b1fc34e8-20cb-4607-9568-0761cf4520a6</v>
+        <v>6b9ae7f0-4a81-4dda-8e55-e49415d98ec6</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
       <c r="E2" t="str">
-        <v>A1</v>
+        <v>A3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>055b0eeb-95e3-48d2-bab8-608bbe0173ce</v>
+        <v>90a868f7-87c2-4b18-888a-1b0729aafd57</v>
       </c>
       <c r="B3" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C3" t="str">
-        <v>6b9ae7f0-4a81-4dda-8e55-e49415d98ec6</v>
+        <v>b1fc34e8-20cb-4607-9568-0761cf4520a6</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
       <c r="E3" t="str">
-        <v>A2</v>
+        <v>A4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>69e786fd-e21d-4e14-88da-7125c5f4a1d2</v>
+        <v>f569744b-ca7b-46c3-b54f-b206d35d07d0</v>
       </c>
       <c r="B4" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C4" t="str">
-        <v>7fc083f6-6be3-42bf-b4e5-fc6412e1c559</v>
+        <v>614641dd-4e94-4c42-a1d9-db37c608dcbe</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
       <c r="E4" t="str">
-        <v>A3</v>
+        <v>A5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>eb8bfbdd-63a6-4079-aba9-5800fb7a540b</v>
+        <v>19fd7f06-6147-4090-b47d-4769aeb855ce</v>
       </c>
       <c r="B5" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C5" t="str">
-        <v>34b3d848-f096-4bc9-bd55-dc4dd85ad1b3</v>
+        <v>e4a52d0d-9c54-4504-8a0f-85845cd88e27</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -2488,330 +2488,92 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>a3858d3d-55d1-4fdb-97d8-320bba44e137</v>
+        <v>01417c60-8dda-4286-a14c-ec8309236d41</v>
       </c>
       <c r="B6" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C6" t="str">
-        <v>e4a52d0d-9c54-4504-8a0f-85845cd88e27</v>
+        <v>96c75db9-b001-4abe-8ddb-d5a73cb04529</v>
       </c>
       <c r="D6">
         <v>1</v>
       </c>
       <c r="E6" t="str">
-        <v>B2</v>
+        <v>B4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>b52bba5a-5df3-4857-bd40-94b252176098</v>
+        <v>7d428f41-6701-460f-8c5e-fcf5f9f1e673</v>
       </c>
       <c r="B7" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C7" t="str">
-        <v>96c75db9-b001-4abe-8ddb-d5a73cb04529</v>
+        <v>646d2ff7-803b-4c80-bdd6-09d44eec6929</v>
       </c>
       <c r="D7">
         <v>1</v>
       </c>
       <c r="E7" t="str">
-        <v>B3</v>
+        <v>B5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>4f0e1cd0-0b97-41cf-8546-066d8aacaa18</v>
+        <v>2b9aa451-0238-45e5-96cd-ebd805d71c7b</v>
       </c>
       <c r="B8" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C8" t="str">
-        <v>d9b76f1c-0867-44fc-9215-6ef7b1184af6</v>
+        <v>917bd31e-7781-44cc-936c-980cb1f844aa</v>
       </c>
       <c r="D8">
         <v>1</v>
       </c>
       <c r="E8" t="str">
-        <v>B4</v>
+        <v>C1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>e1a80551-d2da-4874-91db-588715a4fac4</v>
+        <v>3c5d1dfd-7f7d-4eec-b21f-5596ec0c9e4a</v>
       </c>
       <c r="B9" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C9" t="str">
-        <v>9f63aad3-aae1-4220-825c-8964694ec5d8</v>
+        <v>c60666dd-e08c-4aa0-8582-4e7a3ad280f8</v>
       </c>
       <c r="D9">
         <v>1</v>
       </c>
       <c r="E9" t="str">
-        <v>B5</v>
+        <v>C2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>abc48d6d-e2be-45f3-b39d-aab68fd3a887</v>
+        <v>51037cc9-d563-444d-91e7-4c94330a4d63</v>
       </c>
       <c r="B10" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C10" t="str">
-        <v>97e81b41-1b8d-4562-9e12-3747f87663a9</v>
+        <v>45c7f69f-dd89-41d8-b7f0-a83f77fa9d12</v>
       </c>
       <c r="D10">
         <v>1</v>
       </c>
       <c r="E10" t="str">
-        <v>C1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>1996d94e-e4b6-41eb-9c86-6f2ce57c0d3e</v>
-      </c>
-      <c r="B11" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C11" t="str">
-        <v>614641dd-4e94-4c42-a1d9-db37c608dcbe</v>
-      </c>
-      <c r="D11">
-        <v>1</v>
-      </c>
-      <c r="E11" t="str">
-        <v>C2</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>15371ee3-0b7e-4086-84f6-3720ca1ff543</v>
-      </c>
-      <c r="B12" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C12" t="str">
-        <v>45c7f69f-dd89-41d8-b7f0-a83f77fa9d12</v>
-      </c>
-      <c r="D12">
-        <v>1</v>
-      </c>
-      <c r="E12" t="str">
         <v>C3</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>9c31ffbb-2789-43bb-a60e-90c4b8100cef</v>
-      </c>
-      <c r="B13" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C13" t="str">
-        <v>646d2ff7-803b-4c80-bdd6-09d44eec6929</v>
-      </c>
-      <c r="D13">
-        <v>1</v>
-      </c>
-      <c r="E13" t="str">
-        <v>C4</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>bc578b4a-ddea-41c3-9540-e88f6659f18c</v>
-      </c>
-      <c r="B14" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C14" t="str">
-        <v>cbfeb8b0-bd5d-4614-a055-cbac047cf152</v>
-      </c>
-      <c r="D14">
-        <v>1</v>
-      </c>
-      <c r="E14" t="str">
-        <v>D1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>72473e20-842c-4521-a6c8-ba7c2d625b26</v>
-      </c>
-      <c r="B15" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C15" t="str">
-        <v>ed91813b-2f74-4638-9d1a-ef8c54cff447</v>
-      </c>
-      <c r="D15">
-        <v>1</v>
-      </c>
-      <c r="E15" t="str">
-        <v>D2</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>cdfce1b8-2ada-4f40-a965-ec4421f32195</v>
-      </c>
-      <c r="B16" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C16" t="str">
-        <v>c60666dd-e08c-4aa0-8582-4e7a3ad280f8</v>
-      </c>
-      <c r="D16">
-        <v>1</v>
-      </c>
-      <c r="E16" t="str">
-        <v>D3</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>0bafba7c-79a0-4bae-b175-028f5c764b20</v>
-      </c>
-      <c r="B17" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C17" t="str">
-        <v>917bd31e-7781-44cc-936c-980cb1f844aa</v>
-      </c>
-      <c r="D17">
-        <v>1</v>
-      </c>
-      <c r="E17" t="str">
-        <v>D4</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>94521f77-45d2-4af9-952a-a692cd7c7aa8</v>
-      </c>
-      <c r="B18" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C18" t="str">
-        <v>54de1dd9-b7eb-489d-b4a1-8b3744a385c4</v>
-      </c>
-      <c r="D18">
-        <v>1</v>
-      </c>
-      <c r="E18" t="str">
-        <v>E1</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>38e2c0fc-5873-43aa-9394-f7c2709f8a83</v>
-      </c>
-      <c r="B19" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C19" t="str">
-        <v>1fe25fd6-dc69-4d29-b22f-9a15ad3d457f</v>
-      </c>
-      <c r="D19">
-        <v>1</v>
-      </c>
-      <c r="E19" t="str">
-        <v>E2</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>c21a4154-3157-46c8-a878-b599e0689d93</v>
-      </c>
-      <c r="B20" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C20" t="str">
-        <v>82960b61-d36b-49e2-9ddf-a7b8e0b02a63</v>
-      </c>
-      <c r="D20">
-        <v>2</v>
-      </c>
-      <c r="E20" t="str">
-        <v>A1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>ffc84c94-f1d0-4b10-aa29-30dc6ffbda57</v>
-      </c>
-      <c r="B21" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C21" t="str">
-        <v>4f08069b-d828-429c-af5e-b1eee2c123df</v>
-      </c>
-      <c r="D21">
-        <v>2</v>
-      </c>
-      <c r="E21" t="str">
-        <v>A2</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>b27d2d06-2e2c-4115-9995-db7dd2a60c77</v>
-      </c>
-      <c r="B22" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C22" t="str">
-        <v>419afd3f-2406-423d-942f-2dfafe875f96</v>
-      </c>
-      <c r="D22">
-        <v>2</v>
-      </c>
-      <c r="E22" t="str">
-        <v>A3</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>7a2cb7e6-2374-470d-916d-9e0890d7fde8</v>
-      </c>
-      <c r="B23" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C23" t="str">
-        <v>f7b766dc-a0d0-4a91-98ef-47472cdca803</v>
-      </c>
-      <c r="D23">
-        <v>2</v>
-      </c>
-      <c r="E23" t="str">
-        <v>A4</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>36893ad6-bfef-4de4-b6f2-a5c5f1b825b0</v>
-      </c>
-      <c r="B24" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C24" t="str">
-        <v>de606917-da6f-4fde-881b-7cbfd45cfe56</v>
-      </c>
-      <c r="D24">
-        <v>2</v>
-      </c>
-      <c r="E24" t="str">
-        <v>A5</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H10"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Persist contestant groups created through automatic assignment
Modify the auto-assign logic in `server/routes.ts` to create and persist new groups to the database when contestants are matched via `attendingWith`. This ensures that grouped contestants receive a shared `groupId`, enabling the linked icon to appear correctly on the seating chart. The changes also address an async issue by converting a `forEach` loop to a `for...of` loop to properly handle `await` operations when creating database groups and updating contestant records.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: f123b9d7-6af8-472a-a75c-70d0b78d0583
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: e87a5a41-3e28-4a5e-bb60-b116eb990ab6
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/4ca2a1f8-42ce-4303-beff-eb92e3283d4c/f123b9d7-6af8-472a-a75c-70d0b78d0583/SA70FQN
</commit_message>
<xml_diff>
--- a/storage/backups/automatic-backup.xlsx
+++ b/storage/backups/automatic-backup.xlsx
@@ -736,7 +736,7 @@
         <v>B</v>
       </c>
       <c r="I2" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J2" t="str" xml:space="preserve">
         <v xml:space="preserve">Meenakshi Mehra
@@ -1424,167 +1424,167 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>96c75db9-b001-4abe-8ddb-d5a73cb04529</v>
+        <v>f048c8fe-e8c9-4357-8ec8-ef76793e5bc1</v>
       </c>
       <c r="B23" t="str">
-        <v>Kiran Rao</v>
+        <v>Tamara Mifsud</v>
       </c>
       <c r="C23">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D23" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E23" t="str">
-        <v>kiran.rao07@gmail.com</v>
+        <v>tamara.mifsud@hotmail.com</v>
       </c>
       <c r="F23" t="str">
-        <v>420486042</v>
+        <v>416552122</v>
       </c>
       <c r="G23" t="str">
-        <v>Southbank</v>
+        <v>Aintree</v>
       </c>
       <c r="H23" t="str">
-        <v>B+</v>
+        <v>B</v>
       </c>
       <c r="I23" t="str">
-        <v>assigned</v>
+        <v>available</v>
       </c>
       <c r="J23" t="str">
-        <v>SOLO</v>
-      </c>
-      <c r="M23" t="str">
-        <v>NA</v>
+        <v>Aliye Abcilar</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>f048c8fe-e8c9-4357-8ec8-ef76793e5bc1</v>
+        <v>6bbdadcb-23a8-41c9-964b-6152e234cb33</v>
       </c>
       <c r="B24" t="str">
-        <v>Tamara Mifsud</v>
+        <v>Philip Natoli</v>
       </c>
       <c r="C24">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D24" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E24" t="str">
-        <v>tamara.mifsud@hotmail.com</v>
+        <v>Philip.natoli@outlook.com</v>
       </c>
       <c r="F24" t="str">
-        <v>416552122</v>
+        <v>466021882</v>
       </c>
       <c r="G24" t="str">
-        <v>Aintree</v>
+        <v>Caulfield South</v>
       </c>
       <c r="H24" t="str">
-        <v>B</v>
+        <v>B+</v>
       </c>
       <c r="I24" t="str">
         <v>available</v>
       </c>
       <c r="J24" t="str">
-        <v>Aliye Abcilar</v>
+        <v>Hayley Wright</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>6bbdadcb-23a8-41c9-964b-6152e234cb33</v>
+        <v>6cada433-8344-4d95-97dc-33c9c173ce7c</v>
       </c>
       <c r="B25" t="str">
-        <v>Philip Natoli</v>
+        <v>Jeanette Quy</v>
       </c>
       <c r="C25">
-        <v>29</v>
+        <v>74</v>
       </c>
       <c r="D25" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E25" t="str">
+        <v>quyfamily@tpg.com.au</v>
+      </c>
+      <c r="F25" t="str">
+        <v>402902273</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Rowville</v>
+      </c>
+      <c r="H25" t="str">
+        <v>C</v>
+      </c>
+      <c r="I25" t="str">
+        <v>available</v>
+      </c>
+      <c r="M25" t="str">
+        <v xml:space="preserve">nothing of note </v>
+      </c>
+    </row>
+    <row r="26" xml:space="preserve">
+      <c r="A26" t="str">
+        <v>dcd305dd-c710-4a1e-859c-835031154035</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Nicholas Boicos</v>
+      </c>
+      <c r="C26">
+        <v>22</v>
+      </c>
+      <c r="D26" t="str">
         <v>Male</v>
       </c>
-      <c r="E25" t="str">
-        <v>Philip.natoli@outlook.com</v>
-      </c>
-      <c r="F25" t="str">
-        <v>466021882</v>
-      </c>
-      <c r="G25" t="str">
-        <v>Caulfield South</v>
-      </c>
-      <c r="H25" t="str">
+      <c r="E26" t="str">
+        <v>nboicos@hotmail.com</v>
+      </c>
+      <c r="F26" t="str">
+        <v>429556400</v>
+      </c>
+      <c r="G26" t="str">
+        <v xml:space="preserve">Altona Meadows </v>
+      </c>
+      <c r="H26" t="str">
         <v>B+</v>
       </c>
-      <c r="I25" t="str">
-        <v>available</v>
-      </c>
-      <c r="J25" t="str">
-        <v>Hayley Wright</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>6cada433-8344-4d95-97dc-33c9c173ce7c</v>
-      </c>
-      <c r="B26" t="str">
-        <v>Jeanette Quy</v>
-      </c>
-      <c r="C26">
-        <v>74</v>
-      </c>
-      <c r="D26" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E26" t="str">
-        <v>quyfamily@tpg.com.au</v>
-      </c>
-      <c r="F26" t="str">
-        <v>402902273</v>
-      </c>
-      <c r="G26" t="str">
-        <v>Rowville</v>
-      </c>
-      <c r="H26" t="str">
-        <v>C</v>
-      </c>
       <c r="I26" t="str">
         <v>available</v>
       </c>
-      <c r="M26" t="str">
-        <v xml:space="preserve">nothing of note </v>
-      </c>
-    </row>
-    <row r="27" xml:space="preserve">
-      <c r="A27" t="str">
-        <v>dcd305dd-c710-4a1e-859c-835031154035</v>
-      </c>
-      <c r="B27" t="str">
-        <v>Nicholas Boicos</v>
-      </c>
-      <c r="C27">
-        <v>22</v>
-      </c>
-      <c r="D27" t="str">
-        <v>Male</v>
-      </c>
-      <c r="E27" t="str">
-        <v>nboicos@hotmail.com</v>
-      </c>
-      <c r="F27" t="str">
-        <v>429556400</v>
-      </c>
-      <c r="G27" t="str">
-        <v xml:space="preserve">Altona Meadows </v>
-      </c>
-      <c r="H27" t="str">
-        <v>B+</v>
-      </c>
-      <c r="I27" t="str">
-        <v>available</v>
-      </c>
-      <c r="J27" t="str" xml:space="preserve">
+      <c r="J26" t="str" xml:space="preserve">
         <v xml:space="preserve">Nick Boicos 
 Matthew Boicos
 Brothers</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>96c75db9-b001-4abe-8ddb-d5a73cb04529</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Kiran Rao</v>
+      </c>
+      <c r="C27">
+        <v>35</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E27" t="str">
+        <v>kiran.rao07@gmail.com</v>
+      </c>
+      <c r="F27" t="str">
+        <v>420486042</v>
+      </c>
+      <c r="G27" t="str">
+        <v>Southbank</v>
+      </c>
+      <c r="H27" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I27" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="J27" t="str">
+        <v>SOLO</v>
+      </c>
+      <c r="M27" t="str">
+        <v>NA</v>
       </c>
     </row>
     <row r="28" xml:space="preserve">
@@ -1789,25 +1789,25 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>45c7f69f-dd89-41d8-b7f0-a83f77fa9d12</v>
+        <v>c60666dd-e08c-4aa0-8582-4e7a3ad280f8</v>
       </c>
       <c r="B34" t="str">
-        <v>Sherif Haggag</v>
+        <v>Bashar Mona</v>
       </c>
       <c r="C34">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D34" t="str">
         <v>Male</v>
       </c>
       <c r="E34" t="str">
-        <v>Shaggag87@gmail.com</v>
+        <v>bashar.mona92@gmail.com</v>
       </c>
       <c r="F34" t="str">
-        <v>426233449</v>
+        <v>490871416</v>
       </c>
       <c r="G34" t="str">
-        <v>Belmont</v>
+        <v>Roxburgh park</v>
       </c>
       <c r="H34" t="str">
         <v>B+</v>
@@ -1887,136 +1887,133 @@
     </row>
     <row r="37" xml:space="preserve">
       <c r="A37" t="str">
+        <v>1211456d-ea92-4a7b-9d94-885982cf345c</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Bronwyn Parsons</v>
+      </c>
+      <c r="C37">
+        <v>72</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Babybear61153@gmail.com</v>
+      </c>
+      <c r="F37" t="str">
+        <v>432543647</v>
+      </c>
+      <c r="G37" t="str">
+        <v>Rosebud</v>
+      </c>
+      <c r="H37" t="str">
+        <v>A+</v>
+      </c>
+      <c r="I37" t="str">
+        <v>available</v>
+      </c>
+      <c r="J37" t="str" xml:space="preserve">
+        <v xml:space="preserve">Yolette Huon - yol-et Hue on
+Bronwyn Parsons - Would like to be called Bron Emmerson - maiden name</v>
+      </c>
+    </row>
+    <row r="38" xml:space="preserve">
+      <c r="A38" t="str">
+        <v>23f118f9-20db-422c-8cef-939dc73dd803</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Paige Greig</v>
+      </c>
+      <c r="C38">
+        <v>31</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E38" t="str">
+        <v>paigegreig@hotmail.com</v>
+      </c>
+      <c r="F38" t="str">
+        <v>406598552</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Mooroolbark</v>
+      </c>
+      <c r="H38" t="str">
+        <v>C</v>
+      </c>
+      <c r="I38" t="str">
+        <v>available</v>
+      </c>
+      <c r="J38" t="str" xml:space="preserve">
+        <v xml:space="preserve">Erin
+Morgan (sister) - need to do application</v>
+      </c>
+    </row>
+    <row r="39" xml:space="preserve">
+      <c r="A39" t="str">
         <v>54de1dd9-b7eb-489d-b4a1-8b3744a385c4</v>
       </c>
-      <c r="B37" t="str">
+      <c r="B39" t="str">
         <v>Dhananjay  Mehra</v>
       </c>
-      <c r="C37">
+      <c r="C39">
         <v>68</v>
       </c>
-      <c r="D37" t="str">
+      <c r="D39" t="str">
         <v>Male</v>
       </c>
-      <c r="E37" t="str">
+      <c r="E39" t="str">
         <v>Dmehra@bigpond.net.au</v>
       </c>
-      <c r="F37" t="str">
+      <c r="F39" t="str">
         <v>419353328</v>
       </c>
-      <c r="G37" t="str">
+      <c r="G39" t="str">
         <v xml:space="preserve">Point Cook </v>
       </c>
-      <c r="H37" t="str">
+      <c r="H39" t="str">
         <v>B</v>
       </c>
-      <c r="I37" t="str">
-        <v>available</v>
-      </c>
-      <c r="J37" t="str" xml:space="preserve">
+      <c r="I39" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="J39" t="str" xml:space="preserve">
         <v xml:space="preserve">Meenakshi Mehra
 Dhananjay Mehra</v>
       </c>
     </row>
-    <row r="38" xml:space="preserve">
-      <c r="A38" t="str">
-        <v>1211456d-ea92-4a7b-9d94-885982cf345c</v>
-      </c>
-      <c r="B38" t="str">
-        <v>Bronwyn Parsons</v>
-      </c>
-      <c r="C38">
-        <v>72</v>
-      </c>
-      <c r="D38" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E38" t="str">
-        <v>Babybear61153@gmail.com</v>
-      </c>
-      <c r="F38" t="str">
-        <v>432543647</v>
-      </c>
-      <c r="G38" t="str">
-        <v>Rosebud</v>
-      </c>
-      <c r="H38" t="str">
-        <v>A+</v>
-      </c>
-      <c r="I38" t="str">
-        <v>available</v>
-      </c>
-      <c r="J38" t="str" xml:space="preserve">
-        <v xml:space="preserve">Yolette Huon - yol-et Hue on
-Bronwyn Parsons - Would like to be called Bron Emmerson - maiden name</v>
-      </c>
-    </row>
-    <row r="39" xml:space="preserve">
-      <c r="A39" t="str">
-        <v>23f118f9-20db-422c-8cef-939dc73dd803</v>
-      </c>
-      <c r="B39" t="str">
-        <v>Paige Greig</v>
-      </c>
-      <c r="C39">
-        <v>31</v>
-      </c>
-      <c r="D39" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E39" t="str">
-        <v>paigegreig@hotmail.com</v>
-      </c>
-      <c r="F39" t="str">
-        <v>406598552</v>
-      </c>
-      <c r="G39" t="str">
-        <v>Mooroolbark</v>
-      </c>
-      <c r="H39" t="str">
-        <v>C</v>
-      </c>
-      <c r="I39" t="str">
-        <v>available</v>
-      </c>
-      <c r="J39" t="str" xml:space="preserve">
-        <v xml:space="preserve">Erin
-Morgan (sister) - need to do application</v>
-      </c>
-    </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>cbfeb8b0-bd5d-4614-a055-cbac047cf152</v>
+        <v>917bd31e-7781-44cc-936c-980cb1f844aa</v>
       </c>
       <c r="B40" t="str">
-        <v>Tamika Colville</v>
+        <v>Angela Verspay</v>
       </c>
       <c r="C40">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="D40" t="str">
         <v>Female</v>
       </c>
       <c r="E40" t="str">
-        <v>tamika.colville@gmail.com</v>
+        <v>angelarileysmyth@hotmail.com</v>
       </c>
       <c r="F40" t="str">
-        <v>409132141</v>
+        <v>477660119</v>
       </c>
       <c r="G40" t="str">
-        <v>Golden square</v>
+        <v>Warrnambool</v>
       </c>
       <c r="H40" t="str">
-        <v>B+</v>
+        <v>B</v>
       </c>
       <c r="I40" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J40" t="str">
-        <v>Shinae Colville</v>
-      </c>
-      <c r="L40" t="str">
-        <v>Diagnosed with MS in 2018</v>
+        <v>SOLO</v>
       </c>
       <c r="M40" t="str">
         <v>NA</v>
@@ -2024,25 +2021,25 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>441f345e-57a2-403b-a9a9-8284261eba7b</v>
+        <v>cbfeb8b0-bd5d-4614-a055-cbac047cf152</v>
       </c>
       <c r="B41" t="str">
-        <v>Kadisha  Bruton</v>
+        <v>Tamika Colville</v>
       </c>
       <c r="C41">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="D41" t="str">
         <v>Female</v>
       </c>
       <c r="E41" t="str">
-        <v>kadishaann@icloud.com</v>
+        <v>tamika.colville@gmail.com</v>
       </c>
       <c r="F41" t="str">
-        <v>434829249</v>
+        <v>409132141</v>
       </c>
       <c r="G41" t="str">
-        <v xml:space="preserve">Kurunjang </v>
+        <v>Golden square</v>
       </c>
       <c r="H41" t="str">
         <v>B+</v>
@@ -2051,33 +2048,39 @@
         <v>available</v>
       </c>
       <c r="J41" t="str">
-        <v>Jacob Steele</v>
+        <v>Shinae Colville</v>
+      </c>
+      <c r="L41" t="str">
+        <v>Diagnosed with MS in 2018</v>
+      </c>
+      <c r="M41" t="str">
+        <v>NA</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>646d2ff7-803b-4c80-bdd6-09d44eec6929</v>
+        <v>45c7f69f-dd89-41d8-b7f0-a83f77fa9d12</v>
       </c>
       <c r="B42" t="str">
-        <v>Leanne Bryant</v>
+        <v>Sherif Haggag</v>
       </c>
       <c r="C42">
-        <v>63</v>
+        <v>38</v>
       </c>
       <c r="D42" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E42" t="str">
-        <v>blazeandcougar@gmail.com</v>
+        <v>Shaggag87@gmail.com</v>
       </c>
       <c r="F42" t="str">
-        <v>61415438228</v>
+        <v>426233449</v>
       </c>
       <c r="G42" t="str">
-        <v xml:space="preserve">Hampton Park </v>
+        <v>Belmont</v>
       </c>
       <c r="H42" t="str">
-        <v>B</v>
+        <v>B+</v>
       </c>
       <c r="I42" t="str">
         <v>assigned</v>
@@ -2086,27 +2089,27 @@
         <v>Solo</v>
       </c>
     </row>
-    <row r="43" xml:space="preserve">
+    <row r="43">
       <c r="A43" t="str">
-        <v>37fadce4-5d89-4542-a6e1-5e3e50620b85</v>
+        <v>441f345e-57a2-403b-a9a9-8284261eba7b</v>
       </c>
       <c r="B43" t="str">
-        <v>Sharyn  McKinnis</v>
+        <v>Kadisha  Bruton</v>
       </c>
       <c r="C43">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="D43" t="str">
         <v>Female</v>
       </c>
       <c r="E43" t="str">
-        <v>s.lmckinnis@bigpond.com</v>
+        <v>kadishaann@icloud.com</v>
       </c>
       <c r="F43" t="str">
-        <v>419880873</v>
+        <v>434829249</v>
       </c>
       <c r="G43" t="str">
-        <v>Newtown</v>
+        <v xml:space="preserve">Kurunjang </v>
       </c>
       <c r="H43" t="str">
         <v>B+</v>
@@ -2114,70 +2117,67 @@
       <c r="I43" t="str">
         <v>available</v>
       </c>
-      <c r="J43" t="str" xml:space="preserve">
+      <c r="J43" t="str">
+        <v>Jacob Steele</v>
+      </c>
+    </row>
+    <row r="44" xml:space="preserve">
+      <c r="A44" t="str">
+        <v>37fadce4-5d89-4542-a6e1-5e3e50620b85</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Sharyn  McKinnis</v>
+      </c>
+      <c r="C44">
+        <v>50</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E44" t="str">
+        <v>s.lmckinnis@bigpond.com</v>
+      </c>
+      <c r="F44" t="str">
+        <v>419880873</v>
+      </c>
+      <c r="G44" t="str">
+        <v>Newtown</v>
+      </c>
+      <c r="H44" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I44" t="str">
+        <v>available</v>
+      </c>
+      <c r="J44" t="str" xml:space="preserve">
         <v xml:space="preserve">Isabelle McKinnis, Sharyn McKinnis
 </v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="str">
-        <v>917bd31e-7781-44cc-936c-980cb1f844aa</v>
-      </c>
-      <c r="B44" t="str">
-        <v>Angela Verspay</v>
-      </c>
-      <c r="C44">
-        <v>45</v>
-      </c>
-      <c r="D44" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E44" t="str">
-        <v>angelarileysmyth@hotmail.com</v>
-      </c>
-      <c r="F44" t="str">
-        <v>477660119</v>
-      </c>
-      <c r="G44" t="str">
-        <v>Warrnambool</v>
-      </c>
-      <c r="H44" t="str">
-        <v>B</v>
-      </c>
-      <c r="I44" t="str">
-        <v>assigned</v>
-      </c>
-      <c r="J44" t="str">
-        <v>SOLO</v>
-      </c>
-      <c r="M44" t="str">
-        <v>NA</v>
-      </c>
-    </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>c60666dd-e08c-4aa0-8582-4e7a3ad280f8</v>
+        <v>646d2ff7-803b-4c80-bdd6-09d44eec6929</v>
       </c>
       <c r="B45" t="str">
-        <v>Bashar Mona</v>
+        <v>Leanne Bryant</v>
       </c>
       <c r="C45">
-        <v>33</v>
+        <v>63</v>
       </c>
       <c r="D45" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E45" t="str">
-        <v>bashar.mona92@gmail.com</v>
+        <v>blazeandcougar@gmail.com</v>
       </c>
       <c r="F45" t="str">
-        <v>490871416</v>
+        <v>61415438228</v>
       </c>
       <c r="G45" t="str">
-        <v>Roxburgh park</v>
+        <v xml:space="preserve">Hampton Park </v>
       </c>
       <c r="H45" t="str">
-        <v>B+</v>
+        <v>B</v>
       </c>
       <c r="I45" t="str">
         <v>assigned</v>
@@ -2390,7 +2390,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2420,7 +2420,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>57d358cb-d720-4484-8903-846208a88129</v>
+        <v>9b1755ab-387a-460f-adf3-45b9fddc11fd</v>
       </c>
       <c r="B2" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
@@ -2432,12 +2432,12 @@
         <v>1</v>
       </c>
       <c r="E2" t="str">
-        <v>A3</v>
+        <v>A1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>90a868f7-87c2-4b18-888a-1b0729aafd57</v>
+        <v>86c92277-1eb6-4579-800f-d1569c0254b3</v>
       </c>
       <c r="B3" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
@@ -2449,131 +2449,165 @@
         <v>1</v>
       </c>
       <c r="E3" t="str">
-        <v>A4</v>
+        <v>A2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>f569744b-ca7b-46c3-b54f-b206d35d07d0</v>
+        <v>9f6a0125-b8ba-43db-a2a1-afac55ddf6e8</v>
       </c>
       <c r="B4" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C4" t="str">
-        <v>614641dd-4e94-4c42-a1d9-db37c608dcbe</v>
+        <v>7fc083f6-6be3-42bf-b4e5-fc6412e1c559</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
       <c r="E4" t="str">
-        <v>A5</v>
+        <v>A3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>19fd7f06-6147-4090-b47d-4769aeb855ce</v>
+        <v>83af9978-0312-4c27-8d18-8d049ea42655</v>
       </c>
       <c r="B5" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C5" t="str">
-        <v>e4a52d0d-9c54-4504-8a0f-85845cd88e27</v>
+        <v>54de1dd9-b7eb-489d-b4a1-8b3744a385c4</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
       <c r="E5" t="str">
-        <v>B1</v>
+        <v>A4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>01417c60-8dda-4286-a14c-ec8309236d41</v>
+        <v>3b00db5a-6d9a-4a93-a960-aaabe789f4f7</v>
       </c>
       <c r="B6" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C6" t="str">
-        <v>96c75db9-b001-4abe-8ddb-d5a73cb04529</v>
+        <v>e4a52d0d-9c54-4504-8a0f-85845cd88e27</v>
       </c>
       <c r="D6">
         <v>1</v>
       </c>
       <c r="E6" t="str">
-        <v>B4</v>
+        <v>A5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>7d428f41-6701-460f-8c5e-fcf5f9f1e673</v>
+        <v>99a23277-750a-4b95-a5ac-09f1fe6151c6</v>
       </c>
       <c r="B7" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C7" t="str">
-        <v>646d2ff7-803b-4c80-bdd6-09d44eec6929</v>
+        <v>96c75db9-b001-4abe-8ddb-d5a73cb04529</v>
       </c>
       <c r="D7">
         <v>1</v>
       </c>
       <c r="E7" t="str">
-        <v>B5</v>
+        <v>B1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2b9aa451-0238-45e5-96cd-ebd805d71c7b</v>
+        <v>fe0a3a15-8530-43f2-9d77-806462029506</v>
       </c>
       <c r="B8" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C8" t="str">
-        <v>917bd31e-7781-44cc-936c-980cb1f844aa</v>
+        <v>614641dd-4e94-4c42-a1d9-db37c608dcbe</v>
       </c>
       <c r="D8">
         <v>1</v>
       </c>
       <c r="E8" t="str">
-        <v>C1</v>
+        <v>B2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>3c5d1dfd-7f7d-4eec-b21f-5596ec0c9e4a</v>
+        <v>2ee524eb-d4b2-4297-bc94-bf79bc90fc39</v>
       </c>
       <c r="B9" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C9" t="str">
-        <v>c60666dd-e08c-4aa0-8582-4e7a3ad280f8</v>
+        <v>45c7f69f-dd89-41d8-b7f0-a83f77fa9d12</v>
       </c>
       <c r="D9">
         <v>1</v>
       </c>
       <c r="E9" t="str">
-        <v>C2</v>
+        <v>B3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>51037cc9-d563-444d-91e7-4c94330a4d63</v>
+        <v>43336515-ba8a-43ea-ac49-7c4a2bcac7d2</v>
       </c>
       <c r="B10" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C10" t="str">
-        <v>45c7f69f-dd89-41d8-b7f0-a83f77fa9d12</v>
+        <v>646d2ff7-803b-4c80-bdd6-09d44eec6929</v>
       </c>
       <c r="D10">
         <v>1</v>
       </c>
       <c r="E10" t="str">
-        <v>C3</v>
+        <v>B4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>759931ad-4413-4ca1-8dc6-d240e042cfb1</v>
+      </c>
+      <c r="B11" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C11" t="str">
+        <v>c60666dd-e08c-4aa0-8582-4e7a3ad280f8</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11" t="str">
+        <v>B5</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>a1bf8297-f865-4bc4-acb3-0900a2992ff9</v>
+      </c>
+      <c r="B12" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C12" t="str">
+        <v>917bd31e-7781-44cc-936c-980cb1f844aa</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12" t="str">
+        <v>C1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H12"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add functionality to delete all contestants with multiple confirmations
Implement a "Delete All" button on the contestants tab that triggers a two-step confirmation process before initiating a backend DELETE request to `/api/contestants/all`. This endpoint efficiently bulk-deletes all related data including seat assignments, standby bookings, and availability records using direct database operations.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: f123b9d7-6af8-472a-a75c-70d0b78d0583
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 0d45ead9-a484-4c97-b706-b7f1ae847a02
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/4ca2a1f8-42ce-4303-beff-eb92e3283d4c/f123b9d7-6af8-472a-a75c-70d0b78d0583/SA70FQN
</commit_message>
<xml_diff>
--- a/storage/backups/automatic-backup.xlsx
+++ b/storage/backups/automatic-backup.xlsx
@@ -742,6 +742,9 @@
         <v xml:space="preserve">Meenakshi Mehra
 Dhananjay Mehra</v>
       </c>
+      <c r="K2" t="str">
+        <v>8c760df8-0e51-4b27-b1cb-0754c8b03595</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -915,181 +918,181 @@
         <v>No</v>
       </c>
     </row>
-    <row r="8" xml:space="preserve">
+    <row r="8">
       <c r="A8" t="str">
+        <v>6b9ae7f0-4a81-4dda-8e55-e49415d98ec6</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Tayla Huxtable</v>
+      </c>
+      <c r="C8">
+        <v>28</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Taylahuxtable@gmail.com</v>
+      </c>
+      <c r="F8" t="str">
+        <v>435320280</v>
+      </c>
+      <c r="G8" t="str">
+        <v>FERNTREE GULLY</v>
+      </c>
+      <c r="I8" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Troy Smith</v>
+      </c>
+      <c r="K8" t="str">
+        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>b1fc34e8-20cb-4607-9568-0761cf4520a6</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Troy Smith</v>
+      </c>
+      <c r="C9">
+        <v>31</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Troyssmith94@gmail.com</v>
+      </c>
+      <c r="F9" t="str">
+        <v>429354308</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Melbourne</v>
+      </c>
+      <c r="H9" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I9" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="J9" t="str">
+        <v>Tayla Huxtable</v>
+      </c>
+      <c r="K9" t="str">
+        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
+      </c>
+      <c r="L9" t="str">
+        <v xml:space="preserve">Peanut allergy </v>
+      </c>
+      <c r="M9" t="str">
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10" t="str">
         <v>1fe25fd6-dc69-4d29-b22f-9a15ad3d457f</v>
       </c>
-      <c r="B8" t="str">
+      <c r="B10" t="str">
         <v>Sharon King</v>
       </c>
-      <c r="C8">
+      <c r="C10">
         <v>58</v>
       </c>
-      <c r="D8" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E8" t="str">
+      <c r="D10" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E10" t="str">
         <v>dreamweaversixtyseven@gmail.com</v>
       </c>
-      <c r="F8" t="str">
+      <c r="F10" t="str">
         <v>611488000000</v>
       </c>
-      <c r="G8" t="str">
+      <c r="G10" t="str">
         <v xml:space="preserve">Mooroopna </v>
       </c>
-      <c r="H8" t="str">
+      <c r="H10" t="str">
         <v>A</v>
       </c>
-      <c r="I8" t="str">
-        <v>available</v>
-      </c>
-      <c r="J8" t="str" xml:space="preserve">
+      <c r="I10" t="str">
+        <v>available</v>
+      </c>
+      <c r="J10" t="str" xml:space="preserve">
         <v xml:space="preserve">
 Friend :Jacinda Austin
 ID:b6042a-1-1936475</v>
       </c>
-      <c r="M8" t="str">
+      <c r="M10" t="str">
         <v xml:space="preserve">No </v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>82960b61-d36b-49e2-9ddf-a7b8e0b02a63</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Tara Saltzman</v>
-      </c>
-      <c r="C9">
-        <v>29</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E9" t="str">
-        <v>tarasaltzman@bigpond.com</v>
-      </c>
-      <c r="F9" t="str">
-        <v>448545599</v>
-      </c>
-      <c r="G9" t="str">
-        <v>Melbourne</v>
-      </c>
-      <c r="H9" t="str">
-        <v>B+</v>
-      </c>
-      <c r="I9" t="str">
-        <v>available</v>
-      </c>
-      <c r="J9" t="str">
-        <v xml:space="preserve">JACK AGIUS - NEEDS TO DO APPLICATION </v>
-      </c>
-      <c r="M9" t="str">
-        <v>NA</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>f693566d-ea7c-40d1-89aa-158e842961d0</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Brent Barnett</v>
-      </c>
-      <c r="C10">
-        <v>37</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Male</v>
-      </c>
-      <c r="E10" t="str">
-        <v>brentbarnett88@gmail.com</v>
-      </c>
-      <c r="F10" t="str">
-        <v>423530043</v>
-      </c>
-      <c r="G10" t="str">
-        <v>Preston</v>
-      </c>
-      <c r="H10" t="str">
-        <v>B+</v>
-      </c>
-      <c r="I10" t="str">
-        <v>available</v>
-      </c>
-      <c r="J10" t="str">
-        <v>Stephanie Squillacioti</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>6b9ae7f0-4a81-4dda-8e55-e49415d98ec6</v>
+        <v>82960b61-d36b-49e2-9ddf-a7b8e0b02a63</v>
       </c>
       <c r="B11" t="str">
-        <v>Tayla Huxtable</v>
+        <v>Tara Saltzman</v>
       </c>
       <c r="C11">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D11" t="str">
         <v>Female</v>
       </c>
       <c r="E11" t="str">
-        <v>Taylahuxtable@gmail.com</v>
+        <v>tarasaltzman@bigpond.com</v>
       </c>
       <c r="F11" t="str">
-        <v>435320280</v>
+        <v>448545599</v>
       </c>
       <c r="G11" t="str">
-        <v>FERNTREE GULLY</v>
+        <v>Melbourne</v>
+      </c>
+      <c r="H11" t="str">
+        <v>B+</v>
       </c>
       <c r="I11" t="str">
-        <v>assigned</v>
+        <v>available</v>
       </c>
       <c r="J11" t="str">
-        <v>Troy Smith</v>
-      </c>
-      <c r="K11" t="str">
-        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
+        <v xml:space="preserve">JACK AGIUS - NEEDS TO DO APPLICATION </v>
+      </c>
+      <c r="M11" t="str">
+        <v>NA</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>b1fc34e8-20cb-4607-9568-0761cf4520a6</v>
+        <v>f693566d-ea7c-40d1-89aa-158e842961d0</v>
       </c>
       <c r="B12" t="str">
-        <v>Troy Smith</v>
+        <v>Brent Barnett</v>
       </c>
       <c r="C12">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D12" t="str">
         <v>Male</v>
       </c>
       <c r="E12" t="str">
-        <v>Troyssmith94@gmail.com</v>
+        <v>brentbarnett88@gmail.com</v>
       </c>
       <c r="F12" t="str">
-        <v>429354308</v>
+        <v>423530043</v>
       </c>
       <c r="G12" t="str">
-        <v>Melbourne</v>
+        <v>Preston</v>
       </c>
       <c r="H12" t="str">
         <v>B+</v>
       </c>
       <c r="I12" t="str">
-        <v>assigned</v>
+        <v>available</v>
       </c>
       <c r="J12" t="str">
-        <v>Tayla Huxtable</v>
-      </c>
-      <c r="K12" t="str">
-        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
-      </c>
-      <c r="L12" t="str">
-        <v xml:space="preserve">Peanut allergy </v>
-      </c>
-      <c r="M12" t="str">
-        <v>NA</v>
+        <v>Stephanie Squillacioti</v>
       </c>
     </row>
     <row r="13">
@@ -1291,25 +1294,25 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>e4a52d0d-9c54-4504-8a0f-85845cd88e27</v>
+        <v>96c75db9-b001-4abe-8ddb-d5a73cb04529</v>
       </c>
       <c r="B19" t="str">
-        <v>David Fenwick</v>
+        <v>Kiran Rao</v>
       </c>
       <c r="C19">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D19" t="str">
         <v>Male</v>
       </c>
       <c r="E19" t="str">
-        <v>David.s.fenwick@gmail.com</v>
+        <v>kiran.rao07@gmail.com</v>
       </c>
       <c r="F19" t="str">
-        <v>429811171</v>
+        <v>420486042</v>
       </c>
       <c r="G19" t="str">
-        <v>Teesdale</v>
+        <v>Southbank</v>
       </c>
       <c r="H19" t="str">
         <v>B+</v>
@@ -1318,7 +1321,10 @@
         <v>assigned</v>
       </c>
       <c r="J19" t="str">
-        <v>Solo</v>
+        <v>SOLO</v>
+      </c>
+      <c r="M19" t="str">
+        <v>NA</v>
       </c>
     </row>
     <row r="20">
@@ -1554,25 +1560,25 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>96c75db9-b001-4abe-8ddb-d5a73cb04529</v>
+        <v>e4a52d0d-9c54-4504-8a0f-85845cd88e27</v>
       </c>
       <c r="B27" t="str">
-        <v>Kiran Rao</v>
+        <v>David Fenwick</v>
       </c>
       <c r="C27">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D27" t="str">
         <v>Male</v>
       </c>
       <c r="E27" t="str">
-        <v>kiran.rao07@gmail.com</v>
+        <v>David.s.fenwick@gmail.com</v>
       </c>
       <c r="F27" t="str">
-        <v>420486042</v>
+        <v>429811171</v>
       </c>
       <c r="G27" t="str">
-        <v>Southbank</v>
+        <v>Teesdale</v>
       </c>
       <c r="H27" t="str">
         <v>B+</v>
@@ -1581,10 +1587,7 @@
         <v>assigned</v>
       </c>
       <c r="J27" t="str">
-        <v>SOLO</v>
-      </c>
-      <c r="M27" t="str">
-        <v>NA</v>
+        <v>Solo</v>
       </c>
     </row>
     <row r="28" xml:space="preserve">
@@ -1789,28 +1792,28 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>c60666dd-e08c-4aa0-8582-4e7a3ad280f8</v>
+        <v>646d2ff7-803b-4c80-bdd6-09d44eec6929</v>
       </c>
       <c r="B34" t="str">
-        <v>Bashar Mona</v>
+        <v>Leanne Bryant</v>
       </c>
       <c r="C34">
-        <v>33</v>
+        <v>63</v>
       </c>
       <c r="D34" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E34" t="str">
-        <v>bashar.mona92@gmail.com</v>
+        <v>blazeandcougar@gmail.com</v>
       </c>
       <c r="F34" t="str">
-        <v>490871416</v>
+        <v>61415438228</v>
       </c>
       <c r="G34" t="str">
-        <v>Roxburgh park</v>
+        <v xml:space="preserve">Hampton Park </v>
       </c>
       <c r="H34" t="str">
-        <v>B+</v>
+        <v>B</v>
       </c>
       <c r="I34" t="str">
         <v>assigned</v>
@@ -1885,103 +1888,102 @@
 Aidan Miler</v>
       </c>
     </row>
-    <row r="37" xml:space="preserve">
+    <row r="37">
       <c r="A37" t="str">
+        <v>c60666dd-e08c-4aa0-8582-4e7a3ad280f8</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Bashar Mona</v>
+      </c>
+      <c r="C37">
+        <v>33</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E37" t="str">
+        <v>bashar.mona92@gmail.com</v>
+      </c>
+      <c r="F37" t="str">
+        <v>490871416</v>
+      </c>
+      <c r="G37" t="str">
+        <v>Roxburgh park</v>
+      </c>
+      <c r="H37" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I37" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="J37" t="str">
+        <v>Solo</v>
+      </c>
+    </row>
+    <row r="38" xml:space="preserve">
+      <c r="A38" t="str">
         <v>1211456d-ea92-4a7b-9d94-885982cf345c</v>
       </c>
-      <c r="B37" t="str">
+      <c r="B38" t="str">
         <v>Bronwyn Parsons</v>
       </c>
-      <c r="C37">
+      <c r="C38">
         <v>72</v>
       </c>
-      <c r="D37" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E37" t="str">
+      <c r="D38" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E38" t="str">
         <v>Babybear61153@gmail.com</v>
       </c>
-      <c r="F37" t="str">
+      <c r="F38" t="str">
         <v>432543647</v>
       </c>
-      <c r="G37" t="str">
+      <c r="G38" t="str">
         <v>Rosebud</v>
       </c>
-      <c r="H37" t="str">
+      <c r="H38" t="str">
         <v>A+</v>
       </c>
-      <c r="I37" t="str">
-        <v>available</v>
-      </c>
-      <c r="J37" t="str" xml:space="preserve">
+      <c r="I38" t="str">
+        <v>available</v>
+      </c>
+      <c r="J38" t="str" xml:space="preserve">
         <v xml:space="preserve">Yolette Huon - yol-et Hue on
 Bronwyn Parsons - Would like to be called Bron Emmerson - maiden name</v>
       </c>
     </row>
-    <row r="38" xml:space="preserve">
-      <c r="A38" t="str">
+    <row r="39" xml:space="preserve">
+      <c r="A39" t="str">
         <v>23f118f9-20db-422c-8cef-939dc73dd803</v>
       </c>
-      <c r="B38" t="str">
+      <c r="B39" t="str">
         <v>Paige Greig</v>
       </c>
-      <c r="C38">
+      <c r="C39">
         <v>31</v>
       </c>
-      <c r="D38" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E38" t="str">
+      <c r="D39" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E39" t="str">
         <v>paigegreig@hotmail.com</v>
       </c>
-      <c r="F38" t="str">
+      <c r="F39" t="str">
         <v>406598552</v>
       </c>
-      <c r="G38" t="str">
+      <c r="G39" t="str">
         <v>Mooroolbark</v>
       </c>
-      <c r="H38" t="str">
+      <c r="H39" t="str">
         <v>C</v>
       </c>
-      <c r="I38" t="str">
-        <v>available</v>
-      </c>
-      <c r="J38" t="str" xml:space="preserve">
+      <c r="I39" t="str">
+        <v>available</v>
+      </c>
+      <c r="J39" t="str" xml:space="preserve">
         <v xml:space="preserve">Erin
 Morgan (sister) - need to do application</v>
-      </c>
-    </row>
-    <row r="39" xml:space="preserve">
-      <c r="A39" t="str">
-        <v>54de1dd9-b7eb-489d-b4a1-8b3744a385c4</v>
-      </c>
-      <c r="B39" t="str">
-        <v>Dhananjay  Mehra</v>
-      </c>
-      <c r="C39">
-        <v>68</v>
-      </c>
-      <c r="D39" t="str">
-        <v>Male</v>
-      </c>
-      <c r="E39" t="str">
-        <v>Dmehra@bigpond.net.au</v>
-      </c>
-      <c r="F39" t="str">
-        <v>419353328</v>
-      </c>
-      <c r="G39" t="str">
-        <v xml:space="preserve">Point Cook </v>
-      </c>
-      <c r="H39" t="str">
-        <v>B</v>
-      </c>
-      <c r="I39" t="str">
-        <v>assigned</v>
-      </c>
-      <c r="J39" t="str" xml:space="preserve">
-        <v xml:space="preserve">Meenakshi Mehra
-Dhananjay Mehra</v>
       </c>
     </row>
     <row r="40">
@@ -2057,36 +2059,40 @@
         <v>NA</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" xml:space="preserve">
       <c r="A42" t="str">
-        <v>45c7f69f-dd89-41d8-b7f0-a83f77fa9d12</v>
+        <v>54de1dd9-b7eb-489d-b4a1-8b3744a385c4</v>
       </c>
       <c r="B42" t="str">
-        <v>Sherif Haggag</v>
+        <v>Dhananjay  Mehra</v>
       </c>
       <c r="C42">
-        <v>38</v>
+        <v>68</v>
       </c>
       <c r="D42" t="str">
         <v>Male</v>
       </c>
       <c r="E42" t="str">
-        <v>Shaggag87@gmail.com</v>
+        <v>Dmehra@bigpond.net.au</v>
       </c>
       <c r="F42" t="str">
-        <v>426233449</v>
+        <v>419353328</v>
       </c>
       <c r="G42" t="str">
-        <v>Belmont</v>
+        <v xml:space="preserve">Point Cook </v>
       </c>
       <c r="H42" t="str">
-        <v>B+</v>
+        <v>B</v>
       </c>
       <c r="I42" t="str">
         <v>assigned</v>
       </c>
-      <c r="J42" t="str">
-        <v>Solo</v>
+      <c r="J42" t="str" xml:space="preserve">
+        <v xml:space="preserve">Meenakshi Mehra
+Dhananjay Mehra</v>
+      </c>
+      <c r="K42" t="str">
+        <v>8c760df8-0e51-4b27-b1cb-0754c8b03595</v>
       </c>
     </row>
     <row r="43">
@@ -2156,28 +2162,28 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>646d2ff7-803b-4c80-bdd6-09d44eec6929</v>
+        <v>45c7f69f-dd89-41d8-b7f0-a83f77fa9d12</v>
       </c>
       <c r="B45" t="str">
-        <v>Leanne Bryant</v>
+        <v>Sherif Haggag</v>
       </c>
       <c r="C45">
-        <v>63</v>
+        <v>38</v>
       </c>
       <c r="D45" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E45" t="str">
-        <v>blazeandcougar@gmail.com</v>
+        <v>Shaggag87@gmail.com</v>
       </c>
       <c r="F45" t="str">
-        <v>61415438228</v>
+        <v>426233449</v>
       </c>
       <c r="G45" t="str">
-        <v xml:space="preserve">Hampton Park </v>
+        <v>Belmont</v>
       </c>
       <c r="H45" t="str">
-        <v>B</v>
+        <v>B+</v>
       </c>
       <c r="I45" t="str">
         <v>assigned</v>
@@ -2420,7 +2426,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>9b1755ab-387a-460f-adf3-45b9fddc11fd</v>
+        <v>cbb914d8-4355-4eae-8e6a-d916e6eeab9c</v>
       </c>
       <c r="B2" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
@@ -2437,7 +2443,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>86c92277-1eb6-4579-800f-d1569c0254b3</v>
+        <v>72ec2db4-7ad6-48e7-aada-ebcd77e964de</v>
       </c>
       <c r="B3" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
@@ -2454,7 +2460,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>9f6a0125-b8ba-43db-a2a1-afac55ddf6e8</v>
+        <v>3c715c30-77ec-4327-a1dc-77e587684309</v>
       </c>
       <c r="B4" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
@@ -2471,7 +2477,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>83af9978-0312-4c27-8d18-8d049ea42655</v>
+        <v>98131f5a-2b3c-46c8-876a-215c01d25450</v>
       </c>
       <c r="B5" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
@@ -2488,7 +2494,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>3b00db5a-6d9a-4a93-a960-aaabe789f4f7</v>
+        <v>cd4bdfd0-1ea2-465c-9a88-0c4e8be41c46</v>
       </c>
       <c r="B6" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
@@ -2505,13 +2511,13 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>99a23277-750a-4b95-a5ac-09f1fe6151c6</v>
+        <v>e3f866e4-5581-4731-8857-0d4dad4cee98</v>
       </c>
       <c r="B7" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C7" t="str">
-        <v>96c75db9-b001-4abe-8ddb-d5a73cb04529</v>
+        <v>614641dd-4e94-4c42-a1d9-db37c608dcbe</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -2522,13 +2528,13 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>fe0a3a15-8530-43f2-9d77-806462029506</v>
+        <v>525e206b-a4dc-4cb0-bb8d-350087facf3e</v>
       </c>
       <c r="B8" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C8" t="str">
-        <v>614641dd-4e94-4c42-a1d9-db37c608dcbe</v>
+        <v>96c75db9-b001-4abe-8ddb-d5a73cb04529</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -2539,7 +2545,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2ee524eb-d4b2-4297-bc94-bf79bc90fc39</v>
+        <v>8d7a05d2-98e8-40f7-b7ff-a8b4cbbfcb46</v>
       </c>
       <c r="B9" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
@@ -2556,7 +2562,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>43336515-ba8a-43ea-ac49-7c4a2bcac7d2</v>
+        <v>8d8eddd8-180f-4a64-af6b-a1e848b325b0</v>
       </c>
       <c r="B10" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
@@ -2573,7 +2579,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>759931ad-4413-4ca1-8dc6-d240e042cfb1</v>
+        <v>0b61d3fc-daf3-492d-b9a1-6070b61f0235</v>
       </c>
       <c r="B11" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
@@ -2590,7 +2596,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>a1bf8297-f865-4bc4-acb3-0900a2992ff9</v>
+        <v>cd6ab2c2-d134-4f10-95c6-caa3b4590d32</v>
       </c>
       <c r="B12" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
@@ -2602,7 +2608,7 @@
         <v>1</v>
       </c>
       <c r="E12" t="str">
-        <v>C1</v>
+        <v>D1</v>
       </c>
     </row>
   </sheetData>
@@ -2614,7 +2620,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2640,9 +2646,17 @@
         <v>GRP002</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>8c760df8-0e51-4b27-b1cb-0754c8b03595</v>
+      </c>
+      <c r="B4" t="str">
+        <v>AUTO-MK2NF2KE-kuoa</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Improve contestant grouping and attendance parsing logic
Refactors the server routes to utilize a shared parsing utility for the `attendingWith` field, improving consistency and robustness in group assignment and solo contestant detection.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: f123b9d7-6af8-472a-a75c-70d0b78d0583
Replit-Commit-Checkpoint-Type: intermediate_checkpoint
Replit-Commit-Event-Id: 45b25c95-4c56-437e-9e94-a8dee06e5386
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/4ca2a1f8-42ce-4303-beff-eb92e3283d4c/f123b9d7-6af8-472a-a75c-70d0b78d0583/SA70FQN
</commit_message>
<xml_diff>
--- a/storage/backups/automatic-backup.xlsx
+++ b/storage/backups/automatic-backup.xlsx
@@ -5,9 +5,8 @@
   <sheets>
     <sheet name="Record Days" sheetId="1" r:id="rId1"/>
     <sheet name="Contestants" sheetId="2" r:id="rId2"/>
-    <sheet name="Seat Assignments" sheetId="3" r:id="rId3"/>
-    <sheet name="Groups" sheetId="4" r:id="rId4"/>
-    <sheet name="Block Types" sheetId="5" r:id="rId5"/>
+    <sheet name="Groups" sheetId="3" r:id="rId3"/>
+    <sheet name="Block Types" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -736,7 +735,7 @@
         <v>B</v>
       </c>
       <c r="I2" t="str">
-        <v>assigned</v>
+        <v>available</v>
       </c>
       <c r="J2" t="str" xml:space="preserve">
         <v xml:space="preserve">Meenakshi Mehra
@@ -920,75 +919,75 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>6b9ae7f0-4a81-4dda-8e55-e49415d98ec6</v>
+        <v>b1fc34e8-20cb-4607-9568-0761cf4520a6</v>
       </c>
       <c r="B8" t="str">
+        <v>Troy Smith</v>
+      </c>
+      <c r="C8">
+        <v>31</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Troyssmith94@gmail.com</v>
+      </c>
+      <c r="F8" t="str">
+        <v>429354308</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Melbourne</v>
+      </c>
+      <c r="H8" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I8" t="str">
+        <v>available</v>
+      </c>
+      <c r="J8" t="str">
         <v>Tayla Huxtable</v>
-      </c>
-      <c r="C8">
-        <v>28</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Taylahuxtable@gmail.com</v>
-      </c>
-      <c r="F8" t="str">
-        <v>435320280</v>
-      </c>
-      <c r="G8" t="str">
-        <v>FERNTREE GULLY</v>
-      </c>
-      <c r="I8" t="str">
-        <v>assigned</v>
-      </c>
-      <c r="J8" t="str">
-        <v>Troy Smith</v>
       </c>
       <c r="K8" t="str">
         <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
       </c>
+      <c r="L8" t="str">
+        <v xml:space="preserve">Peanut allergy </v>
+      </c>
+      <c r="M8" t="str">
+        <v>NA</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>b1fc34e8-20cb-4607-9568-0761cf4520a6</v>
+        <v>6b9ae7f0-4a81-4dda-8e55-e49415d98ec6</v>
       </c>
       <c r="B9" t="str">
+        <v>Tayla Huxtable</v>
+      </c>
+      <c r="C9">
+        <v>28</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Taylahuxtable@gmail.com</v>
+      </c>
+      <c r="F9" t="str">
+        <v>435320280</v>
+      </c>
+      <c r="G9" t="str">
+        <v>FERNTREE GULLY</v>
+      </c>
+      <c r="I9" t="str">
+        <v>available</v>
+      </c>
+      <c r="J9" t="str">
         <v>Troy Smith</v>
-      </c>
-      <c r="C9">
-        <v>31</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Male</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Troyssmith94@gmail.com</v>
-      </c>
-      <c r="F9" t="str">
-        <v>429354308</v>
-      </c>
-      <c r="G9" t="str">
-        <v>Melbourne</v>
-      </c>
-      <c r="H9" t="str">
-        <v>B+</v>
-      </c>
-      <c r="I9" t="str">
-        <v>assigned</v>
-      </c>
-      <c r="J9" t="str">
-        <v>Tayla Huxtable</v>
       </c>
       <c r="K9" t="str">
         <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
-      </c>
-      <c r="L9" t="str">
-        <v xml:space="preserve">Peanut allergy </v>
-      </c>
-      <c r="M9" t="str">
-        <v>NA</v>
       </c>
     </row>
     <row r="10" xml:space="preserve">
@@ -1294,193 +1293,190 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>96c75db9-b001-4abe-8ddb-d5a73cb04529</v>
+        <v>1bc7d8fc-def3-4f9f-8376-80b79696d1a5</v>
       </c>
       <c r="B19" t="str">
-        <v>Kiran Rao</v>
+        <v>Eden Hayes</v>
       </c>
       <c r="C19">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="D19" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E19" t="str">
-        <v>kiran.rao07@gmail.com</v>
+        <v>edenhayes19@gmail.com</v>
       </c>
       <c r="F19" t="str">
-        <v>420486042</v>
+        <v>448096139</v>
       </c>
       <c r="G19" t="str">
-        <v>Southbank</v>
+        <v>Elwood</v>
       </c>
       <c r="H19" t="str">
         <v>B+</v>
       </c>
       <c r="I19" t="str">
-        <v>assigned</v>
+        <v>available</v>
       </c>
       <c r="J19" t="str">
-        <v>SOLO</v>
-      </c>
-      <c r="M19" t="str">
-        <v>NA</v>
+        <v>Jackson Harris</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>1bc7d8fc-def3-4f9f-8376-80b79696d1a5</v>
+        <v>419afd3f-2406-423d-942f-2dfafe875f96</v>
       </c>
       <c r="B20" t="str">
-        <v>Eden Hayes</v>
+        <v>Anna Fonua</v>
       </c>
       <c r="C20">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="D20" t="str">
         <v>Female</v>
       </c>
       <c r="E20" t="str">
-        <v>edenhayes19@gmail.com</v>
+        <v>Annawallace89@hotmail.com</v>
       </c>
       <c r="F20" t="str">
-        <v>448096139</v>
+        <v>452452442</v>
       </c>
       <c r="G20" t="str">
-        <v>Elwood</v>
+        <v>Truganina</v>
       </c>
       <c r="H20" t="str">
+        <v>A</v>
+      </c>
+      <c r="I20" t="str">
+        <v>available</v>
+      </c>
+      <c r="J20" t="str">
+        <v>Dad Michael Wallace - b6042a-1-1936372</v>
+      </c>
+      <c r="M20" t="str">
+        <v xml:space="preserve">no </v>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str">
+        <v>d9b76f1c-0867-44fc-9215-6ef7b1184af6</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Kayla Lorenzini</v>
+      </c>
+      <c r="C21">
+        <v>29</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E21" t="str">
+        <v>kaylalorenzini_@hotmail.com</v>
+      </c>
+      <c r="F21" t="str">
+        <v>430517653</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Melbourne</v>
+      </c>
+      <c r="H21" t="str">
         <v>B+</v>
       </c>
-      <c r="I20" t="str">
-        <v>available</v>
-      </c>
-      <c r="J20" t="str">
-        <v>Jackson Harris</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>419afd3f-2406-423d-942f-2dfafe875f96</v>
-      </c>
-      <c r="B21" t="str">
-        <v>Anna Fonua</v>
-      </c>
-      <c r="C21">
-        <v>36</v>
-      </c>
-      <c r="D21" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E21" t="str">
-        <v>Annawallace89@hotmail.com</v>
-      </c>
-      <c r="F21" t="str">
-        <v>452452442</v>
-      </c>
-      <c r="G21" t="str">
-        <v>Truganina</v>
-      </c>
-      <c r="H21" t="str">
-        <v>A</v>
-      </c>
       <c r="I21" t="str">
         <v>available</v>
       </c>
-      <c r="J21" t="str">
-        <v>Dad Michael Wallace - b6042a-1-1936372</v>
-      </c>
-      <c r="M21" t="str">
-        <v xml:space="preserve">no </v>
-      </c>
-    </row>
-    <row r="22" xml:space="preserve">
-      <c r="A22" t="str">
-        <v>d9b76f1c-0867-44fc-9215-6ef7b1184af6</v>
-      </c>
-      <c r="B22" t="str">
-        <v>Kayla Lorenzini</v>
-      </c>
-      <c r="C22">
-        <v>29</v>
-      </c>
-      <c r="D22" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E22" t="str">
-        <v>kaylalorenzini_@hotmail.com</v>
-      </c>
-      <c r="F22" t="str">
-        <v>430517653</v>
-      </c>
-      <c r="G22" t="str">
-        <v>Melbourne</v>
-      </c>
-      <c r="H22" t="str">
-        <v>B+</v>
-      </c>
-      <c r="I22" t="str">
-        <v>available</v>
-      </c>
-      <c r="J22" t="str" xml:space="preserve">
+      <c r="J21" t="str" xml:space="preserve">
         <v xml:space="preserve">Kayla Lorenzini
 James Lorenzini
 Deanna Gramola</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>f048c8fe-e8c9-4357-8ec8-ef76793e5bc1</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Tamara Mifsud</v>
+      </c>
+      <c r="C22">
+        <v>32</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E22" t="str">
+        <v>tamara.mifsud@hotmail.com</v>
+      </c>
+      <c r="F22" t="str">
+        <v>416552122</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Aintree</v>
+      </c>
+      <c r="H22" t="str">
+        <v>B</v>
+      </c>
+      <c r="I22" t="str">
+        <v>available</v>
+      </c>
+      <c r="J22" t="str">
+        <v>Aliye Abcilar</v>
+      </c>
+    </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>f048c8fe-e8c9-4357-8ec8-ef76793e5bc1</v>
+        <v>6bbdadcb-23a8-41c9-964b-6152e234cb33</v>
       </c>
       <c r="B23" t="str">
-        <v>Tamara Mifsud</v>
+        <v>Philip Natoli</v>
       </c>
       <c r="C23">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D23" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E23" t="str">
-        <v>tamara.mifsud@hotmail.com</v>
+        <v>Philip.natoli@outlook.com</v>
       </c>
       <c r="F23" t="str">
-        <v>416552122</v>
+        <v>466021882</v>
       </c>
       <c r="G23" t="str">
-        <v>Aintree</v>
+        <v>Caulfield South</v>
       </c>
       <c r="H23" t="str">
-        <v>B</v>
+        <v>B+</v>
       </c>
       <c r="I23" t="str">
         <v>available</v>
       </c>
       <c r="J23" t="str">
-        <v>Aliye Abcilar</v>
+        <v>Hayley Wright</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>6bbdadcb-23a8-41c9-964b-6152e234cb33</v>
+        <v>614641dd-4e94-4c42-a1d9-db37c608dcbe</v>
       </c>
       <c r="B24" t="str">
-        <v>Philip Natoli</v>
+        <v>Antonio Freno</v>
       </c>
       <c r="C24">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="D24" t="str">
         <v>Male</v>
       </c>
       <c r="E24" t="str">
-        <v>Philip.natoli@outlook.com</v>
+        <v>frenoantonio@hotmail.it</v>
       </c>
       <c r="F24" t="str">
-        <v>466021882</v>
+        <v>422177371</v>
       </c>
       <c r="G24" t="str">
-        <v>Caulfield South</v>
+        <v>Glenroy</v>
       </c>
       <c r="H24" t="str">
         <v>B+</v>
@@ -1489,7 +1485,7 @@
         <v>available</v>
       </c>
       <c r="J24" t="str">
-        <v>Hayley Wright</v>
+        <v>Solo</v>
       </c>
     </row>
     <row r="25">
@@ -1558,96 +1554,99 @@
 Brothers</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" xml:space="preserve">
       <c r="A27" t="str">
-        <v>e4a52d0d-9c54-4504-8a0f-85845cd88e27</v>
+        <v>15fb53d0-3916-4c9a-9f73-c28c879dec33</v>
       </c>
       <c r="B27" t="str">
-        <v>David Fenwick</v>
+        <v>Mozgda  Alime</v>
       </c>
       <c r="C27">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D27" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E27" t="str">
-        <v>David.s.fenwick@gmail.com</v>
+        <v>smalimi@hotmail.com</v>
       </c>
       <c r="F27" t="str">
-        <v>429811171</v>
+        <v>402010235</v>
       </c>
       <c r="G27" t="str">
-        <v>Teesdale</v>
+        <v xml:space="preserve">Melbourne </v>
       </c>
       <c r="H27" t="str">
-        <v>B+</v>
+        <v>C</v>
       </c>
       <c r="I27" t="str">
-        <v>assigned</v>
-      </c>
-      <c r="J27" t="str">
-        <v>Solo</v>
-      </c>
-    </row>
-    <row r="28" xml:space="preserve">
-      <c r="A28" t="str">
-        <v>15fb53d0-3916-4c9a-9f73-c28c879dec33</v>
-      </c>
-      <c r="B28" t="str">
-        <v>Mozgda  Alime</v>
-      </c>
-      <c r="C28">
-        <v>39</v>
-      </c>
-      <c r="D28" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E28" t="str">
-        <v>smalimi@hotmail.com</v>
-      </c>
-      <c r="F28" t="str">
-        <v>402010235</v>
-      </c>
-      <c r="G28" t="str">
-        <v xml:space="preserve">Melbourne </v>
-      </c>
-      <c r="H28" t="str">
-        <v>C</v>
-      </c>
-      <c r="I28" t="str">
-        <v>available</v>
-      </c>
-      <c r="J28" t="str" xml:space="preserve">
+        <v>available</v>
+      </c>
+      <c r="J27" t="str" xml:space="preserve">
         <v xml:space="preserve">Sadaf Almini - I believe this is her cousin 
 Lida Alime - I believe this is her cousin or sister 
 Ahmad Alime - Ahmad is Lina's husband </v>
       </c>
+      <c r="M27" t="str">
+        <v xml:space="preserve">No </v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>f7b766dc-a0d0-4a91-98ef-47472cdca803</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Mara Baumgardner</v>
+      </c>
+      <c r="C28">
+        <v>40</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Granic@hotmail.com</v>
+      </c>
+      <c r="F28" t="str">
+        <v>407364450</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Cockatoo</v>
+      </c>
+      <c r="H28" t="str">
+        <v>B</v>
+      </c>
+      <c r="I28" t="str">
+        <v>available</v>
+      </c>
+      <c r="J28" t="str">
+        <v xml:space="preserve">Mum - Mira Granic </v>
+      </c>
       <c r="M28" t="str">
         <v xml:space="preserve">No </v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>f7b766dc-a0d0-4a91-98ef-47472cdca803</v>
+        <v>607e3750-92e2-4480-b39d-1cb0e026cd4b</v>
       </c>
       <c r="B29" t="str">
-        <v>Mara Baumgardner</v>
+        <v>Natasha Devers</v>
       </c>
       <c r="C29">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="D29" t="str">
         <v>Female</v>
       </c>
       <c r="E29" t="str">
-        <v>Granic@hotmail.com</v>
+        <v>natashadevers@gmail.com</v>
       </c>
       <c r="F29" t="str">
-        <v>407364450</v>
+        <v>484003770</v>
       </c>
       <c r="G29" t="str">
-        <v>Cockatoo</v>
+        <v xml:space="preserve">Waterways </v>
       </c>
       <c r="H29" t="str">
         <v>B</v>
@@ -1656,74 +1655,74 @@
         <v>available</v>
       </c>
       <c r="J29" t="str">
-        <v xml:space="preserve">Mum - Mira Granic </v>
-      </c>
-      <c r="M29" t="str">
-        <v xml:space="preserve">No </v>
+        <v>Oliver Moran</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>607e3750-92e2-4480-b39d-1cb0e026cd4b</v>
+        <v>e4a52d0d-9c54-4504-8a0f-85845cd88e27</v>
       </c>
       <c r="B30" t="str">
-        <v>Natasha Devers</v>
+        <v>David Fenwick</v>
       </c>
       <c r="C30">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="D30" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E30" t="str">
-        <v>natashadevers@gmail.com</v>
+        <v>David.s.fenwick@gmail.com</v>
       </c>
       <c r="F30" t="str">
-        <v>484003770</v>
+        <v>429811171</v>
       </c>
       <c r="G30" t="str">
-        <v xml:space="preserve">Waterways </v>
+        <v>Teesdale</v>
       </c>
       <c r="H30" t="str">
-        <v>B</v>
+        <v>B+</v>
       </c>
       <c r="I30" t="str">
         <v>available</v>
       </c>
       <c r="J30" t="str">
-        <v>Oliver Moran</v>
+        <v>Solo</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>614641dd-4e94-4c42-a1d9-db37c608dcbe</v>
+        <v>96c75db9-b001-4abe-8ddb-d5a73cb04529</v>
       </c>
       <c r="B31" t="str">
-        <v>Antonio Freno</v>
+        <v>Kiran Rao</v>
       </c>
       <c r="C31">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D31" t="str">
         <v>Male</v>
       </c>
       <c r="E31" t="str">
-        <v>frenoantonio@hotmail.it</v>
+        <v>kiran.rao07@gmail.com</v>
       </c>
       <c r="F31" t="str">
-        <v>422177371</v>
+        <v>420486042</v>
       </c>
       <c r="G31" t="str">
-        <v>Glenroy</v>
+        <v>Southbank</v>
       </c>
       <c r="H31" t="str">
         <v>B+</v>
       </c>
       <c r="I31" t="str">
-        <v>assigned</v>
+        <v>available</v>
       </c>
       <c r="J31" t="str">
-        <v>Solo</v>
+        <v>SOLO</v>
+      </c>
+      <c r="M31" t="str">
+        <v>NA</v>
       </c>
     </row>
     <row r="32">
@@ -1792,129 +1791,130 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>646d2ff7-803b-4c80-bdd6-09d44eec6929</v>
+        <v>2aadb3db-ad8e-4edd-a81d-f045a926ceb9</v>
       </c>
       <c r="B34" t="str">
-        <v>Leanne Bryant</v>
+        <v>Alexander Leonard</v>
       </c>
       <c r="C34">
-        <v>63</v>
+        <v>38</v>
       </c>
       <c r="D34" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E34" t="str">
-        <v>blazeandcougar@gmail.com</v>
+        <v>alexleonardedit@gmail.com</v>
       </c>
       <c r="F34" t="str">
-        <v>61415438228</v>
+        <v>421834476</v>
       </c>
       <c r="G34" t="str">
-        <v xml:space="preserve">Hampton Park </v>
+        <v>Croydon</v>
       </c>
       <c r="H34" t="str">
+        <v>A+</v>
+      </c>
+      <c r="I34" t="str">
+        <v>available</v>
+      </c>
+      <c r="J34" t="str">
+        <v>melissa francis, Alexander Leonard</v>
+      </c>
+    </row>
+    <row r="35" xml:space="preserve">
+      <c r="A35" t="str">
+        <v>ed91813b-2f74-4638-9d1a-ef8c54cff447</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Linda Browne</v>
+      </c>
+      <c r="C35">
+        <v>54</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Lindabrowne@iprimus.com.au</v>
+      </c>
+      <c r="F35" t="str">
+        <v>429570177</v>
+      </c>
+      <c r="G35" t="str">
+        <v>OFFICER</v>
+      </c>
+      <c r="H35" t="str">
         <v>B</v>
       </c>
-      <c r="I34" t="str">
-        <v>assigned</v>
-      </c>
-      <c r="J34" t="str">
-        <v>Solo</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v>2aadb3db-ad8e-4edd-a81d-f045a926ceb9</v>
-      </c>
-      <c r="B35" t="str">
-        <v>Alexander Leonard</v>
-      </c>
-      <c r="C35">
-        <v>38</v>
-      </c>
-      <c r="D35" t="str">
-        <v>Male</v>
-      </c>
-      <c r="E35" t="str">
-        <v>alexleonardedit@gmail.com</v>
-      </c>
-      <c r="F35" t="str">
-        <v>421834476</v>
-      </c>
-      <c r="G35" t="str">
-        <v>Croydon</v>
-      </c>
-      <c r="H35" t="str">
-        <v>A+</v>
-      </c>
       <c r="I35" t="str">
         <v>available</v>
       </c>
-      <c r="J35" t="str">
-        <v>melissa francis, Alexander Leonard</v>
-      </c>
-    </row>
-    <row r="36" xml:space="preserve">
-      <c r="A36" t="str">
-        <v>ed91813b-2f74-4638-9d1a-ef8c54cff447</v>
-      </c>
-      <c r="B36" t="str">
-        <v>Linda Browne</v>
-      </c>
-      <c r="C36">
-        <v>54</v>
-      </c>
-      <c r="D36" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E36" t="str">
-        <v>Lindabrowne@iprimus.com.au</v>
-      </c>
-      <c r="F36" t="str">
-        <v>429570177</v>
-      </c>
-      <c r="G36" t="str">
-        <v>OFFICER</v>
-      </c>
-      <c r="H36" t="str">
-        <v>B</v>
-      </c>
-      <c r="I36" t="str">
-        <v>available</v>
-      </c>
-      <c r="J36" t="str" xml:space="preserve">
+      <c r="J35" t="str" xml:space="preserve">
         <v xml:space="preserve">Natalie Browne
 Linda Browne
 Aidan Miler</v>
       </c>
     </row>
+    <row r="36" xml:space="preserve">
+      <c r="A36" t="str">
+        <v>1211456d-ea92-4a7b-9d94-885982cf345c</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Bronwyn Parsons</v>
+      </c>
+      <c r="C36">
+        <v>72</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Babybear61153@gmail.com</v>
+      </c>
+      <c r="F36" t="str">
+        <v>432543647</v>
+      </c>
+      <c r="G36" t="str">
+        <v>Rosebud</v>
+      </c>
+      <c r="H36" t="str">
+        <v>A+</v>
+      </c>
+      <c r="I36" t="str">
+        <v>available</v>
+      </c>
+      <c r="J36" t="str" xml:space="preserve">
+        <v xml:space="preserve">Yolette Huon - yol-et Hue on
+Bronwyn Parsons - Would like to be called Bron Emmerson - maiden name</v>
+      </c>
+    </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>c60666dd-e08c-4aa0-8582-4e7a3ad280f8</v>
+        <v>45c7f69f-dd89-41d8-b7f0-a83f77fa9d12</v>
       </c>
       <c r="B37" t="str">
-        <v>Bashar Mona</v>
+        <v>Sherif Haggag</v>
       </c>
       <c r="C37">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D37" t="str">
         <v>Male</v>
       </c>
       <c r="E37" t="str">
-        <v>bashar.mona92@gmail.com</v>
+        <v>Shaggag87@gmail.com</v>
       </c>
       <c r="F37" t="str">
-        <v>490871416</v>
+        <v>426233449</v>
       </c>
       <c r="G37" t="str">
-        <v>Roxburgh park</v>
+        <v>Belmont</v>
       </c>
       <c r="H37" t="str">
         <v>B+</v>
       </c>
       <c r="I37" t="str">
-        <v>assigned</v>
+        <v>available</v>
       </c>
       <c r="J37" t="str">
         <v>Solo</v>
@@ -1922,100 +1922,102 @@
     </row>
     <row r="38" xml:space="preserve">
       <c r="A38" t="str">
-        <v>1211456d-ea92-4a7b-9d94-885982cf345c</v>
+        <v>23f118f9-20db-422c-8cef-939dc73dd803</v>
       </c>
       <c r="B38" t="str">
-        <v>Bronwyn Parsons</v>
+        <v>Paige Greig</v>
       </c>
       <c r="C38">
-        <v>72</v>
+        <v>31</v>
       </c>
       <c r="D38" t="str">
         <v>Female</v>
       </c>
       <c r="E38" t="str">
-        <v>Babybear61153@gmail.com</v>
+        <v>paigegreig@hotmail.com</v>
       </c>
       <c r="F38" t="str">
-        <v>432543647</v>
+        <v>406598552</v>
       </c>
       <c r="G38" t="str">
-        <v>Rosebud</v>
+        <v>Mooroolbark</v>
       </c>
       <c r="H38" t="str">
-        <v>A+</v>
+        <v>C</v>
       </c>
       <c r="I38" t="str">
         <v>available</v>
       </c>
       <c r="J38" t="str" xml:space="preserve">
-        <v xml:space="preserve">Yolette Huon - yol-et Hue on
-Bronwyn Parsons - Would like to be called Bron Emmerson - maiden name</v>
-      </c>
-    </row>
-    <row r="39" xml:space="preserve">
-      <c r="A39" t="str">
-        <v>23f118f9-20db-422c-8cef-939dc73dd803</v>
-      </c>
-      <c r="B39" t="str">
-        <v>Paige Greig</v>
-      </c>
-      <c r="C39">
-        <v>31</v>
-      </c>
-      <c r="D39" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E39" t="str">
-        <v>paigegreig@hotmail.com</v>
-      </c>
-      <c r="F39" t="str">
-        <v>406598552</v>
-      </c>
-      <c r="G39" t="str">
-        <v>Mooroolbark</v>
-      </c>
-      <c r="H39" t="str">
-        <v>C</v>
-      </c>
-      <c r="I39" t="str">
-        <v>available</v>
-      </c>
-      <c r="J39" t="str" xml:space="preserve">
         <v xml:space="preserve">Erin
 Morgan (sister) - need to do application</v>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>c60666dd-e08c-4aa0-8582-4e7a3ad280f8</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Bashar Mona</v>
+      </c>
+      <c r="C39">
+        <v>33</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E39" t="str">
+        <v>bashar.mona92@gmail.com</v>
+      </c>
+      <c r="F39" t="str">
+        <v>490871416</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Roxburgh park</v>
+      </c>
+      <c r="H39" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I39" t="str">
+        <v>available</v>
+      </c>
+      <c r="J39" t="str">
+        <v>Solo</v>
+      </c>
+    </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>917bd31e-7781-44cc-936c-980cb1f844aa</v>
+        <v>cbfeb8b0-bd5d-4614-a055-cbac047cf152</v>
       </c>
       <c r="B40" t="str">
-        <v>Angela Verspay</v>
+        <v>Tamika Colville</v>
       </c>
       <c r="C40">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="D40" t="str">
         <v>Female</v>
       </c>
       <c r="E40" t="str">
-        <v>angelarileysmyth@hotmail.com</v>
+        <v>tamika.colville@gmail.com</v>
       </c>
       <c r="F40" t="str">
-        <v>477660119</v>
+        <v>409132141</v>
       </c>
       <c r="G40" t="str">
-        <v>Warrnambool</v>
+        <v>Golden square</v>
       </c>
       <c r="H40" t="str">
-        <v>B</v>
+        <v>B+</v>
       </c>
       <c r="I40" t="str">
-        <v>assigned</v>
+        <v>available</v>
       </c>
       <c r="J40" t="str">
-        <v>SOLO</v>
+        <v>Shinae Colville</v>
+      </c>
+      <c r="L40" t="str">
+        <v>Diagnosed with MS in 2018</v>
       </c>
       <c r="M40" t="str">
         <v>NA</v>
@@ -2023,25 +2025,25 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>cbfeb8b0-bd5d-4614-a055-cbac047cf152</v>
+        <v>441f345e-57a2-403b-a9a9-8284261eba7b</v>
       </c>
       <c r="B41" t="str">
-        <v>Tamika Colville</v>
+        <v>Kadisha  Bruton</v>
       </c>
       <c r="C41">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="D41" t="str">
         <v>Female</v>
       </c>
       <c r="E41" t="str">
-        <v>tamika.colville@gmail.com</v>
+        <v>kadishaann@icloud.com</v>
       </c>
       <c r="F41" t="str">
-        <v>409132141</v>
+        <v>434829249</v>
       </c>
       <c r="G41" t="str">
-        <v>Golden square</v>
+        <v xml:space="preserve">Kurunjang </v>
       </c>
       <c r="H41" t="str">
         <v>B+</v>
@@ -2050,13 +2052,7 @@
         <v>available</v>
       </c>
       <c r="J41" t="str">
-        <v>Shinae Colville</v>
-      </c>
-      <c r="L41" t="str">
-        <v>Diagnosed with MS in 2018</v>
-      </c>
-      <c r="M41" t="str">
-        <v>NA</v>
+        <v>Jacob Steele</v>
       </c>
     </row>
     <row r="42" xml:space="preserve">
@@ -2085,7 +2081,7 @@
         <v>B</v>
       </c>
       <c r="I42" t="str">
-        <v>assigned</v>
+        <v>available</v>
       </c>
       <c r="J42" t="str" xml:space="preserve">
         <v xml:space="preserve">Meenakshi Mehra
@@ -2095,27 +2091,27 @@
         <v>8c760df8-0e51-4b27-b1cb-0754c8b03595</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" xml:space="preserve">
       <c r="A43" t="str">
-        <v>441f345e-57a2-403b-a9a9-8284261eba7b</v>
+        <v>37fadce4-5d89-4542-a6e1-5e3e50620b85</v>
       </c>
       <c r="B43" t="str">
-        <v>Kadisha  Bruton</v>
+        <v>Sharyn  McKinnis</v>
       </c>
       <c r="C43">
-        <v>23</v>
+        <v>50</v>
       </c>
       <c r="D43" t="str">
         <v>Female</v>
       </c>
       <c r="E43" t="str">
-        <v>kadishaann@icloud.com</v>
+        <v>s.lmckinnis@bigpond.com</v>
       </c>
       <c r="F43" t="str">
-        <v>434829249</v>
+        <v>419880873</v>
       </c>
       <c r="G43" t="str">
-        <v xml:space="preserve">Kurunjang </v>
+        <v>Newtown</v>
       </c>
       <c r="H43" t="str">
         <v>B+</v>
@@ -2123,192 +2119,192 @@
       <c r="I43" t="str">
         <v>available</v>
       </c>
-      <c r="J43" t="str">
-        <v>Jacob Steele</v>
-      </c>
-    </row>
-    <row r="44" xml:space="preserve">
-      <c r="A44" t="str">
-        <v>37fadce4-5d89-4542-a6e1-5e3e50620b85</v>
-      </c>
-      <c r="B44" t="str">
-        <v>Sharyn  McKinnis</v>
-      </c>
-      <c r="C44">
-        <v>50</v>
-      </c>
-      <c r="D44" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E44" t="str">
-        <v>s.lmckinnis@bigpond.com</v>
-      </c>
-      <c r="F44" t="str">
-        <v>419880873</v>
-      </c>
-      <c r="G44" t="str">
-        <v>Newtown</v>
-      </c>
-      <c r="H44" t="str">
-        <v>B+</v>
-      </c>
-      <c r="I44" t="str">
-        <v>available</v>
-      </c>
-      <c r="J44" t="str" xml:space="preserve">
+      <c r="J43" t="str" xml:space="preserve">
         <v xml:space="preserve">Isabelle McKinnis, Sharyn McKinnis
 </v>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>646d2ff7-803b-4c80-bdd6-09d44eec6929</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Leanne Bryant</v>
+      </c>
+      <c r="C44">
+        <v>63</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E44" t="str">
+        <v>blazeandcougar@gmail.com</v>
+      </c>
+      <c r="F44" t="str">
+        <v>61415438228</v>
+      </c>
+      <c r="G44" t="str">
+        <v xml:space="preserve">Hampton Park </v>
+      </c>
+      <c r="H44" t="str">
+        <v>B</v>
+      </c>
+      <c r="I44" t="str">
+        <v>available</v>
+      </c>
+      <c r="J44" t="str">
+        <v>Solo</v>
+      </c>
+    </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>45c7f69f-dd89-41d8-b7f0-a83f77fa9d12</v>
+        <v>cfd3f567-ab69-4fa9-8a35-ca9c949fba91</v>
       </c>
       <c r="B45" t="str">
-        <v>Sherif Haggag</v>
+        <v>Michael Stevens</v>
       </c>
       <c r="C45">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="D45" t="str">
         <v>Male</v>
       </c>
       <c r="E45" t="str">
-        <v>Shaggag87@gmail.com</v>
+        <v>mjstevens1306@gmail.com</v>
       </c>
       <c r="F45" t="str">
-        <v>426233449</v>
+        <v>424659733</v>
       </c>
       <c r="G45" t="str">
-        <v>Belmont</v>
+        <v xml:space="preserve">Heathcote Junction </v>
       </c>
       <c r="H45" t="str">
-        <v>B+</v>
+        <v>A</v>
       </c>
       <c r="I45" t="str">
-        <v>assigned</v>
+        <v>available</v>
       </c>
       <c r="J45" t="str">
-        <v>Solo</v>
+        <v>Libby Dunbar</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>cfd3f567-ab69-4fa9-8a35-ca9c949fba91</v>
+        <v>f50d5074-9b3e-4386-9039-5e4cbd121267</v>
       </c>
       <c r="B46" t="str">
-        <v>Michael Stevens</v>
+        <v>Keera Bell</v>
       </c>
       <c r="C46">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="D46" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E46" t="str">
-        <v>mjstevens1306@gmail.com</v>
+        <v>Keera_b@hotmail.com</v>
       </c>
       <c r="F46" t="str">
-        <v>424659733</v>
+        <v>404754383</v>
       </c>
       <c r="G46" t="str">
-        <v xml:space="preserve">Heathcote Junction </v>
+        <v xml:space="preserve">Melbourne </v>
       </c>
       <c r="H46" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="I46" t="str">
         <v>available</v>
       </c>
       <c r="J46" t="str">
-        <v>Libby Dunbar</v>
+        <v>Dek Bell</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>f50d5074-9b3e-4386-9039-5e4cbd121267</v>
+        <v>0b96f877-e1c4-4c17-aa89-21b4a5f7f002</v>
       </c>
       <c r="B47" t="str">
-        <v>Keera Bell</v>
+        <v>Stephen Deacon</v>
       </c>
       <c r="C47">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="D47" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E47" t="str">
-        <v>Keera_b@hotmail.com</v>
+        <v>StephenDeacon@duck.com</v>
       </c>
       <c r="F47" t="str">
-        <v>404754383</v>
+        <v>435353108</v>
       </c>
       <c r="G47" t="str">
-        <v xml:space="preserve">Melbourne </v>
+        <v>St Kilda</v>
       </c>
       <c r="H47" t="str">
-        <v>B</v>
+        <v>B+</v>
       </c>
       <c r="I47" t="str">
         <v>available</v>
       </c>
       <c r="J47" t="str">
-        <v>Dek Bell</v>
+        <v>Chanyapach Deacon</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>0b96f877-e1c4-4c17-aa89-21b4a5f7f002</v>
+        <v>eb3b2a7d-e6b0-421b-8987-00bfff95dda9</v>
       </c>
       <c r="B48" t="str">
-        <v>Stephen Deacon</v>
+        <v>Jasmine Miller</v>
       </c>
       <c r="C48">
-        <v>67</v>
+        <v>32</v>
       </c>
       <c r="D48" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E48" t="str">
-        <v>StephenDeacon@duck.com</v>
+        <v>jasmine_courtney@hotmail.com</v>
       </c>
       <c r="F48" t="str">
-        <v>435353108</v>
+        <v>0432 387 712</v>
       </c>
       <c r="G48" t="str">
-        <v>St Kilda</v>
+        <v>Hughesdale</v>
       </c>
       <c r="H48" t="str">
-        <v>B+</v>
+        <v>C</v>
       </c>
       <c r="I48" t="str">
         <v>available</v>
       </c>
       <c r="J48" t="str">
-        <v>Chanyapach Deacon</v>
+        <v>ablo - partner</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>eb3b2a7d-e6b0-421b-8987-00bfff95dda9</v>
+        <v>300ac025-db3a-42ba-a9dd-777f02fb3454</v>
       </c>
       <c r="B49" t="str">
-        <v>Jasmine Miller</v>
+        <v>Jeanette Quy</v>
       </c>
       <c r="C49">
-        <v>32</v>
+        <v>74</v>
       </c>
       <c r="D49" t="str">
         <v>Female</v>
       </c>
       <c r="E49" t="str">
-        <v>jasmine_courtney@hotmail.com</v>
+        <v>koalaleaf@hotmail.com</v>
       </c>
       <c r="F49" t="str">
-        <v>0432 387 712</v>
+        <v>402902273</v>
       </c>
       <c r="G49" t="str">
-        <v>Hughesdale</v>
+        <v>Rowville</v>
       </c>
       <c r="H49" t="str">
         <v>C</v>
@@ -2317,30 +2313,33 @@
         <v>available</v>
       </c>
       <c r="J49" t="str">
-        <v>ablo - partner</v>
+        <v>Husband Ted Quy b6042a-1-1872960</v>
+      </c>
+      <c r="M49" t="str">
+        <v xml:space="preserve">Nothing of note </v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>300ac025-db3a-42ba-a9dd-777f02fb3454</v>
+        <v>0ea22efb-f85f-400a-b28d-d1312568ba67</v>
       </c>
       <c r="B50" t="str">
-        <v>Jeanette Quy</v>
+        <v>Jess Cossari</v>
       </c>
       <c r="C50">
-        <v>74</v>
+        <v>35</v>
       </c>
       <c r="D50" t="str">
         <v>Female</v>
       </c>
       <c r="E50" t="str">
-        <v>koalaleaf@hotmail.com</v>
+        <v>Jcossari@hotmail.com</v>
       </c>
       <c r="F50" t="str">
-        <v>402902273</v>
+        <v xml:space="preserve">0458 746 551 </v>
       </c>
       <c r="G50" t="str">
-        <v>Rowville</v>
+        <v xml:space="preserve">Melbourne </v>
       </c>
       <c r="H50" t="str">
         <v>C</v>
@@ -2349,42 +2348,42 @@
         <v>available</v>
       </c>
       <c r="J50" t="str">
-        <v>Husband Ted Quy b6042a-1-1872960</v>
-      </c>
-      <c r="M50" t="str">
-        <v xml:space="preserve">Nothing of note </v>
+        <v>Andrea Cocco</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>0ea22efb-f85f-400a-b28d-d1312568ba67</v>
+        <v>917bd31e-7781-44cc-936c-980cb1f844aa</v>
       </c>
       <c r="B51" t="str">
-        <v>Jess Cossari</v>
+        <v>Angela Verspay</v>
       </c>
       <c r="C51">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="D51" t="str">
         <v>Female</v>
       </c>
       <c r="E51" t="str">
-        <v>Jcossari@hotmail.com</v>
+        <v>angelarileysmyth@hotmail.com</v>
       </c>
       <c r="F51" t="str">
-        <v xml:space="preserve">0458 746 551 </v>
+        <v>477660119</v>
       </c>
       <c r="G51" t="str">
-        <v xml:space="preserve">Melbourne </v>
+        <v>Warrnambool</v>
       </c>
       <c r="H51" t="str">
-        <v>C</v>
+        <v>B</v>
       </c>
       <c r="I51" t="str">
         <v>available</v>
       </c>
       <c r="J51" t="str">
-        <v>Andrea Cocco</v>
+        <v>SOLO</v>
+      </c>
+      <c r="M51" t="str">
+        <v>NA</v>
       </c>
     </row>
   </sheetData>
@@ -2396,230 +2395,6 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H12"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>ID</v>
-      </c>
-      <c r="B1" t="str">
-        <v>RecordDayID</v>
-      </c>
-      <c r="C1" t="str">
-        <v>ContestantID</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Block</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Seat</v>
-      </c>
-      <c r="F1" t="str">
-        <v>BookingEmailSent</v>
-      </c>
-      <c r="G1" t="str">
-        <v>ConfirmedRSVP</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Notes</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>cbb914d8-4355-4eae-8e6a-d916e6eeab9c</v>
-      </c>
-      <c r="B2" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C2" t="str">
-        <v>6b9ae7f0-4a81-4dda-8e55-e49415d98ec6</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2" t="str">
-        <v>A1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>72ec2db4-7ad6-48e7-aada-ebcd77e964de</v>
-      </c>
-      <c r="B3" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C3" t="str">
-        <v>b1fc34e8-20cb-4607-9568-0761cf4520a6</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3" t="str">
-        <v>A2</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>3c715c30-77ec-4327-a1dc-77e587684309</v>
-      </c>
-      <c r="B4" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C4" t="str">
-        <v>7fc083f6-6be3-42bf-b4e5-fc6412e1c559</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4" t="str">
-        <v>A3</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>98131f5a-2b3c-46c8-876a-215c01d25450</v>
-      </c>
-      <c r="B5" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C5" t="str">
-        <v>54de1dd9-b7eb-489d-b4a1-8b3744a385c4</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5" t="str">
-        <v>A4</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>cd4bdfd0-1ea2-465c-9a88-0c4e8be41c46</v>
-      </c>
-      <c r="B6" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C6" t="str">
-        <v>e4a52d0d-9c54-4504-8a0f-85845cd88e27</v>
-      </c>
-      <c r="D6">
-        <v>1</v>
-      </c>
-      <c r="E6" t="str">
-        <v>A5</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>e3f866e4-5581-4731-8857-0d4dad4cee98</v>
-      </c>
-      <c r="B7" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C7" t="str">
-        <v>614641dd-4e94-4c42-a1d9-db37c608dcbe</v>
-      </c>
-      <c r="D7">
-        <v>1</v>
-      </c>
-      <c r="E7" t="str">
-        <v>B1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>525e206b-a4dc-4cb0-bb8d-350087facf3e</v>
-      </c>
-      <c r="B8" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C8" t="str">
-        <v>96c75db9-b001-4abe-8ddb-d5a73cb04529</v>
-      </c>
-      <c r="D8">
-        <v>1</v>
-      </c>
-      <c r="E8" t="str">
-        <v>B2</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>8d7a05d2-98e8-40f7-b7ff-a8b4cbbfcb46</v>
-      </c>
-      <c r="B9" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C9" t="str">
-        <v>45c7f69f-dd89-41d8-b7f0-a83f77fa9d12</v>
-      </c>
-      <c r="D9">
-        <v>1</v>
-      </c>
-      <c r="E9" t="str">
-        <v>B3</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>8d8eddd8-180f-4a64-af6b-a1e848b325b0</v>
-      </c>
-      <c r="B10" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C10" t="str">
-        <v>646d2ff7-803b-4c80-bdd6-09d44eec6929</v>
-      </c>
-      <c r="D10">
-        <v>1</v>
-      </c>
-      <c r="E10" t="str">
-        <v>B4</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>0b61d3fc-daf3-492d-b9a1-6070b61f0235</v>
-      </c>
-      <c r="B11" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C11" t="str">
-        <v>c60666dd-e08c-4aa0-8582-4e7a3ad280f8</v>
-      </c>
-      <c r="D11">
-        <v>1</v>
-      </c>
-      <c r="E11" t="str">
-        <v>B5</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>cd6ab2c2-d134-4f10-95c6-caa3b4590d32</v>
-      </c>
-      <c r="B12" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C12" t="str">
-        <v>917bd31e-7781-44cc-936c-980cb1f844aa</v>
-      </c>
-      <c r="D12">
-        <v>1</v>
-      </c>
-      <c r="E12" t="str">
-        <v>D1</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H12"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B4"/>
   <sheetData>
     <row r="1">
@@ -2661,7 +2436,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D27"/>
   <sheetData>

</xml_diff>

<commit_message>
Add ability to send paperwork emails and track receipt status
Implement bulk sending of paperwork emails with Adobe Sign links, add filtering for the paperwork tab, and introduce checkboxes for tracking received paperwork status.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: f123b9d7-6af8-472a-a75c-70d0b78d0583
Replit-Commit-Checkpoint-Type: intermediate_checkpoint
Replit-Commit-Event-Id: df10a9dc-1857-4d40-aaa2-1259b88c85e2
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/4ca2a1f8-42ce-4303-beff-eb92e3283d4c/f123b9d7-6af8-472a-a75c-70d0b78d0583/JBhUDJT
</commit_message>
<xml_diff>
--- a/storage/backups/automatic-backup.xlsx
+++ b/storage/backups/automatic-backup.xlsx
@@ -5,8 +5,9 @@
   <sheets>
     <sheet name="Record Days" sheetId="1" r:id="rId1"/>
     <sheet name="Contestants" sheetId="2" r:id="rId2"/>
-    <sheet name="Groups" sheetId="3" r:id="rId3"/>
-    <sheet name="Block Types" sheetId="4" r:id="rId4"/>
+    <sheet name="Seat Assignments" sheetId="3" r:id="rId3"/>
+    <sheet name="Groups" sheetId="4" r:id="rId4"/>
+    <sheet name="Block Types" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -735,7 +736,7 @@
         <v>B</v>
       </c>
       <c r="I2" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J2" t="str" xml:space="preserve">
         <v xml:space="preserve">Meenakshi Mehra
@@ -917,134 +918,128 @@
         <v>No</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" xml:space="preserve">
       <c r="A8" t="str">
-        <v>b1fc34e8-20cb-4607-9568-0761cf4520a6</v>
+        <v>1fe25fd6-dc69-4d29-b22f-9a15ad3d457f</v>
       </c>
       <c r="B8" t="str">
-        <v>Troy Smith</v>
+        <v>Sharon King</v>
       </c>
       <c r="C8">
-        <v>31</v>
+        <v>58</v>
       </c>
       <c r="D8" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E8" t="str">
-        <v>Troyssmith94@gmail.com</v>
+        <v>dreamweaversixtyseven@gmail.com</v>
       </c>
       <c r="F8" t="str">
-        <v>429354308</v>
+        <v>611488000000</v>
       </c>
       <c r="G8" t="str">
-        <v>Melbourne</v>
+        <v xml:space="preserve">Mooroopna </v>
       </c>
       <c r="H8" t="str">
-        <v>B+</v>
+        <v>A</v>
       </c>
       <c r="I8" t="str">
         <v>available</v>
       </c>
-      <c r="J8" t="str">
-        <v>Tayla Huxtable</v>
-      </c>
-      <c r="K8" t="str">
-        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
-      </c>
-      <c r="L8" t="str">
-        <v xml:space="preserve">Peanut allergy </v>
-      </c>
-      <c r="M8" t="str">
-        <v>NA</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>6b9ae7f0-4a81-4dda-8e55-e49415d98ec6</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Tayla Huxtable</v>
-      </c>
-      <c r="C9">
-        <v>28</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Taylahuxtable@gmail.com</v>
-      </c>
-      <c r="F9" t="str">
-        <v>435320280</v>
-      </c>
-      <c r="G9" t="str">
-        <v>FERNTREE GULLY</v>
-      </c>
-      <c r="I9" t="str">
-        <v>available</v>
-      </c>
-      <c r="J9" t="str">
-        <v>Troy Smith</v>
-      </c>
-      <c r="K9" t="str">
-        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
-      </c>
-    </row>
-    <row r="10" xml:space="preserve">
-      <c r="A10" t="str">
-        <v>1fe25fd6-dc69-4d29-b22f-9a15ad3d457f</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Sharon King</v>
-      </c>
-      <c r="C10">
-        <v>58</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E10" t="str">
-        <v>dreamweaversixtyseven@gmail.com</v>
-      </c>
-      <c r="F10" t="str">
-        <v>611488000000</v>
-      </c>
-      <c r="G10" t="str">
-        <v xml:space="preserve">Mooroopna </v>
-      </c>
-      <c r="H10" t="str">
-        <v>A</v>
-      </c>
-      <c r="I10" t="str">
-        <v>available</v>
-      </c>
-      <c r="J10" t="str" xml:space="preserve">
+      <c r="J8" t="str" xml:space="preserve">
         <v xml:space="preserve">
 Friend :Jacinda Austin
 ID:b6042a-1-1936475</v>
       </c>
-      <c r="M10" t="str">
+      <c r="M8" t="str">
         <v xml:space="preserve">No </v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>82960b61-d36b-49e2-9ddf-a7b8e0b02a63</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Tara Saltzman</v>
+      </c>
+      <c r="C9">
+        <v>29</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E9" t="str">
+        <v>tarasaltzman@bigpond.com</v>
+      </c>
+      <c r="F9" t="str">
+        <v>448545599</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Melbourne</v>
+      </c>
+      <c r="H9" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I9" t="str">
+        <v>available</v>
+      </c>
+      <c r="J9" t="str">
+        <v xml:space="preserve">JACK AGIUS - NEEDS TO DO APPLICATION </v>
+      </c>
+      <c r="M9" t="str">
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>f693566d-ea7c-40d1-89aa-158e842961d0</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Brent Barnett</v>
+      </c>
+      <c r="C10">
+        <v>37</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E10" t="str">
+        <v>brentbarnett88@gmail.com</v>
+      </c>
+      <c r="F10" t="str">
+        <v>423530043</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Preston</v>
+      </c>
+      <c r="H10" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I10" t="str">
+        <v>available</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Stephanie Squillacioti</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>82960b61-d36b-49e2-9ddf-a7b8e0b02a63</v>
+        <v>b1fc34e8-20cb-4607-9568-0761cf4520a6</v>
       </c>
       <c r="B11" t="str">
-        <v>Tara Saltzman</v>
+        <v>Troy Smith</v>
       </c>
       <c r="C11">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D11" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E11" t="str">
-        <v>tarasaltzman@bigpond.com</v>
+        <v>Troyssmith94@gmail.com</v>
       </c>
       <c r="F11" t="str">
-        <v>448545599</v>
+        <v>429354308</v>
       </c>
       <c r="G11" t="str">
         <v>Melbourne</v>
@@ -1053,10 +1048,16 @@
         <v>B+</v>
       </c>
       <c r="I11" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J11" t="str">
-        <v xml:space="preserve">JACK AGIUS - NEEDS TO DO APPLICATION </v>
+        <v>Tayla Huxtable</v>
+      </c>
+      <c r="K11" t="str">
+        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
+      </c>
+      <c r="L11" t="str">
+        <v xml:space="preserve">Peanut allergy </v>
       </c>
       <c r="M11" t="str">
         <v>NA</v>
@@ -1064,34 +1065,34 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>f693566d-ea7c-40d1-89aa-158e842961d0</v>
+        <v>6b9ae7f0-4a81-4dda-8e55-e49415d98ec6</v>
       </c>
       <c r="B12" t="str">
-        <v>Brent Barnett</v>
+        <v>Tayla Huxtable</v>
       </c>
       <c r="C12">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="D12" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E12" t="str">
-        <v>brentbarnett88@gmail.com</v>
+        <v>Taylahuxtable@gmail.com</v>
       </c>
       <c r="F12" t="str">
-        <v>423530043</v>
+        <v>435320280</v>
       </c>
       <c r="G12" t="str">
-        <v>Preston</v>
-      </c>
-      <c r="H12" t="str">
-        <v>B+</v>
+        <v>FERNTREE GULLY</v>
       </c>
       <c r="I12" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J12" t="str">
-        <v>Stephanie Squillacioti</v>
+        <v>Troy Smith</v>
+      </c>
+      <c r="K12" t="str">
+        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
       </c>
     </row>
     <row r="13">
@@ -1394,89 +1395,89 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>f048c8fe-e8c9-4357-8ec8-ef76793e5bc1</v>
+        <v>6cada433-8344-4d95-97dc-33c9c173ce7c</v>
       </c>
       <c r="B22" t="str">
-        <v>Tamara Mifsud</v>
+        <v>Jeanette Quy</v>
       </c>
       <c r="C22">
-        <v>32</v>
+        <v>74</v>
       </c>
       <c r="D22" t="str">
         <v>Female</v>
       </c>
       <c r="E22" t="str">
-        <v>tamara.mifsud@hotmail.com</v>
+        <v>quyfamily@tpg.com.au</v>
       </c>
       <c r="F22" t="str">
-        <v>416552122</v>
+        <v>402902273</v>
       </c>
       <c r="G22" t="str">
-        <v>Aintree</v>
+        <v>Rowville</v>
       </c>
       <c r="H22" t="str">
-        <v>B</v>
+        <v>C</v>
       </c>
       <c r="I22" t="str">
-        <v>available</v>
-      </c>
-      <c r="J22" t="str">
-        <v>Aliye Abcilar</v>
+        <v>assigned</v>
+      </c>
+      <c r="M22" t="str">
+        <v xml:space="preserve">nothing of note </v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>6bbdadcb-23a8-41c9-964b-6152e234cb33</v>
+        <v>f048c8fe-e8c9-4357-8ec8-ef76793e5bc1</v>
       </c>
       <c r="B23" t="str">
-        <v>Philip Natoli</v>
+        <v>Tamara Mifsud</v>
       </c>
       <c r="C23">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D23" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E23" t="str">
-        <v>Philip.natoli@outlook.com</v>
+        <v>tamara.mifsud@hotmail.com</v>
       </c>
       <c r="F23" t="str">
-        <v>466021882</v>
+        <v>416552122</v>
       </c>
       <c r="G23" t="str">
-        <v>Caulfield South</v>
+        <v>Aintree</v>
       </c>
       <c r="H23" t="str">
-        <v>B+</v>
+        <v>B</v>
       </c>
       <c r="I23" t="str">
         <v>available</v>
       </c>
       <c r="J23" t="str">
-        <v>Hayley Wright</v>
+        <v>Aliye Abcilar</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>614641dd-4e94-4c42-a1d9-db37c608dcbe</v>
+        <v>6bbdadcb-23a8-41c9-964b-6152e234cb33</v>
       </c>
       <c r="B24" t="str">
-        <v>Antonio Freno</v>
+        <v>Philip Natoli</v>
       </c>
       <c r="C24">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="D24" t="str">
         <v>Male</v>
       </c>
       <c r="E24" t="str">
-        <v>frenoantonio@hotmail.it</v>
+        <v>Philip.natoli@outlook.com</v>
       </c>
       <c r="F24" t="str">
-        <v>422177371</v>
+        <v>466021882</v>
       </c>
       <c r="G24" t="str">
-        <v>Glenroy</v>
+        <v>Caulfield South</v>
       </c>
       <c r="H24" t="str">
         <v>B+</v>
@@ -1485,39 +1486,39 @@
         <v>available</v>
       </c>
       <c r="J24" t="str">
-        <v>Solo</v>
+        <v>Hayley Wright</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>6cada433-8344-4d95-97dc-33c9c173ce7c</v>
+        <v>614641dd-4e94-4c42-a1d9-db37c608dcbe</v>
       </c>
       <c r="B25" t="str">
-        <v>Jeanette Quy</v>
+        <v>Antonio Freno</v>
       </c>
       <c r="C25">
-        <v>74</v>
+        <v>39</v>
       </c>
       <c r="D25" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E25" t="str">
-        <v>quyfamily@tpg.com.au</v>
+        <v>frenoantonio@hotmail.it</v>
       </c>
       <c r="F25" t="str">
-        <v>402902273</v>
+        <v>422177371</v>
       </c>
       <c r="G25" t="str">
-        <v>Rowville</v>
+        <v>Glenroy</v>
       </c>
       <c r="H25" t="str">
-        <v>C</v>
+        <v>B+</v>
       </c>
       <c r="I25" t="str">
-        <v>available</v>
-      </c>
-      <c r="M25" t="str">
-        <v xml:space="preserve">nothing of note </v>
+        <v>assigned</v>
+      </c>
+      <c r="J25" t="str">
+        <v>Solo</v>
       </c>
     </row>
     <row r="26" xml:space="preserve">
@@ -1684,7 +1685,7 @@
         <v>B+</v>
       </c>
       <c r="I30" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J30" t="str">
         <v>Solo</v>
@@ -1716,7 +1717,7 @@
         <v>B+</v>
       </c>
       <c r="I31" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J31" t="str">
         <v>SOLO</v>
@@ -1791,133 +1792,136 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
+        <v>917bd31e-7781-44cc-936c-980cb1f844aa</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Angela Verspay</v>
+      </c>
+      <c r="C34">
+        <v>45</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E34" t="str">
+        <v>angelarileysmyth@hotmail.com</v>
+      </c>
+      <c r="F34" t="str">
+        <v>477660119</v>
+      </c>
+      <c r="G34" t="str">
+        <v>Warrnambool</v>
+      </c>
+      <c r="H34" t="str">
+        <v>B</v>
+      </c>
+      <c r="I34" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="J34" t="str">
+        <v>SOLO</v>
+      </c>
+      <c r="M34" t="str">
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
         <v>2aadb3db-ad8e-4edd-a81d-f045a926ceb9</v>
       </c>
-      <c r="B34" t="str">
+      <c r="B35" t="str">
         <v>Alexander Leonard</v>
       </c>
-      <c r="C34">
+      <c r="C35">
         <v>38</v>
       </c>
-      <c r="D34" t="str">
+      <c r="D35" t="str">
         <v>Male</v>
       </c>
-      <c r="E34" t="str">
+      <c r="E35" t="str">
         <v>alexleonardedit@gmail.com</v>
       </c>
-      <c r="F34" t="str">
+      <c r="F35" t="str">
         <v>421834476</v>
       </c>
-      <c r="G34" t="str">
+      <c r="G35" t="str">
         <v>Croydon</v>
       </c>
-      <c r="H34" t="str">
+      <c r="H35" t="str">
         <v>A+</v>
       </c>
-      <c r="I34" t="str">
-        <v>available</v>
-      </c>
-      <c r="J34" t="str">
+      <c r="I35" t="str">
+        <v>available</v>
+      </c>
+      <c r="J35" t="str">
         <v>melissa francis, Alexander Leonard</v>
       </c>
     </row>
-    <row r="35" xml:space="preserve">
-      <c r="A35" t="str">
+    <row r="36" xml:space="preserve">
+      <c r="A36" t="str">
         <v>ed91813b-2f74-4638-9d1a-ef8c54cff447</v>
       </c>
-      <c r="B35" t="str">
+      <c r="B36" t="str">
         <v>Linda Browne</v>
       </c>
-      <c r="C35">
+      <c r="C36">
         <v>54</v>
       </c>
-      <c r="D35" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E35" t="str">
+      <c r="D36" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E36" t="str">
         <v>Lindabrowne@iprimus.com.au</v>
       </c>
-      <c r="F35" t="str">
+      <c r="F36" t="str">
         <v>429570177</v>
       </c>
-      <c r="G35" t="str">
+      <c r="G36" t="str">
         <v>OFFICER</v>
       </c>
-      <c r="H35" t="str">
+      <c r="H36" t="str">
         <v>B</v>
       </c>
-      <c r="I35" t="str">
-        <v>available</v>
-      </c>
-      <c r="J35" t="str" xml:space="preserve">
+      <c r="I36" t="str">
+        <v>available</v>
+      </c>
+      <c r="J36" t="str" xml:space="preserve">
         <v xml:space="preserve">Natalie Browne
 Linda Browne
 Aidan Miler</v>
       </c>
     </row>
-    <row r="36" xml:space="preserve">
-      <c r="A36" t="str">
+    <row r="37" xml:space="preserve">
+      <c r="A37" t="str">
         <v>1211456d-ea92-4a7b-9d94-885982cf345c</v>
       </c>
-      <c r="B36" t="str">
+      <c r="B37" t="str">
         <v>Bronwyn Parsons</v>
       </c>
-      <c r="C36">
+      <c r="C37">
         <v>72</v>
       </c>
-      <c r="D36" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E36" t="str">
+      <c r="D37" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E37" t="str">
         <v>Babybear61153@gmail.com</v>
       </c>
-      <c r="F36" t="str">
+      <c r="F37" t="str">
         <v>432543647</v>
       </c>
-      <c r="G36" t="str">
+      <c r="G37" t="str">
         <v>Rosebud</v>
       </c>
-      <c r="H36" t="str">
+      <c r="H37" t="str">
         <v>A+</v>
       </c>
-      <c r="I36" t="str">
-        <v>available</v>
-      </c>
-      <c r="J36" t="str" xml:space="preserve">
+      <c r="I37" t="str">
+        <v>available</v>
+      </c>
+      <c r="J37" t="str" xml:space="preserve">
         <v xml:space="preserve">Yolette Huon - yol-et Hue on
 Bronwyn Parsons - Would like to be called Bron Emmerson - maiden name</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <v>45c7f69f-dd89-41d8-b7f0-a83f77fa9d12</v>
-      </c>
-      <c r="B37" t="str">
-        <v>Sherif Haggag</v>
-      </c>
-      <c r="C37">
-        <v>38</v>
-      </c>
-      <c r="D37" t="str">
-        <v>Male</v>
-      </c>
-      <c r="E37" t="str">
-        <v>Shaggag87@gmail.com</v>
-      </c>
-      <c r="F37" t="str">
-        <v>426233449</v>
-      </c>
-      <c r="G37" t="str">
-        <v>Belmont</v>
-      </c>
-      <c r="H37" t="str">
-        <v>B+</v>
-      </c>
-      <c r="I37" t="str">
-        <v>available</v>
-      </c>
-      <c r="J37" t="str">
-        <v>Solo</v>
       </c>
     </row>
     <row r="38" xml:space="preserve">
@@ -1955,31 +1959,31 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>c60666dd-e08c-4aa0-8582-4e7a3ad280f8</v>
+        <v>45c7f69f-dd89-41d8-b7f0-a83f77fa9d12</v>
       </c>
       <c r="B39" t="str">
-        <v>Bashar Mona</v>
+        <v>Sherif Haggag</v>
       </c>
       <c r="C39">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D39" t="str">
         <v>Male</v>
       </c>
       <c r="E39" t="str">
-        <v>bashar.mona92@gmail.com</v>
+        <v>Shaggag87@gmail.com</v>
       </c>
       <c r="F39" t="str">
-        <v>490871416</v>
+        <v>426233449</v>
       </c>
       <c r="G39" t="str">
-        <v>Roxburgh park</v>
+        <v>Belmont</v>
       </c>
       <c r="H39" t="str">
         <v>B+</v>
       </c>
       <c r="I39" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J39" t="str">
         <v>Solo</v>
@@ -1987,63 +1991,57 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>cbfeb8b0-bd5d-4614-a055-cbac047cf152</v>
+        <v>c60666dd-e08c-4aa0-8582-4e7a3ad280f8</v>
       </c>
       <c r="B40" t="str">
-        <v>Tamika Colville</v>
+        <v>Bashar Mona</v>
       </c>
       <c r="C40">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D40" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E40" t="str">
-        <v>tamika.colville@gmail.com</v>
+        <v>bashar.mona92@gmail.com</v>
       </c>
       <c r="F40" t="str">
-        <v>409132141</v>
+        <v>490871416</v>
       </c>
       <c r="G40" t="str">
-        <v>Golden square</v>
+        <v>Roxburgh park</v>
       </c>
       <c r="H40" t="str">
         <v>B+</v>
       </c>
       <c r="I40" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J40" t="str">
-        <v>Shinae Colville</v>
-      </c>
-      <c r="L40" t="str">
-        <v>Diagnosed with MS in 2018</v>
-      </c>
-      <c r="M40" t="str">
-        <v>NA</v>
+        <v>Solo</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>441f345e-57a2-403b-a9a9-8284261eba7b</v>
+        <v>cbfeb8b0-bd5d-4614-a055-cbac047cf152</v>
       </c>
       <c r="B41" t="str">
-        <v>Kadisha  Bruton</v>
+        <v>Tamika Colville</v>
       </c>
       <c r="C41">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="D41" t="str">
         <v>Female</v>
       </c>
       <c r="E41" t="str">
-        <v>kadishaann@icloud.com</v>
+        <v>tamika.colville@gmail.com</v>
       </c>
       <c r="F41" t="str">
-        <v>434829249</v>
+        <v>409132141</v>
       </c>
       <c r="G41" t="str">
-        <v xml:space="preserve">Kurunjang </v>
+        <v>Golden square</v>
       </c>
       <c r="H41" t="str">
         <v>B+</v>
@@ -2052,7 +2050,13 @@
         <v>available</v>
       </c>
       <c r="J41" t="str">
-        <v>Jacob Steele</v>
+        <v>Shinae Colville</v>
+      </c>
+      <c r="L41" t="str">
+        <v>Diagnosed with MS in 2018</v>
+      </c>
+      <c r="M41" t="str">
+        <v>NA</v>
       </c>
     </row>
     <row r="42" xml:space="preserve">
@@ -2081,7 +2085,7 @@
         <v>B</v>
       </c>
       <c r="I42" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J42" t="str" xml:space="preserve">
         <v xml:space="preserve">Meenakshi Mehra
@@ -2091,27 +2095,27 @@
         <v>8c760df8-0e51-4b27-b1cb-0754c8b03595</v>
       </c>
     </row>
-    <row r="43" xml:space="preserve">
+    <row r="43">
       <c r="A43" t="str">
-        <v>37fadce4-5d89-4542-a6e1-5e3e50620b85</v>
+        <v>441f345e-57a2-403b-a9a9-8284261eba7b</v>
       </c>
       <c r="B43" t="str">
-        <v>Sharyn  McKinnis</v>
+        <v>Kadisha  Bruton</v>
       </c>
       <c r="C43">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="D43" t="str">
         <v>Female</v>
       </c>
       <c r="E43" t="str">
-        <v>s.lmckinnis@bigpond.com</v>
+        <v>kadishaann@icloud.com</v>
       </c>
       <c r="F43" t="str">
-        <v>419880873</v>
+        <v>434829249</v>
       </c>
       <c r="G43" t="str">
-        <v>Newtown</v>
+        <v xml:space="preserve">Kurunjang </v>
       </c>
       <c r="H43" t="str">
         <v>B+</v>
@@ -2119,192 +2123,192 @@
       <c r="I43" t="str">
         <v>available</v>
       </c>
-      <c r="J43" t="str" xml:space="preserve">
+      <c r="J43" t="str">
+        <v>Jacob Steele</v>
+      </c>
+    </row>
+    <row r="44" xml:space="preserve">
+      <c r="A44" t="str">
+        <v>37fadce4-5d89-4542-a6e1-5e3e50620b85</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Sharyn  McKinnis</v>
+      </c>
+      <c r="C44">
+        <v>50</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E44" t="str">
+        <v>s.lmckinnis@bigpond.com</v>
+      </c>
+      <c r="F44" t="str">
+        <v>419880873</v>
+      </c>
+      <c r="G44" t="str">
+        <v>Newtown</v>
+      </c>
+      <c r="H44" t="str">
+        <v>B+</v>
+      </c>
+      <c r="I44" t="str">
+        <v>available</v>
+      </c>
+      <c r="J44" t="str" xml:space="preserve">
         <v xml:space="preserve">Isabelle McKinnis, Sharyn McKinnis
 </v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="str">
-        <v>646d2ff7-803b-4c80-bdd6-09d44eec6929</v>
-      </c>
-      <c r="B44" t="str">
-        <v>Leanne Bryant</v>
-      </c>
-      <c r="C44">
-        <v>63</v>
-      </c>
-      <c r="D44" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E44" t="str">
-        <v>blazeandcougar@gmail.com</v>
-      </c>
-      <c r="F44" t="str">
-        <v>61415438228</v>
-      </c>
-      <c r="G44" t="str">
-        <v xml:space="preserve">Hampton Park </v>
-      </c>
-      <c r="H44" t="str">
-        <v>B</v>
-      </c>
-      <c r="I44" t="str">
-        <v>available</v>
-      </c>
-      <c r="J44" t="str">
-        <v>Solo</v>
-      </c>
-    </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>cfd3f567-ab69-4fa9-8a35-ca9c949fba91</v>
+        <v>646d2ff7-803b-4c80-bdd6-09d44eec6929</v>
       </c>
       <c r="B45" t="str">
-        <v>Michael Stevens</v>
+        <v>Leanne Bryant</v>
       </c>
       <c r="C45">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="D45" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E45" t="str">
-        <v>mjstevens1306@gmail.com</v>
+        <v>blazeandcougar@gmail.com</v>
       </c>
       <c r="F45" t="str">
-        <v>424659733</v>
+        <v>61415438228</v>
       </c>
       <c r="G45" t="str">
-        <v xml:space="preserve">Heathcote Junction </v>
+        <v xml:space="preserve">Hampton Park </v>
       </c>
       <c r="H45" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="I45" t="str">
-        <v>available</v>
+        <v>assigned</v>
       </c>
       <c r="J45" t="str">
-        <v>Libby Dunbar</v>
+        <v>Solo</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>f50d5074-9b3e-4386-9039-5e4cbd121267</v>
+        <v>cfd3f567-ab69-4fa9-8a35-ca9c949fba91</v>
       </c>
       <c r="B46" t="str">
-        <v>Keera Bell</v>
+        <v>Michael Stevens</v>
       </c>
       <c r="C46">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="D46" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E46" t="str">
-        <v>Keera_b@hotmail.com</v>
+        <v>mjstevens1306@gmail.com</v>
       </c>
       <c r="F46" t="str">
-        <v>404754383</v>
+        <v>424659733</v>
       </c>
       <c r="G46" t="str">
-        <v xml:space="preserve">Melbourne </v>
+        <v xml:space="preserve">Heathcote Junction </v>
       </c>
       <c r="H46" t="str">
-        <v>B</v>
+        <v>A</v>
       </c>
       <c r="I46" t="str">
         <v>available</v>
       </c>
       <c r="J46" t="str">
-        <v>Dek Bell</v>
+        <v>Libby Dunbar</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>0b96f877-e1c4-4c17-aa89-21b4a5f7f002</v>
+        <v>f50d5074-9b3e-4386-9039-5e4cbd121267</v>
       </c>
       <c r="B47" t="str">
-        <v>Stephen Deacon</v>
+        <v>Keera Bell</v>
       </c>
       <c r="C47">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="D47" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E47" t="str">
-        <v>StephenDeacon@duck.com</v>
+        <v>Keera_b@hotmail.com</v>
       </c>
       <c r="F47" t="str">
-        <v>435353108</v>
+        <v>404754383</v>
       </c>
       <c r="G47" t="str">
-        <v>St Kilda</v>
+        <v xml:space="preserve">Melbourne </v>
       </c>
       <c r="H47" t="str">
-        <v>B+</v>
+        <v>B</v>
       </c>
       <c r="I47" t="str">
         <v>available</v>
       </c>
       <c r="J47" t="str">
-        <v>Chanyapach Deacon</v>
+        <v>Dek Bell</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>eb3b2a7d-e6b0-421b-8987-00bfff95dda9</v>
+        <v>0b96f877-e1c4-4c17-aa89-21b4a5f7f002</v>
       </c>
       <c r="B48" t="str">
-        <v>Jasmine Miller</v>
+        <v>Stephen Deacon</v>
       </c>
       <c r="C48">
-        <v>32</v>
+        <v>67</v>
       </c>
       <c r="D48" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E48" t="str">
-        <v>jasmine_courtney@hotmail.com</v>
+        <v>StephenDeacon@duck.com</v>
       </c>
       <c r="F48" t="str">
-        <v>0432 387 712</v>
+        <v>435353108</v>
       </c>
       <c r="G48" t="str">
-        <v>Hughesdale</v>
+        <v>St Kilda</v>
       </c>
       <c r="H48" t="str">
-        <v>C</v>
+        <v>B+</v>
       </c>
       <c r="I48" t="str">
         <v>available</v>
       </c>
       <c r="J48" t="str">
-        <v>ablo - partner</v>
+        <v>Chanyapach Deacon</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>300ac025-db3a-42ba-a9dd-777f02fb3454</v>
+        <v>eb3b2a7d-e6b0-421b-8987-00bfff95dda9</v>
       </c>
       <c r="B49" t="str">
-        <v>Jeanette Quy</v>
+        <v>Jasmine Miller</v>
       </c>
       <c r="C49">
-        <v>74</v>
+        <v>32</v>
       </c>
       <c r="D49" t="str">
         <v>Female</v>
       </c>
       <c r="E49" t="str">
-        <v>koalaleaf@hotmail.com</v>
+        <v>jasmine_courtney@hotmail.com</v>
       </c>
       <c r="F49" t="str">
-        <v>402902273</v>
+        <v>0432 387 712</v>
       </c>
       <c r="G49" t="str">
-        <v>Rowville</v>
+        <v>Hughesdale</v>
       </c>
       <c r="H49" t="str">
         <v>C</v>
@@ -2313,33 +2317,30 @@
         <v>available</v>
       </c>
       <c r="J49" t="str">
-        <v>Husband Ted Quy b6042a-1-1872960</v>
-      </c>
-      <c r="M49" t="str">
-        <v xml:space="preserve">Nothing of note </v>
+        <v>ablo - partner</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>0ea22efb-f85f-400a-b28d-d1312568ba67</v>
+        <v>300ac025-db3a-42ba-a9dd-777f02fb3454</v>
       </c>
       <c r="B50" t="str">
-        <v>Jess Cossari</v>
+        <v>Jeanette Quy</v>
       </c>
       <c r="C50">
-        <v>35</v>
+        <v>74</v>
       </c>
       <c r="D50" t="str">
         <v>Female</v>
       </c>
       <c r="E50" t="str">
-        <v>Jcossari@hotmail.com</v>
+        <v>koalaleaf@hotmail.com</v>
       </c>
       <c r="F50" t="str">
-        <v xml:space="preserve">0458 746 551 </v>
+        <v>402902273</v>
       </c>
       <c r="G50" t="str">
-        <v xml:space="preserve">Melbourne </v>
+        <v>Rowville</v>
       </c>
       <c r="H50" t="str">
         <v>C</v>
@@ -2348,42 +2349,42 @@
         <v>available</v>
       </c>
       <c r="J50" t="str">
-        <v>Andrea Cocco</v>
+        <v>Husband Ted Quy b6042a-1-1872960</v>
+      </c>
+      <c r="M50" t="str">
+        <v xml:space="preserve">Nothing of note </v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>917bd31e-7781-44cc-936c-980cb1f844aa</v>
+        <v>0ea22efb-f85f-400a-b28d-d1312568ba67</v>
       </c>
       <c r="B51" t="str">
-        <v>Angela Verspay</v>
+        <v>Jess Cossari</v>
       </c>
       <c r="C51">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="D51" t="str">
         <v>Female</v>
       </c>
       <c r="E51" t="str">
-        <v>angelarileysmyth@hotmail.com</v>
+        <v>Jcossari@hotmail.com</v>
       </c>
       <c r="F51" t="str">
-        <v>477660119</v>
+        <v xml:space="preserve">0458 746 551 </v>
       </c>
       <c r="G51" t="str">
-        <v>Warrnambool</v>
+        <v xml:space="preserve">Melbourne </v>
       </c>
       <c r="H51" t="str">
-        <v>B</v>
+        <v>C</v>
       </c>
       <c r="I51" t="str">
         <v>available</v>
       </c>
       <c r="J51" t="str">
-        <v>SOLO</v>
-      </c>
-      <c r="M51" t="str">
-        <v>NA</v>
+        <v>Andrea Cocco</v>
       </c>
     </row>
   </sheetData>
@@ -2395,6 +2396,247 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H13"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>RecordDayID</v>
+      </c>
+      <c r="C1" t="str">
+        <v>ContestantID</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Block</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Seat</v>
+      </c>
+      <c r="F1" t="str">
+        <v>BookingEmailSent</v>
+      </c>
+      <c r="G1" t="str">
+        <v>ConfirmedRSVP</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>c428090e-0851-4b9f-9cdf-b348454d0c4e</v>
+      </c>
+      <c r="B2" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C2" t="str">
+        <v>b1fc34e8-20cb-4607-9568-0761cf4520a6</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="str">
+        <v>A1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>f0011d52-8ade-4f64-8ae4-ac21e90ea107</v>
+      </c>
+      <c r="B3" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C3" t="str">
+        <v>6b9ae7f0-4a81-4dda-8e55-e49415d98ec6</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3" t="str">
+        <v>A2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>71557816-b068-469d-81bc-86890e16382c</v>
+      </c>
+      <c r="B4" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C4" t="str">
+        <v>614641dd-4e94-4c42-a1d9-db37c608dcbe</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" t="str">
+        <v>A3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>038813f4-6e6c-4514-a5d1-48ddd8b23b1a</v>
+      </c>
+      <c r="B5" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C5" t="str">
+        <v>e4a52d0d-9c54-4504-8a0f-85845cd88e27</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" t="str">
+        <v>A4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>9eff4738-21c1-4c84-a047-c967ca2455b8</v>
+      </c>
+      <c r="B6" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C6" t="str">
+        <v>96c75db9-b001-4abe-8ddb-d5a73cb04529</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" t="str">
+        <v>A5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>4d40a2f2-bd3f-4706-bf35-af6009f63454</v>
+      </c>
+      <c r="B7" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C7" t="str">
+        <v>45c7f69f-dd89-41d8-b7f0-a83f77fa9d12</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7" t="str">
+        <v>A1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>d70bd36a-e512-49d1-a282-af50e4a270be</v>
+      </c>
+      <c r="B8" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C8" t="str">
+        <v>c60666dd-e08c-4aa0-8582-4e7a3ad280f8</v>
+      </c>
+      <c r="D8">
+        <v>3</v>
+      </c>
+      <c r="E8" t="str">
+        <v>A1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>2a8393a8-50cd-4281-adca-3a3a3dc4ebd0</v>
+      </c>
+      <c r="B9" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C9" t="str">
+        <v>646d2ff7-803b-4c80-bdd6-09d44eec6929</v>
+      </c>
+      <c r="D9">
+        <v>3</v>
+      </c>
+      <c r="E9" t="str">
+        <v>A2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>e6be730c-352f-480e-a6ea-22218cf952b5</v>
+      </c>
+      <c r="B10" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C10" t="str">
+        <v>917bd31e-7781-44cc-936c-980cb1f844aa</v>
+      </c>
+      <c r="D10">
+        <v>3</v>
+      </c>
+      <c r="E10" t="str">
+        <v>A3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>119c5658-ecfd-4a4f-a9eb-5ca7b7a6f5f7</v>
+      </c>
+      <c r="B11" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C11" t="str">
+        <v>6cada433-8344-4d95-97dc-33c9c173ce7c</v>
+      </c>
+      <c r="D11">
+        <v>5</v>
+      </c>
+      <c r="E11" t="str">
+        <v>A1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>d9f5032e-edab-4349-a70d-e4c64699eb6b</v>
+      </c>
+      <c r="B12" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C12" t="str">
+        <v>7fc083f6-6be3-42bf-b4e5-fc6412e1c559</v>
+      </c>
+      <c r="D12">
+        <v>5</v>
+      </c>
+      <c r="E12" t="str">
+        <v>A2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>115ba5a2-17a0-426b-8ed1-38ed2cb0bce3</v>
+      </c>
+      <c r="B13" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C13" t="str">
+        <v>54de1dd9-b7eb-489d-b4a1-8b3744a385c4</v>
+      </c>
+      <c r="D13">
+        <v>5</v>
+      </c>
+      <c r="E13" t="str">
+        <v>A3</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H13"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B4"/>
   <sheetData>
     <row r="1">
@@ -2436,7 +2678,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D27"/>
   <sheetData>

</xml_diff>

<commit_message>
Add ability to link and unlink contestants into groups
Adds manual group linking functionality via a new API endpoint and associated UI components. Also introduces the ability to unlink contestants from groups. Fixes an import error in routes.ts related to drizzle-orm's `eq` function. Updates test data with sample contestants and groups.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: f123b9d7-6af8-472a-a75c-70d0b78d0583
Replit-Commit-Checkpoint-Type: intermediate_checkpoint
Replit-Commit-Event-Id: 345cfe5f-8324-4767-82e8-074dd2e13343
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/4ca2a1f8-42ce-4303-beff-eb92e3283d4c/f123b9d7-6af8-472a-a75c-70d0b78d0583/rlQXkaM
</commit_message>
<xml_diff>
--- a/storage/backups/automatic-backup.xlsx
+++ b/storage/backups/automatic-backup.xlsx
@@ -4,8 +4,9 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Record Days" sheetId="1" r:id="rId1"/>
-    <sheet name="Groups" sheetId="2" r:id="rId2"/>
-    <sheet name="Block Types" sheetId="3" r:id="rId3"/>
+    <sheet name="Contestants" sheetId="2" r:id="rId2"/>
+    <sheet name="Groups" sheetId="3" r:id="rId3"/>
+    <sheet name="Block Types" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -665,49 +666,163 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:M3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>ID</v>
       </c>
       <c r="B1" t="str">
-        <v>ReferenceNumber</v>
+        <v>Name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Age</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Gender</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Email</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Phone</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Location</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Rating</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="J1" t="str">
+        <v>AttendingWith</v>
+      </c>
+      <c r="K1" t="str">
+        <v>GroupID</v>
+      </c>
+      <c r="L1" t="str">
+        <v>MedicalInfo</v>
+      </c>
+      <c r="M1" t="str">
+        <v>MobilityNotes</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>f25a6094-c1a5-4eb4-a709-1cc3d9b3ab5e</v>
+        <v>test-link-a</v>
       </c>
       <c r="B2" t="str">
-        <v>GRP001</v>
+        <v>Alice Test</v>
+      </c>
+      <c r="C2">
+        <v>28</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E2" t="str">
+        <v>alice@test.com</v>
+      </c>
+      <c r="F2" t="str">
+        <v>555-1001</v>
+      </c>
+      <c r="I2" t="str">
+        <v>available</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
+        <v>test-link-b</v>
       </c>
       <c r="B3" t="str">
-        <v>GRP002</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>8c760df8-0e51-4b27-b1cb-0754c8b03595</v>
-      </c>
-      <c r="B4" t="str">
-        <v>AUTO-MK2NF2KE-kuoa</v>
+        <v>Bob Test</v>
+      </c>
+      <c r="C3">
+        <v>32</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E3" t="str">
+        <v>bob@test.com</v>
+      </c>
+      <c r="F3" t="str">
+        <v>555-1002</v>
+      </c>
+      <c r="I3" t="str">
+        <v>available</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B6"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>ReferenceNumber</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>f25a6094-c1a5-4eb4-a709-1cc3d9b3ab5e</v>
+      </c>
+      <c r="B2" t="str">
+        <v>GRP001</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
+      </c>
+      <c r="B3" t="str">
+        <v>GRP002</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>8c760df8-0e51-4b27-b1cb-0754c8b03595</v>
+      </c>
+      <c r="B4" t="str">
+        <v>AUTO-MK2NF2KE-kuoa</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>632fede5-4c1f-4f47-8a24-f4c94563915f</v>
+      </c>
+      <c r="B5" t="str">
+        <v>MANUAL-MKB8V43C</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>d5513a17-247e-49c4-be46-eca3c0aa0c4c</v>
+      </c>
+      <c r="B6" t="str">
+        <v>MANUAL-MKB952R9</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D27"/>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Fix nested paragraph errors in contestant dialogs
Updates UI components in `client/src/pages/contestants.tsx` to resolve invalid HTML by changing nested `<p>` tags within `DialogDescription` to `<span>` elements. Also modifies `storage/backups/automatic-backup.json` to remove existing test contestant data and update `exportedAt` timestamp.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: f123b9d7-6af8-472a-a75c-70d0b78d0583
Replit-Commit-Checkpoint-Type: intermediate_checkpoint
Replit-Commit-Event-Id: a41ca4e6-8b3e-4c4f-b5df-f48e66f969cb
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/4ca2a1f8-42ce-4303-beff-eb92e3283d4c/f123b9d7-6af8-472a-a75c-70d0b78d0583/rlQXkaM
</commit_message>
<xml_diff>
--- a/storage/backups/automatic-backup.xlsx
+++ b/storage/backups/automatic-backup.xlsx
@@ -4,9 +4,8 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Record Days" sheetId="1" r:id="rId1"/>
-    <sheet name="Contestants" sheetId="2" r:id="rId2"/>
-    <sheet name="Groups" sheetId="3" r:id="rId3"/>
-    <sheet name="Block Types" sheetId="4" r:id="rId4"/>
+    <sheet name="Groups" sheetId="2" r:id="rId2"/>
+    <sheet name="Block Types" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -666,104 +665,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M3"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>ID</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Name</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Age</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Gender</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Email</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Phone</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Location</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Rating</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="J1" t="str">
-        <v>AttendingWith</v>
-      </c>
-      <c r="K1" t="str">
-        <v>GroupID</v>
-      </c>
-      <c r="L1" t="str">
-        <v>MedicalInfo</v>
-      </c>
-      <c r="M1" t="str">
-        <v>MobilityNotes</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>test-link-a</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Alice Test</v>
-      </c>
-      <c r="C2">
-        <v>28</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Female</v>
-      </c>
-      <c r="E2" t="str">
-        <v>alice@test.com</v>
-      </c>
-      <c r="F2" t="str">
-        <v>555-1001</v>
-      </c>
-      <c r="I2" t="str">
-        <v>available</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>test-link-b</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Bob Test</v>
-      </c>
-      <c r="C3">
-        <v>32</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Male</v>
-      </c>
-      <c r="E3" t="str">
-        <v>bob@test.com</v>
-      </c>
-      <c r="F3" t="str">
-        <v>555-1002</v>
-      </c>
-      <c r="I3" t="str">
-        <v>available</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B6"/>
   <sheetData>
     <row r="1">
@@ -821,7 +722,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D27"/>
   <sheetData>

</xml_diff>

<commit_message>
Add email preview to booking responses dialog
Adds email preview functionality to the booking responses dialog by updating the `booking-responses.tsx` component and allowing access to email preview endpoints without authentication.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: f123b9d7-6af8-472a-a75c-70d0b78d0583
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 7f0314a9-aae7-4a1c-9956-12eae9885136
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/4ca2a1f8-42ce-4303-beff-eb92e3283d4c/f123b9d7-6af8-472a-a75c-70d0b78d0583/H0vcR7T
</commit_message>
<xml_diff>
--- a/storage/backups/automatic-backup.xlsx
+++ b/storage/backups/automatic-backup.xlsx
@@ -4,8 +4,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Record Days" sheetId="1" r:id="rId1"/>
-    <sheet name="Groups" sheetId="2" r:id="rId2"/>
-    <sheet name="Block Types" sheetId="3" r:id="rId3"/>
+    <sheet name="Contestants" sheetId="2" r:id="rId2"/>
+    <sheet name="Seat Assignments" sheetId="3" r:id="rId3"/>
+    <sheet name="Groups" sheetId="4" r:id="rId4"/>
+    <sheet name="Block Types" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -665,65 +667,263 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:M3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>ID</v>
       </c>
       <c r="B1" t="str">
-        <v>ReferenceNumber</v>
+        <v>Name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Age</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Gender</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Email</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Phone</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Location</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Rating</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="J1" t="str">
+        <v>AttendingWith</v>
+      </c>
+      <c r="K1" t="str">
+        <v>GroupID</v>
+      </c>
+      <c r="L1" t="str">
+        <v>MedicalInfo</v>
+      </c>
+      <c r="M1" t="str">
+        <v>MobilityNotes</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>f25a6094-c1a5-4eb4-a709-1cc3d9b3ab5e</v>
+        <v>df1eee3b-9186-4dcb-8dff-b88f5ac053e5</v>
       </c>
       <c r="B2" t="str">
-        <v>GRP001</v>
+        <v>Kathleen Reynolds</v>
+      </c>
+      <c r="C2">
+        <v>33</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E2" t="str">
+        <v>kathleenmonicareynolds@gmail.com</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Footscray</v>
+      </c>
+      <c r="H2" t="str">
+        <v>A</v>
+      </c>
+      <c r="I2" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Peter Adamidis</v>
+      </c>
+      <c r="K2" t="str">
+        <v>44a98d78-5aac-4530-bb14-36dd87ed6cfb</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
+        <v>c9ff7c4e-e24d-43e0-844b-ccf99323c69a</v>
       </c>
       <c r="B3" t="str">
-        <v>GRP002</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>8c760df8-0e51-4b27-b1cb-0754c8b03595</v>
-      </c>
-      <c r="B4" t="str">
-        <v>AUTO-MK2NF2KE-kuoa</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>632fede5-4c1f-4f47-8a24-f4c94563915f</v>
-      </c>
-      <c r="B5" t="str">
-        <v>MANUAL-MKB8V43C</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>d5513a17-247e-49c4-be46-eca3c0aa0c4c</v>
-      </c>
-      <c r="B6" t="str">
-        <v>MANUAL-MKB952R9</v>
+        <v>Peter Adamidis</v>
+      </c>
+      <c r="C3">
+        <v>34</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E3" t="str">
+        <v>peter.adamidis@gmail.com</v>
+      </c>
+      <c r="F3" t="str">
+        <v>498086080</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Greenvale</v>
+      </c>
+      <c r="H3" t="str">
+        <v>B</v>
+      </c>
+      <c r="I3" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Kathleen Reynolds</v>
+      </c>
+      <c r="K3" t="str">
+        <v>44a98d78-5aac-4530-bb14-36dd87ed6cfb</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>RecordDayID</v>
+      </c>
+      <c r="C1" t="str">
+        <v>ContestantID</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Block</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Seat</v>
+      </c>
+      <c r="F1" t="str">
+        <v>BookingEmailSent</v>
+      </c>
+      <c r="G1" t="str">
+        <v>ConfirmedRSVP</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>32a65917-9e14-41de-8f93-c9049de2b2fa</v>
+      </c>
+      <c r="B2" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C2" t="str">
+        <v>df1eee3b-9186-4dcb-8dff-b88f5ac053e5</v>
+      </c>
+      <c r="D2">
+        <v>4</v>
+      </c>
+      <c r="E2" t="str">
+        <v>D2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>ed805d47-d9cc-43fe-b44b-d40e665ed5fd</v>
+      </c>
+      <c r="B3" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C3" t="str">
+        <v>c9ff7c4e-e24d-43e0-844b-ccf99323c69a</v>
+      </c>
+      <c r="D3">
+        <v>4</v>
+      </c>
+      <c r="E3" t="str">
+        <v>D3</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B7"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>ReferenceNumber</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>f25a6094-c1a5-4eb4-a709-1cc3d9b3ab5e</v>
+      </c>
+      <c r="B2" t="str">
+        <v>GRP001</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>6b341038-788f-4120-a2ca-16551bbc1d11</v>
+      </c>
+      <c r="B3" t="str">
+        <v>GRP002</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>8c760df8-0e51-4b27-b1cb-0754c8b03595</v>
+      </c>
+      <c r="B4" t="str">
+        <v>AUTO-MK2NF2KE-kuoa</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>632fede5-4c1f-4f47-8a24-f4c94563915f</v>
+      </c>
+      <c r="B5" t="str">
+        <v>MANUAL-MKB8V43C</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>d5513a17-247e-49c4-be46-eca3c0aa0c4c</v>
+      </c>
+      <c r="B6" t="str">
+        <v>MANUAL-MKB952R9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>44a98d78-5aac-4530-bb14-36dd87ed6cfb</v>
+      </c>
+      <c r="B7" t="str">
+        <v>GRP003</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D27"/>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Update contestant and standby data in backup file
Updates the 'exportedAt' timestamp and adds a new standby entry with associated contestant and record day data to the automatic backup file.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: f123b9d7-6af8-472a-a75c-70d0b78d0583
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: d9c2530a-66c7-42e5-81f9-a9164d136bf7
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/4ca2a1f8-42ce-4303-beff-eb92e3283d4c/f123b9d7-6af8-472a-a75c-70d0b78d0583/H0vcR7T
</commit_message>
<xml_diff>
--- a/storage/backups/automatic-backup.xlsx
+++ b/storage/backups/automatic-backup.xlsx
@@ -6,8 +6,9 @@
     <sheet name="Record Days" sheetId="1" r:id="rId1"/>
     <sheet name="Contestants" sheetId="2" r:id="rId2"/>
     <sheet name="Seat Assignments" sheetId="3" r:id="rId3"/>
-    <sheet name="Groups" sheetId="4" r:id="rId4"/>
-    <sheet name="Block Types" sheetId="5" r:id="rId5"/>
+    <sheet name="Standbys" sheetId="4" r:id="rId4"/>
+    <sheet name="Groups" sheetId="5" r:id="rId5"/>
+    <sheet name="Block Types" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -786,7 +787,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -831,31 +832,56 @@
         <v>D2</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>ed805d47-d9cc-43fe-b44b-d40e665ed5fd</v>
-      </c>
-      <c r="B3" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C3" t="str">
-        <v>c9ff7c4e-e24d-43e0-844b-ccf99323c69a</v>
-      </c>
-      <c r="D3">
-        <v>4</v>
-      </c>
-      <c r="E3" t="str">
-        <v>D3</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>RecordDayID</v>
+      </c>
+      <c r="C1" t="str">
+        <v>ContestantID</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>55f716f6-1aea-4732-b4ff-deb3b65a8203</v>
+      </c>
+      <c r="B2" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C2" t="str">
+        <v>c9ff7c4e-e24d-43e0-844b-ccf99323c69a</v>
+      </c>
+      <c r="D2" t="str">
+        <v>pending</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
   <sheetData>
@@ -922,7 +948,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D27"/>
   <sheetData>

</xml_diff>

<commit_message>
Add a toggle to filter and show only confirmed contestants
Adds a new state `filterConfirmedOnly` and a corresponding button to the Booking Master page. This allows users to filter the contestant list to display only those who have confirmed their RSVP. The filtering logic is integrated into the existing row filtering mechanism. The automatic backup file has been updated to reflect changes in seat assignments and standby data.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: f123b9d7-6af8-472a-a75c-70d0b78d0583
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: addfcc5b-ad56-4617-aea1-78b91d651777
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/4ca2a1f8-42ce-4303-beff-eb92e3283d4c/f123b9d7-6af8-472a-a75c-70d0b78d0583/H0vcR7T
</commit_message>
<xml_diff>
--- a/storage/backups/automatic-backup.xlsx
+++ b/storage/backups/automatic-backup.xlsx
@@ -6,9 +6,8 @@
     <sheet name="Record Days" sheetId="1" r:id="rId1"/>
     <sheet name="Contestants" sheetId="2" r:id="rId2"/>
     <sheet name="Seat Assignments" sheetId="3" r:id="rId3"/>
-    <sheet name="Standbys" sheetId="4" r:id="rId4"/>
-    <sheet name="Groups" sheetId="5" r:id="rId5"/>
-    <sheet name="Block Types" sheetId="6" r:id="rId6"/>
+    <sheet name="Groups" sheetId="4" r:id="rId4"/>
+    <sheet name="Block Types" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -787,7 +786,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -817,7 +816,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>32a65917-9e14-41de-8f93-c9049de2b2fa</v>
+        <v>70f80dcf-ade2-4f1d-abe5-ea68a6443a19</v>
       </c>
       <c r="B2" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
@@ -826,62 +825,37 @@
         <v>df1eee3b-9186-4dcb-8dff-b88f5ac053e5</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E2" t="str">
         <v>D2</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>c9f9f9a5-223f-43c1-92c6-0f0a39ad4ab7</v>
+      </c>
+      <c r="B3" t="str">
+        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
+      </c>
+      <c r="C3" t="str">
+        <v>c9ff7c4e-e24d-43e0-844b-ccf99323c69a</v>
+      </c>
+      <c r="D3">
+        <v>7</v>
+      </c>
+      <c r="E3" t="str">
+        <v>D3</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>ID</v>
-      </c>
-      <c r="B1" t="str">
-        <v>RecordDayID</v>
-      </c>
-      <c r="C1" t="str">
-        <v>ContestantID</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Notes</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>55f716f6-1aea-4732-b4ff-deb3b65a8203</v>
-      </c>
-      <c r="B2" t="str">
-        <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
-      </c>
-      <c r="C2" t="str">
-        <v>c9ff7c4e-e24d-43e0-844b-ccf99323c69a</v>
-      </c>
-      <c r="D2" t="str">
-        <v>pending</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
   <sheetData>
@@ -948,7 +922,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D27"/>
   <sheetData>

</xml_diff>

<commit_message>
Improve seating chart interaction by disabling seat hover info during drag
Introduce `isGlobalDragging` prop to conditionally disable `HoverCard` components within `SeatCard` when a drag operation is active, preventing hover information from appearing on seats while a contestant is being moved.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: f123b9d7-6af8-472a-a75c-70d0b78d0583
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: c750a603-e67b-4e0b-9ec4-ba25a4a90f4b
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/4ca2a1f8-42ce-4303-beff-eb92e3283d4c/f123b9d7-6af8-472a-a75c-70d0b78d0583/AeQHNWO
</commit_message>
<xml_diff>
--- a/storage/backups/automatic-backup.xlsx
+++ b/storage/backups/automatic-backup.xlsx
@@ -16558,7 +16558,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D28"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -16912,10 +16912,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>badc1981-587e-4ebe-a4ca-d09f25a98a6b</v>
+        <v>4024cdf1-46c9-4af4-b451-6e106c607a2e</v>
       </c>
       <c r="B26" t="str">
-        <v>eec54567-3e21-424c-8d62-28772c0a6c25</v>
+        <v>59f9cd94-162d-413c-9797-5a881676a706</v>
       </c>
       <c r="C26">
         <v>1</v>
@@ -16926,21 +16926,35 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>321d3111-fcc3-4246-8800-231133dd823d</v>
+        <v>badc1981-587e-4ebe-a4ca-d09f25a98a6b</v>
       </c>
       <c r="B27" t="str">
         <v>eec54567-3e21-424c-8d62-28772c0a6c25</v>
       </c>
       <c r="C27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D27" t="str">
         <v>PB</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>321d3111-fcc3-4246-8800-231133dd823d</v>
+      </c>
+      <c r="B28" t="str">
+        <v>eec54567-3e21-424c-8d62-28772c0a6c25</v>
+      </c>
+      <c r="C28">
+        <v>2</v>
+      </c>
+      <c r="D28" t="str">
+        <v>PB</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D28"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Restore contestant data to the backup file after accidental removal
Restore a deleted contestant record in the automatic backup JSON file and update the exported timestamp.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: f123b9d7-6af8-472a-a75c-70d0b78d0583
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: a0260c25-e3d4-497c-aad9-733b39461f66
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/4ca2a1f8-42ce-4303-beff-eb92e3283d4c/f123b9d7-6af8-472a-a75c-70d0b78d0583/VkaJ7eU
</commit_message>
<xml_diff>
--- a/storage/backups/automatic-backup.xlsx
+++ b/storage/backups/automatic-backup.xlsx
@@ -15195,342 +15195,342 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>70f80dcf-ade2-4f1d-abe5-ea68a6443a19</v>
+        <v>c9f9f9a5-223f-43c1-92c6-0f0a39ad4ab7</v>
       </c>
       <c r="B2" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C2" t="str">
-        <v>df1eee3b-9186-4dcb-8dff-b88f5ac053e5</v>
+        <v>c9ff7c4e-e24d-43e0-844b-ccf99323c69a</v>
       </c>
       <c r="D2">
         <v>7</v>
       </c>
       <c r="E2" t="str">
-        <v>D2</v>
+        <v>D3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>c9f9f9a5-223f-43c1-92c6-0f0a39ad4ab7</v>
+        <v>20e92b66-46e9-4eb7-80cf-b20ed2afa92c</v>
       </c>
       <c r="B3" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C3" t="str">
-        <v>c9ff7c4e-e24d-43e0-844b-ccf99323c69a</v>
+        <v>1373bff6-1fa6-4e22-a5be-810587cb7056</v>
       </c>
       <c r="D3">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E3" t="str">
-        <v>D3</v>
+        <v>B1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>20e92b66-46e9-4eb7-80cf-b20ed2afa92c</v>
+        <v>d7d0a055-b2d4-4231-84ba-3a6049c57715</v>
       </c>
       <c r="B4" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C4" t="str">
-        <v>1373bff6-1fa6-4e22-a5be-810587cb7056</v>
+        <v>c2568561-9563-4f98-83f7-0658e14bed36</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
       <c r="E4" t="str">
-        <v>B1</v>
+        <v>B2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>d7d0a055-b2d4-4231-84ba-3a6049c57715</v>
+        <v>3a8396e9-22fd-4db5-b8d3-a791ee3f206e</v>
       </c>
       <c r="B5" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C5" t="str">
-        <v>c2568561-9563-4f98-83f7-0658e14bed36</v>
+        <v>f066c255-163d-4c17-8441-e7673d2646f3</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
       <c r="E5" t="str">
-        <v>B2</v>
+        <v>B3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>3a8396e9-22fd-4db5-b8d3-a791ee3f206e</v>
+        <v>52696136-4d33-47a1-9605-aae3f328c29d</v>
       </c>
       <c r="B6" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C6" t="str">
-        <v>f066c255-163d-4c17-8441-e7673d2646f3</v>
+        <v>16a56913-24a5-4bd8-9c45-78f2ae55a11d</v>
       </c>
       <c r="D6">
         <v>1</v>
       </c>
       <c r="E6" t="str">
-        <v>B3</v>
+        <v>B4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>52696136-4d33-47a1-9605-aae3f328c29d</v>
+        <v>bae99a6d-aa62-4e41-9a56-54aaf7d037d3</v>
       </c>
       <c r="B7" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C7" t="str">
-        <v>16a56913-24a5-4bd8-9c45-78f2ae55a11d</v>
+        <v>c4a59423-d8ff-4b63-aa35-62c78b050663</v>
       </c>
       <c r="D7">
         <v>1</v>
       </c>
       <c r="E7" t="str">
-        <v>B4</v>
+        <v>C1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>bae99a6d-aa62-4e41-9a56-54aaf7d037d3</v>
+        <v>33778eb7-9030-4fea-b9c6-b2a4cf28b7ad</v>
       </c>
       <c r="B8" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C8" t="str">
-        <v>c4a59423-d8ff-4b63-aa35-62c78b050663</v>
+        <v>3c4c0dd0-e98b-449e-b2fe-38d8927a3f3a</v>
       </c>
       <c r="D8">
         <v>1</v>
       </c>
       <c r="E8" t="str">
-        <v>C1</v>
+        <v>C2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>33778eb7-9030-4fea-b9c6-b2a4cf28b7ad</v>
+        <v>ed2c1c4b-610a-4f9c-92f8-353df202c677</v>
       </c>
       <c r="B9" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C9" t="str">
-        <v>3c4c0dd0-e98b-449e-b2fe-38d8927a3f3a</v>
+        <v>0ac07194-cfd3-43c3-93a4-e21b0470f833</v>
       </c>
       <c r="D9">
         <v>1</v>
       </c>
       <c r="E9" t="str">
-        <v>C2</v>
+        <v>C3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>ed2c1c4b-610a-4f9c-92f8-353df202c677</v>
+        <v>7fe3b0ab-fa8c-4993-b046-89982206ff8d</v>
       </c>
       <c r="B10" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C10" t="str">
-        <v>0ac07194-cfd3-43c3-93a4-e21b0470f833</v>
+        <v>65a7d185-32fb-4518-96c6-a8b8a0314939</v>
       </c>
       <c r="D10">
         <v>1</v>
       </c>
       <c r="E10" t="str">
-        <v>C3</v>
+        <v>D3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>7fe3b0ab-fa8c-4993-b046-89982206ff8d</v>
+        <v>033e9966-1308-4b1e-9c87-7198d93b3c0f</v>
       </c>
       <c r="B11" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C11" t="str">
-        <v>65a7d185-32fb-4518-96c6-a8b8a0314939</v>
+        <v>b42f2517-90d3-4c2e-aec1-7338c18cd14f</v>
       </c>
       <c r="D11">
         <v>1</v>
       </c>
       <c r="E11" t="str">
-        <v>D3</v>
+        <v>D4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>033e9966-1308-4b1e-9c87-7198d93b3c0f</v>
+        <v>d79f293f-1b26-4443-ac34-382a81fd09f3</v>
       </c>
       <c r="B12" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C12" t="str">
-        <v>b42f2517-90d3-4c2e-aec1-7338c18cd14f</v>
+        <v>8cb8a9bf-a712-4ad3-b537-f0eebc912e58</v>
       </c>
       <c r="D12">
         <v>1</v>
       </c>
       <c r="E12" t="str">
-        <v>D4</v>
+        <v>E1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>d79f293f-1b26-4443-ac34-382a81fd09f3</v>
+        <v>49e57d2c-e52e-43d6-8105-8f8f87cd393e</v>
       </c>
       <c r="B13" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C13" t="str">
-        <v>8cb8a9bf-a712-4ad3-b537-f0eebc912e58</v>
+        <v>5fb55209-4753-4095-b21f-a62a5c711d7d</v>
       </c>
       <c r="D13">
         <v>1</v>
       </c>
       <c r="E13" t="str">
-        <v>E1</v>
+        <v>E2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>49e57d2c-e52e-43d6-8105-8f8f87cd393e</v>
+        <v>3034a004-0f03-4137-bb27-d11448c0abdb</v>
       </c>
       <c r="B14" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C14" t="str">
-        <v>5fb55209-4753-4095-b21f-a62a5c711d7d</v>
+        <v>034c094f-f76d-434f-8b89-909c23c8ad42</v>
       </c>
       <c r="D14">
         <v>1</v>
       </c>
       <c r="E14" t="str">
-        <v>E2</v>
+        <v>E3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>3034a004-0f03-4137-bb27-d11448c0abdb</v>
+        <v>592fd454-318d-40aa-9e12-d3e6036e2e34</v>
       </c>
       <c r="B15" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C15" t="str">
-        <v>034c094f-f76d-434f-8b89-909c23c8ad42</v>
+        <v>c37d275c-1560-4d86-9b7a-22963f478a91</v>
       </c>
       <c r="D15">
         <v>1</v>
       </c>
       <c r="E15" t="str">
-        <v>E3</v>
+        <v>E4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>592fd454-318d-40aa-9e12-d3e6036e2e34</v>
+        <v>4f2e9b92-f970-4f97-a5bf-31b2204c6dbb</v>
       </c>
       <c r="B16" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C16" t="str">
-        <v>c37d275c-1560-4d86-9b7a-22963f478a91</v>
+        <v>71d827af-973f-4c3a-a074-dd419b4a9c27</v>
       </c>
       <c r="D16">
         <v>1</v>
       </c>
       <c r="E16" t="str">
-        <v>E4</v>
+        <v>A1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>4f2e9b92-f970-4f97-a5bf-31b2204c6dbb</v>
+        <v>32d58a77-f34a-4cd2-b9a7-559df3c555d1</v>
       </c>
       <c r="B17" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C17" t="str">
-        <v>71d827af-973f-4c3a-a074-dd419b4a9c27</v>
+        <v>7f88f66e-bf77-4937-bfe1-44d447960afc</v>
       </c>
       <c r="D17">
         <v>1</v>
       </c>
       <c r="E17" t="str">
-        <v>A1</v>
+        <v>A2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>32d58a77-f34a-4cd2-b9a7-559df3c555d1</v>
+        <v>9d49646c-54a0-43cc-b5a8-9a42788aaf6f</v>
       </c>
       <c r="B18" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C18" t="str">
-        <v>7f88f66e-bf77-4937-bfe1-44d447960afc</v>
+        <v>9520e1b4-1889-4925-9628-eb625555036c</v>
       </c>
       <c r="D18">
         <v>1</v>
       </c>
       <c r="E18" t="str">
-        <v>A2</v>
+        <v>A3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>9d49646c-54a0-43cc-b5a8-9a42788aaf6f</v>
+        <v>3411d007-571a-484a-a508-360fe9c6c33e</v>
       </c>
       <c r="B19" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C19" t="str">
-        <v>9520e1b4-1889-4925-9628-eb625555036c</v>
+        <v>293e11eb-227f-4247-8788-b270b2af2d63</v>
       </c>
       <c r="D19">
         <v>1</v>
       </c>
       <c r="E19" t="str">
-        <v>A3</v>
+        <v>B5</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>3411d007-571a-484a-a508-360fe9c6c33e</v>
+        <v>2457f5d9-ae65-4242-ab9c-2fb3902296fb</v>
       </c>
       <c r="B20" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C20" t="str">
-        <v>293e11eb-227f-4247-8788-b270b2af2d63</v>
+        <v>efcb7955-b4bc-487b-b45b-02a50d7f5ba2</v>
       </c>
       <c r="D20">
         <v>1</v>
       </c>
       <c r="E20" t="str">
-        <v>B5</v>
+        <v>C4</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2457f5d9-ae65-4242-ab9c-2fb3902296fb</v>
+        <v>70f80dcf-ade2-4f1d-abe5-ea68a6443a19</v>
       </c>
       <c r="B21" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C21" t="str">
-        <v>efcb7955-b4bc-487b-b45b-02a50d7f5ba2</v>
+        <v>df1eee3b-9186-4dcb-8dff-b88f5ac053e5</v>
       </c>
       <c r="D21">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E21" t="str">
-        <v>C4</v>
+        <v>D2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add casting card upload and management functionality for players
Integrates a new feature allowing users to upload, view, and delete casting cards for player assignments. This involves adding a `castingCardUrl` field to the `SeatAssignment` interface, implementing mutations for card upload and deletion, and updating the player card display to include relevant buttons. The backend API for handling casting card uploads via FormData has also been considered.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: f123b9d7-6af8-472a-a75c-70d0b78d0583
Replit-Commit-Checkpoint-Type: intermediate_checkpoint
Replit-Commit-Event-Id: effecaf5-e601-4157-bec9-28bec50f3ed0
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/4ca2a1f8-42ce-4303-beff-eb92e3283d4c/f123b9d7-6af8-472a-a75c-70d0b78d0583/782Yg2o
</commit_message>
<xml_diff>
--- a/storage/backups/automatic-backup.xlsx
+++ b/storage/backups/automatic-backup.xlsx
@@ -712,25 +712,25 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>9528376e-b4d9-4b58-87ac-757ac76c3509</v>
+        <v>97ce0b2a-8b18-4079-8405-31b1a13ffdab</v>
       </c>
       <c r="B2" t="str">
-        <v>Michelle  Richardson</v>
+        <v>Chelsea  Fanning</v>
       </c>
       <c r="C2">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="D2" t="str">
         <v>Female</v>
       </c>
       <c r="E2" t="str">
-        <v>mrichardson17@outlook.com.au</v>
+        <v>cmaryf01@icloud.com</v>
       </c>
       <c r="F2" t="str">
-        <v>0459150497</v>
+        <v>0401507791</v>
       </c>
       <c r="G2" t="str">
-        <v>Portland</v>
+        <v xml:space="preserve">Gladstone </v>
       </c>
       <c r="H2" t="str">
         <v>B+</v>
@@ -739,33 +739,33 @@
         <v>available</v>
       </c>
       <c r="J2" t="str">
-        <v>Chelsea Fanning</v>
+        <v>Michelle Richardson</v>
       </c>
       <c r="K2" t="str">
         <v>64c49e8a-746f-4336-b779-194a3e136339</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" xml:space="preserve">
       <c r="A3" t="str">
-        <v>97ce0b2a-8b18-4079-8405-31b1a13ffdab</v>
+        <v>2da73fbf-9373-4a15-98b4-1dc259db08b0</v>
       </c>
       <c r="B3" t="str">
-        <v>Chelsea  Fanning</v>
+        <v>Sandra  Anderson</v>
       </c>
       <c r="C3">
-        <v>24</v>
+        <v>79</v>
       </c>
       <c r="D3" t="str">
         <v>Female</v>
       </c>
       <c r="E3" t="str">
-        <v>cmaryf01@icloud.com</v>
+        <v>mathewsally1c@gmail.com</v>
       </c>
       <c r="F3" t="str">
-        <v>0401507791</v>
+        <v>0439352004</v>
       </c>
       <c r="G3" t="str">
-        <v xml:space="preserve">Gladstone </v>
+        <v xml:space="preserve">Dromana </v>
       </c>
       <c r="H3" t="str">
         <v>B+</v>
@@ -773,34 +773,38 @@
       <c r="I3" t="str">
         <v>available</v>
       </c>
-      <c r="J3" t="str">
-        <v>Michelle Richardson</v>
+      <c r="J3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jessy Brown
+Matilda Davis
+Colin Anderson
+Sandra Anderson
+Sally Davis</v>
       </c>
       <c r="K3" t="str">
-        <v>64c49e8a-746f-4336-b779-194a3e136339</v>
+        <v>1b3b852f-d9f5-491a-86d6-2ebe1fdac3f9</v>
       </c>
     </row>
     <row r="4" xml:space="preserve">
       <c r="A4" t="str">
-        <v>2da73fbf-9373-4a15-98b4-1dc259db08b0</v>
+        <v>ef612e09-b066-4880-a01c-1aa0836a93aa</v>
       </c>
       <c r="B4" t="str">
-        <v>Sandra  Anderson</v>
+        <v>Sally Davis</v>
       </c>
       <c r="C4">
-        <v>79</v>
+        <v>57</v>
       </c>
       <c r="D4" t="str">
         <v>Female</v>
       </c>
       <c r="E4" t="str">
-        <v>mathewsally1c@gmail.com</v>
+        <v>matsal1c@bigpond.com</v>
       </c>
       <c r="F4" t="str">
-        <v>0439352004</v>
+        <v>0434871103</v>
       </c>
       <c r="G4" t="str">
-        <v xml:space="preserve">Dromana </v>
+        <v>My Martha</v>
       </c>
       <c r="H4" t="str">
         <v>B+</v>
@@ -819,66 +823,59 @@
         <v>1b3b852f-d9f5-491a-86d6-2ebe1fdac3f9</v>
       </c>
     </row>
-    <row r="5" xml:space="preserve">
+    <row r="5">
       <c r="A5" t="str">
-        <v>ef612e09-b066-4880-a01c-1aa0836a93aa</v>
+        <v>71d827af-973f-4c3a-a074-dd419b4a9c27</v>
       </c>
       <c r="B5" t="str">
-        <v>Sally Davis</v>
+        <v>Angela Verspay</v>
       </c>
       <c r="C5">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="D5" t="str">
         <v>Female</v>
       </c>
       <c r="E5" t="str">
-        <v>matsal1c@bigpond.com</v>
+        <v>angelarileysmyth@hotmail.com</v>
       </c>
       <c r="F5" t="str">
-        <v>0434871103</v>
+        <v>0477660119</v>
       </c>
       <c r="G5" t="str">
-        <v>My Martha</v>
+        <v>Warrnambool</v>
       </c>
       <c r="H5" t="str">
-        <v>B+</v>
+        <v>B</v>
       </c>
       <c r="I5" t="str">
-        <v>available</v>
-      </c>
-      <c r="J5" t="str" xml:space="preserve">
-        <v xml:space="preserve">Jessy Brown
-Matilda Davis
-Colin Anderson
-Sandra Anderson
-Sally Davis</v>
-      </c>
-      <c r="K5" t="str">
-        <v>1b3b852f-d9f5-491a-86d6-2ebe1fdac3f9</v>
+        <v>assigned</v>
+      </c>
+      <c r="J5" t="str">
+        <v>SOLO</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>71d827af-973f-4c3a-a074-dd419b4a9c27</v>
+        <v>c9ff7c4e-e24d-43e0-844b-ccf99323c69a</v>
       </c>
       <c r="B6" t="str">
-        <v>Angela Verspay</v>
+        <v>Peter Adamidis</v>
       </c>
       <c r="C6">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="D6" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E6" t="str">
-        <v>angelarileysmyth@hotmail.com</v>
+        <v>peter.adamidis@gmail.com</v>
       </c>
       <c r="F6" t="str">
-        <v>0477660119</v>
+        <v>0498086080</v>
       </c>
       <c r="G6" t="str">
-        <v>Warrnambool</v>
+        <v>Greenvale</v>
       </c>
       <c r="H6" t="str">
         <v>B</v>
@@ -887,65 +884,68 @@
         <v>assigned</v>
       </c>
       <c r="J6" t="str">
-        <v>SOLO</v>
+        <v>Kathleen Reynolds</v>
+      </c>
+      <c r="K6" t="str">
+        <v>44a98d78-5aac-4530-bb14-36dd87ed6cfb</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>c9ff7c4e-e24d-43e0-844b-ccf99323c69a</v>
+        <v>08958291-6c32-49d6-a9ef-1aa84b760b54</v>
       </c>
       <c r="B7" t="str">
-        <v>Peter Adamidis</v>
+        <v>Brent Barnett</v>
       </c>
       <c r="C7">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D7" t="str">
         <v>Male</v>
       </c>
       <c r="E7" t="str">
-        <v>peter.adamidis@gmail.com</v>
+        <v>brentbarnett88@gmail.com</v>
       </c>
       <c r="F7" t="str">
-        <v>0498086080</v>
+        <v>0423530043</v>
       </c>
       <c r="G7" t="str">
-        <v>Greenvale</v>
+        <v>Preston</v>
       </c>
       <c r="H7" t="str">
-        <v>B</v>
+        <v>B+</v>
       </c>
       <c r="I7" t="str">
-        <v>assigned</v>
+        <v>available</v>
       </c>
       <c r="J7" t="str">
-        <v>Kathleen Reynolds</v>
+        <v>Stephanie Squillacioti</v>
       </c>
       <c r="K7" t="str">
-        <v>44a98d78-5aac-4530-bb14-36dd87ed6cfb</v>
+        <v>9b12e80e-a626-4481-95b4-484e64b6f474</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>08958291-6c32-49d6-a9ef-1aa84b760b54</v>
+        <v>5e33fa3c-fe11-46d0-89b0-09389e33b12f</v>
       </c>
       <c r="B8" t="str">
-        <v>Brent Barnett</v>
+        <v>Tara Saltzman</v>
       </c>
       <c r="C8">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="D8" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E8" t="str">
-        <v>brentbarnett88@gmail.com</v>
+        <v>tarasaltzman@bigpond.com</v>
       </c>
       <c r="F8" t="str">
-        <v>0423530043</v>
+        <v>0448545599</v>
       </c>
       <c r="G8" t="str">
-        <v>Preston</v>
+        <v>Melbourne</v>
       </c>
       <c r="H8" t="str">
         <v>B+</v>
@@ -954,33 +954,30 @@
         <v>available</v>
       </c>
       <c r="J8" t="str">
-        <v>Stephanie Squillacioti</v>
-      </c>
-      <c r="K8" t="str">
-        <v>9b12e80e-a626-4481-95b4-484e64b6f474</v>
+        <v xml:space="preserve">JACK AGIUS - NEEDS TO DO APPLICATION </v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>5e33fa3c-fe11-46d0-89b0-09389e33b12f</v>
+        <v>01eae1ca-b0d3-4b95-8800-b73c7ccd999f</v>
       </c>
       <c r="B9" t="str">
-        <v>Tara Saltzman</v>
+        <v>Karina  Richmond</v>
       </c>
       <c r="C9">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="D9" t="str">
         <v>Female</v>
       </c>
       <c r="E9" t="str">
-        <v>tarasaltzman@bigpond.com</v>
+        <v>richmondkarina@yahoo.com</v>
       </c>
       <c r="F9" t="str">
-        <v>0448545599</v>
+        <v>0400554609</v>
       </c>
       <c r="G9" t="str">
-        <v>Melbourne</v>
+        <v>Newcomb</v>
       </c>
       <c r="H9" t="str">
         <v>B+</v>
@@ -989,30 +986,30 @@
         <v>available</v>
       </c>
       <c r="J9" t="str">
-        <v xml:space="preserve">JACK AGIUS - NEEDS TO DO APPLICATION </v>
+        <v>AMY DILLON</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>01eae1ca-b0d3-4b95-8800-b73c7ccd999f</v>
+        <v>9cea8138-f43e-49b8-b2c7-849645bf2a59</v>
       </c>
       <c r="B10" t="str">
-        <v>Karina  Richmond</v>
+        <v>Troy Smith</v>
       </c>
       <c r="C10">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="D10" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E10" t="str">
-        <v>richmondkarina@yahoo.com</v>
+        <v>Troyssmith94@gmail.com</v>
       </c>
       <c r="F10" t="str">
-        <v>0400554609</v>
+        <v>0429354308</v>
       </c>
       <c r="G10" t="str">
-        <v>Newcomb</v>
+        <v>Melbourne</v>
       </c>
       <c r="H10" t="str">
         <v>B+</v>
@@ -1021,30 +1018,33 @@
         <v>available</v>
       </c>
       <c r="J10" t="str">
-        <v>AMY DILLON</v>
+        <v>Tayla Huxtable</v>
+      </c>
+      <c r="L10" t="str">
+        <v xml:space="preserve">Peanut allergy </v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>9cea8138-f43e-49b8-b2c7-849645bf2a59</v>
+        <v>e64cdfc2-e9c8-4ab5-84e1-c4b636b79efb</v>
       </c>
       <c r="B11" t="str">
-        <v>Troy Smith</v>
+        <v>Deb  Jones</v>
       </c>
       <c r="C11">
-        <v>31</v>
+        <v>66</v>
       </c>
       <c r="D11" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E11" t="str">
-        <v>Troyssmith94@gmail.com</v>
+        <v>fullhouse5@optusnet.com.au</v>
       </c>
       <c r="F11" t="str">
-        <v>0429354308</v>
+        <v>0438561474</v>
       </c>
       <c r="G11" t="str">
-        <v>Melbourne</v>
+        <v>Bayswater North</v>
       </c>
       <c r="H11" t="str">
         <v>B+</v>
@@ -1053,33 +1053,36 @@
         <v>available</v>
       </c>
       <c r="J11" t="str">
-        <v>Tayla Huxtable</v>
-      </c>
-      <c r="L11" t="str">
-        <v xml:space="preserve">Peanut allergy </v>
+        <v>Daryl Jones</v>
+      </c>
+      <c r="K11" t="str">
+        <v>3bd0ea54-9969-49c7-af92-796fd54643e7</v>
+      </c>
+      <c r="M11" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>e64cdfc2-e9c8-4ab5-84e1-c4b636b79efb</v>
+        <v>3d46906e-68f4-44ae-a430-a3225a7be977</v>
       </c>
       <c r="B12" t="str">
-        <v>Deb  Jones</v>
+        <v>Philip Natoli</v>
       </c>
       <c r="C12">
-        <v>66</v>
+        <v>29</v>
       </c>
       <c r="D12" t="str">
-        <v>Female</v>
+        <v>Male</v>
       </c>
       <c r="E12" t="str">
-        <v>fullhouse5@optusnet.com.au</v>
+        <v>Philip.natoli@outlook.com</v>
       </c>
       <c r="F12" t="str">
-        <v>0438561474</v>
+        <v>0466021882</v>
       </c>
       <c r="G12" t="str">
-        <v>Bayswater North</v>
+        <v>Caulfield South</v>
       </c>
       <c r="H12" t="str">
         <v>B+</v>
@@ -1088,48 +1091,51 @@
         <v>available</v>
       </c>
       <c r="J12" t="str">
-        <v>Daryl Jones</v>
+        <v>Hayley Wright</v>
       </c>
       <c r="K12" t="str">
-        <v>3bd0ea54-9969-49c7-af92-796fd54643e7</v>
-      </c>
-      <c r="M12" t="str">
-        <v>No</v>
+        <v>7989cb62-884e-4e52-a28b-cca0e64f2a6f</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>3d46906e-68f4-44ae-a430-a3225a7be977</v>
+        <v>9528376e-b4d9-4b58-87ac-757ac76c3509</v>
       </c>
       <c r="B13" t="str">
-        <v>Philip Natoli</v>
+        <v>Michelle  Richardson</v>
       </c>
       <c r="C13">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D13" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="E13" t="str">
-        <v>Philip.natoli@outlook.com</v>
+        <v>mrichardson17@outlook.com.au</v>
       </c>
       <c r="F13" t="str">
-        <v>0466021882</v>
+        <v>0459150497</v>
       </c>
       <c r="G13" t="str">
-        <v>Caulfield South</v>
+        <v>Portland</v>
       </c>
       <c r="H13" t="str">
-        <v>B+</v>
+        <v>A</v>
       </c>
       <c r="I13" t="str">
         <v>available</v>
       </c>
       <c r="J13" t="str">
-        <v>Hayley Wright</v>
+        <v>Chelsea Fanning</v>
       </c>
       <c r="K13" t="str">
-        <v>7989cb62-884e-4e52-a28b-cca0e64f2a6f</v>
+        <v>64c49e8a-746f-4336-b779-194a3e136339</v>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v/>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
Improve editing experience for contestant notes on hover cards
Modifies the client/src/components/seat-card.tsx component to require a click on an edit button to modify the notes field in hover cards, preventing accidental edits during hover. Updates the backup file storage/backups/automatic-backup.json to reflect the changes.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: f123b9d7-6af8-472a-a75c-70d0b78d0583
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 2ef89f66-c092-45b2-84dd-c95c98a0ca5c
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/4ca2a1f8-42ce-4303-beff-eb92e3283d4c/f123b9d7-6af8-472a-a75c-70d0b78d0583/782Yg2o
</commit_message>
<xml_diff>
--- a/storage/backups/automatic-backup.xlsx
+++ b/storage/backups/automatic-backup.xlsx
@@ -15201,342 +15201,342 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>c9f9f9a5-223f-43c1-92c6-0f0a39ad4ab7</v>
+        <v>70f80dcf-ade2-4f1d-abe5-ea68a6443a19</v>
       </c>
       <c r="B2" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C2" t="str">
-        <v>c9ff7c4e-e24d-43e0-844b-ccf99323c69a</v>
+        <v>df1eee3b-9186-4dcb-8dff-b88f5ac053e5</v>
       </c>
       <c r="D2">
         <v>7</v>
       </c>
       <c r="E2" t="str">
-        <v>D3</v>
+        <v>D2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>20e92b66-46e9-4eb7-80cf-b20ed2afa92c</v>
+        <v>c9f9f9a5-223f-43c1-92c6-0f0a39ad4ab7</v>
       </c>
       <c r="B3" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C3" t="str">
-        <v>1373bff6-1fa6-4e22-a5be-810587cb7056</v>
+        <v>c9ff7c4e-e24d-43e0-844b-ccf99323c69a</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E3" t="str">
-        <v>B1</v>
+        <v>D3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>d7d0a055-b2d4-4231-84ba-3a6049c57715</v>
+        <v>20e92b66-46e9-4eb7-80cf-b20ed2afa92c</v>
       </c>
       <c r="B4" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C4" t="str">
-        <v>c2568561-9563-4f98-83f7-0658e14bed36</v>
+        <v>1373bff6-1fa6-4e22-a5be-810587cb7056</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
       <c r="E4" t="str">
-        <v>B2</v>
+        <v>B1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>3a8396e9-22fd-4db5-b8d3-a791ee3f206e</v>
+        <v>d7d0a055-b2d4-4231-84ba-3a6049c57715</v>
       </c>
       <c r="B5" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C5" t="str">
-        <v>f066c255-163d-4c17-8441-e7673d2646f3</v>
+        <v>c2568561-9563-4f98-83f7-0658e14bed36</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
       <c r="E5" t="str">
-        <v>B3</v>
+        <v>B2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>52696136-4d33-47a1-9605-aae3f328c29d</v>
+        <v>3a8396e9-22fd-4db5-b8d3-a791ee3f206e</v>
       </c>
       <c r="B6" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C6" t="str">
-        <v>16a56913-24a5-4bd8-9c45-78f2ae55a11d</v>
+        <v>f066c255-163d-4c17-8441-e7673d2646f3</v>
       </c>
       <c r="D6">
         <v>1</v>
       </c>
       <c r="E6" t="str">
-        <v>B4</v>
+        <v>B3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>bae99a6d-aa62-4e41-9a56-54aaf7d037d3</v>
+        <v>52696136-4d33-47a1-9605-aae3f328c29d</v>
       </c>
       <c r="B7" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C7" t="str">
-        <v>c4a59423-d8ff-4b63-aa35-62c78b050663</v>
+        <v>16a56913-24a5-4bd8-9c45-78f2ae55a11d</v>
       </c>
       <c r="D7">
         <v>1</v>
       </c>
       <c r="E7" t="str">
-        <v>C1</v>
+        <v>B4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>33778eb7-9030-4fea-b9c6-b2a4cf28b7ad</v>
+        <v>bae99a6d-aa62-4e41-9a56-54aaf7d037d3</v>
       </c>
       <c r="B8" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C8" t="str">
-        <v>3c4c0dd0-e98b-449e-b2fe-38d8927a3f3a</v>
+        <v>c4a59423-d8ff-4b63-aa35-62c78b050663</v>
       </c>
       <c r="D8">
         <v>1</v>
       </c>
       <c r="E8" t="str">
-        <v>C2</v>
+        <v>C1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ed2c1c4b-610a-4f9c-92f8-353df202c677</v>
+        <v>33778eb7-9030-4fea-b9c6-b2a4cf28b7ad</v>
       </c>
       <c r="B9" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C9" t="str">
-        <v>0ac07194-cfd3-43c3-93a4-e21b0470f833</v>
+        <v>3c4c0dd0-e98b-449e-b2fe-38d8927a3f3a</v>
       </c>
       <c r="D9">
         <v>1</v>
       </c>
       <c r="E9" t="str">
-        <v>C3</v>
+        <v>C2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>7fe3b0ab-fa8c-4993-b046-89982206ff8d</v>
+        <v>ed2c1c4b-610a-4f9c-92f8-353df202c677</v>
       </c>
       <c r="B10" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C10" t="str">
-        <v>65a7d185-32fb-4518-96c6-a8b8a0314939</v>
+        <v>0ac07194-cfd3-43c3-93a4-e21b0470f833</v>
       </c>
       <c r="D10">
         <v>1</v>
       </c>
       <c r="E10" t="str">
-        <v>D3</v>
+        <v>C3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>033e9966-1308-4b1e-9c87-7198d93b3c0f</v>
+        <v>7fe3b0ab-fa8c-4993-b046-89982206ff8d</v>
       </c>
       <c r="B11" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C11" t="str">
-        <v>b42f2517-90d3-4c2e-aec1-7338c18cd14f</v>
+        <v>65a7d185-32fb-4518-96c6-a8b8a0314939</v>
       </c>
       <c r="D11">
         <v>1</v>
       </c>
       <c r="E11" t="str">
-        <v>D4</v>
+        <v>D3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>d79f293f-1b26-4443-ac34-382a81fd09f3</v>
+        <v>033e9966-1308-4b1e-9c87-7198d93b3c0f</v>
       </c>
       <c r="B12" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C12" t="str">
-        <v>8cb8a9bf-a712-4ad3-b537-f0eebc912e58</v>
+        <v>b42f2517-90d3-4c2e-aec1-7338c18cd14f</v>
       </c>
       <c r="D12">
         <v>1</v>
       </c>
       <c r="E12" t="str">
-        <v>E1</v>
+        <v>D4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>49e57d2c-e52e-43d6-8105-8f8f87cd393e</v>
+        <v>d79f293f-1b26-4443-ac34-382a81fd09f3</v>
       </c>
       <c r="B13" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C13" t="str">
-        <v>5fb55209-4753-4095-b21f-a62a5c711d7d</v>
+        <v>8cb8a9bf-a712-4ad3-b537-f0eebc912e58</v>
       </c>
       <c r="D13">
         <v>1</v>
       </c>
       <c r="E13" t="str">
-        <v>E2</v>
+        <v>E1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>3034a004-0f03-4137-bb27-d11448c0abdb</v>
+        <v>49e57d2c-e52e-43d6-8105-8f8f87cd393e</v>
       </c>
       <c r="B14" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C14" t="str">
-        <v>034c094f-f76d-434f-8b89-909c23c8ad42</v>
+        <v>5fb55209-4753-4095-b21f-a62a5c711d7d</v>
       </c>
       <c r="D14">
         <v>1</v>
       </c>
       <c r="E14" t="str">
-        <v>E3</v>
+        <v>E2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>592fd454-318d-40aa-9e12-d3e6036e2e34</v>
+        <v>3034a004-0f03-4137-bb27-d11448c0abdb</v>
       </c>
       <c r="B15" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C15" t="str">
-        <v>c37d275c-1560-4d86-9b7a-22963f478a91</v>
+        <v>034c094f-f76d-434f-8b89-909c23c8ad42</v>
       </c>
       <c r="D15">
         <v>1</v>
       </c>
       <c r="E15" t="str">
-        <v>E4</v>
+        <v>E3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>4f2e9b92-f970-4f97-a5bf-31b2204c6dbb</v>
+        <v>592fd454-318d-40aa-9e12-d3e6036e2e34</v>
       </c>
       <c r="B16" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C16" t="str">
-        <v>71d827af-973f-4c3a-a074-dd419b4a9c27</v>
+        <v>c37d275c-1560-4d86-9b7a-22963f478a91</v>
       </c>
       <c r="D16">
         <v>1</v>
       </c>
       <c r="E16" t="str">
-        <v>A1</v>
+        <v>E4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>32d58a77-f34a-4cd2-b9a7-559df3c555d1</v>
+        <v>4f2e9b92-f970-4f97-a5bf-31b2204c6dbb</v>
       </c>
       <c r="B17" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C17" t="str">
-        <v>7f88f66e-bf77-4937-bfe1-44d447960afc</v>
+        <v>71d827af-973f-4c3a-a074-dd419b4a9c27</v>
       </c>
       <c r="D17">
         <v>1</v>
       </c>
       <c r="E17" t="str">
-        <v>A2</v>
+        <v>A1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>9d49646c-54a0-43cc-b5a8-9a42788aaf6f</v>
+        <v>32d58a77-f34a-4cd2-b9a7-559df3c555d1</v>
       </c>
       <c r="B18" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C18" t="str">
-        <v>9520e1b4-1889-4925-9628-eb625555036c</v>
+        <v>7f88f66e-bf77-4937-bfe1-44d447960afc</v>
       </c>
       <c r="D18">
         <v>1</v>
       </c>
       <c r="E18" t="str">
-        <v>A3</v>
+        <v>A2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>3411d007-571a-484a-a508-360fe9c6c33e</v>
+        <v>9d49646c-54a0-43cc-b5a8-9a42788aaf6f</v>
       </c>
       <c r="B19" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C19" t="str">
-        <v>293e11eb-227f-4247-8788-b270b2af2d63</v>
+        <v>9520e1b4-1889-4925-9628-eb625555036c</v>
       </c>
       <c r="D19">
         <v>1</v>
       </c>
       <c r="E19" t="str">
-        <v>B5</v>
+        <v>A3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2457f5d9-ae65-4242-ab9c-2fb3902296fb</v>
+        <v>3411d007-571a-484a-a508-360fe9c6c33e</v>
       </c>
       <c r="B20" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C20" t="str">
-        <v>efcb7955-b4bc-487b-b45b-02a50d7f5ba2</v>
+        <v>293e11eb-227f-4247-8788-b270b2af2d63</v>
       </c>
       <c r="D20">
         <v>1</v>
       </c>
       <c r="E20" t="str">
-        <v>C4</v>
+        <v>B5</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>70f80dcf-ade2-4f1d-abe5-ea68a6443a19</v>
+        <v>2457f5d9-ae65-4242-ab9c-2fb3902296fb</v>
       </c>
       <c r="B21" t="str">
         <v>e432f0fe-1383-44a2-990c-5f787da5008a</v>
       </c>
       <c r="C21" t="str">
-        <v>df1eee3b-9186-4dcb-8dff-b88f5ac053e5</v>
+        <v>efcb7955-b4bc-487b-b45b-02a50d7f5ba2</v>
       </c>
       <c r="D21">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E21" t="str">
-        <v>D2</v>
+        <v>C4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>